<commit_message>
fix cb replenishment api url
</commit_message>
<xml_diff>
--- a/data/input/CB Replenishment_Master.xlsx
+++ b/data/input/CB Replenishment_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE2E22D-580E-4BA7-AE5E-648BDE86EA66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5EDE381-5347-4E11-9779-2217E51CC726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CFE25F1-D4D7-4072-B0D8-85CA58EF1A1A}"/>
   </bookViews>
@@ -16,10 +16,9 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$N$62</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -567,7 +566,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -590,20 +589,19 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -933,7 +931,7 @@
     <col min="9" max="9" width="23" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="30.88671875" customWidth="1"/>
     <col min="11" max="11" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.5546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="8.109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -998,43 +996,43 @@
       <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="8">
         <v>624</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="8">
         <v>1910</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="8">
         <v>25</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="8">
         <f>E2+F2</f>
         <v>1935</v>
       </c>
-      <c r="H2" s="10">
+      <c r="H2" s="9">
         <f>G2/3</f>
         <v>645</v>
       </c>
-      <c r="I2" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J2" s="11">
+      <c r="I2" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J2" s="10">
         <f>ROUNDUP(H2*I2,0)</f>
         <v>968</v>
       </c>
-      <c r="K2" s="10">
+      <c r="K2" s="9">
         <f>J2-D2</f>
         <v>344</v>
       </c>
-      <c r="L2" s="12">
+      <c r="L2" s="11">
         <v>300</v>
       </c>
-      <c r="M2" s="9" t="s">
+      <c r="M2" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="N2" s="9"/>
-      <c r="O2" s="9"/>
-      <c r="P2" s="9"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
+      <c r="P2" s="8"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -1046,41 +1044,41 @@
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>89</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="8">
         <v>240</v>
       </c>
-      <c r="F3" s="9">
-        <v>5</v>
-      </c>
-      <c r="G3" s="9">
+      <c r="F3" s="8">
+        <v>5</v>
+      </c>
+      <c r="G3" s="8">
         <f t="shared" ref="G3:G62" si="0">E3+F3</f>
         <v>245</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="9">
         <f t="shared" ref="H3:H62" si="1">G3/3</f>
         <v>81.666666666666671</v>
       </c>
-      <c r="I3" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J3" s="11">
+      <c r="I3" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J3" s="10">
         <f t="shared" ref="J3:J62" si="2">ROUNDUP(H3*I3,0)</f>
         <v>123</v>
       </c>
-      <c r="K3" s="10">
+      <c r="K3" s="9">
         <f t="shared" ref="K3:K62" si="3">J3-D3</f>
         <v>34</v>
       </c>
-      <c r="L3" s="12">
+      <c r="L3" s="11">
         <v>30</v>
       </c>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -1092,43 +1090,43 @@
       <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>230</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="8">
         <v>731</v>
       </c>
-      <c r="F4" s="9">
-        <v>5</v>
-      </c>
-      <c r="G4" s="9">
+      <c r="F4" s="8">
+        <v>5</v>
+      </c>
+      <c r="G4" s="8">
         <f t="shared" si="0"/>
         <v>736</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="9">
         <f t="shared" si="1"/>
         <v>245.33333333333334</v>
       </c>
-      <c r="I4" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J4" s="11">
+      <c r="I4" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J4" s="10">
         <f t="shared" si="2"/>
         <v>368</v>
       </c>
-      <c r="K4" s="10">
+      <c r="K4" s="9">
         <f t="shared" si="3"/>
         <v>138</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4" s="11">
         <v>100</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="M4" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -1140,41 +1138,41 @@
       <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="8">
         <v>8</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="8">
         <v>37</v>
       </c>
-      <c r="F5" s="9">
-        <v>5</v>
-      </c>
-      <c r="G5" s="9">
+      <c r="F5" s="8">
+        <v>5</v>
+      </c>
+      <c r="G5" s="8">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="9">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
-      <c r="I5" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J5" s="11">
+      <c r="I5" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J5" s="10">
         <f t="shared" si="2"/>
         <v>21</v>
       </c>
-      <c r="K5" s="10">
+      <c r="K5" s="9">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="L5" s="12">
+      <c r="L5" s="11">
         <v>50</v>
       </c>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="9"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -1186,41 +1184,41 @@
       <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="8">
         <v>2</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="8">
         <v>1</v>
       </c>
-      <c r="F6" s="9">
-        <v>5</v>
-      </c>
-      <c r="G6" s="9">
+      <c r="F6" s="8">
+        <v>5</v>
+      </c>
+      <c r="G6" s="8">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="9">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="I6" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J6" s="11">
+      <c r="I6" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J6" s="10">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K6" s="10">
+      <c r="K6" s="9">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="L6" s="12">
+      <c r="L6" s="11">
         <v>20</v>
       </c>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
@@ -1232,43 +1230,43 @@
       <c r="C7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="8">
         <v>47</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="8">
         <v>202</v>
       </c>
-      <c r="F7" s="9">
-        <v>5</v>
-      </c>
-      <c r="G7" s="9">
+      <c r="F7" s="8">
+        <v>5</v>
+      </c>
+      <c r="G7" s="8">
         <f t="shared" si="0"/>
         <v>207</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="9">
         <f t="shared" si="1"/>
         <v>69</v>
       </c>
-      <c r="I7" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J7" s="11">
+      <c r="I7" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J7" s="10">
         <f t="shared" si="2"/>
         <v>104</v>
       </c>
-      <c r="K7" s="10">
+      <c r="K7" s="9">
         <f t="shared" si="3"/>
         <v>57</v>
       </c>
-      <c r="L7" s="12">
+      <c r="L7" s="11">
         <v>120</v>
       </c>
-      <c r="M7" s="9" t="s">
+      <c r="M7" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -1280,41 +1278,41 @@
       <c r="C8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D8" s="8">
         <v>165</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="8">
         <v>662</v>
       </c>
-      <c r="F8" s="9">
-        <v>5</v>
-      </c>
-      <c r="G8" s="9">
+      <c r="F8" s="8">
+        <v>5</v>
+      </c>
+      <c r="G8" s="8">
         <f t="shared" si="0"/>
         <v>667</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="9">
         <f t="shared" si="1"/>
         <v>222.33333333333334</v>
       </c>
-      <c r="I8" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J8" s="11">
+      <c r="I8" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J8" s="10">
         <f t="shared" si="2"/>
         <v>334</v>
       </c>
-      <c r="K8" s="10">
+      <c r="K8" s="9">
         <f t="shared" si="3"/>
         <v>169</v>
       </c>
-      <c r="L8" s="12">
+      <c r="L8" s="11">
         <v>120</v>
       </c>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -1326,41 +1324,41 @@
       <c r="C9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="8">
         <v>72</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="8">
         <v>175</v>
       </c>
-      <c r="F9" s="9">
-        <v>5</v>
-      </c>
-      <c r="G9" s="9">
+      <c r="F9" s="8">
+        <v>5</v>
+      </c>
+      <c r="G9" s="8">
         <f t="shared" si="0"/>
         <v>180</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="9">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
-      <c r="I9" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J9" s="11">
+      <c r="I9" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J9" s="10">
         <f t="shared" si="2"/>
         <v>90</v>
       </c>
-      <c r="K9" s="10">
+      <c r="K9" s="9">
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="11">
         <v>10</v>
       </c>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
@@ -1372,41 +1370,41 @@
       <c r="C10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="8">
         <v>26</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="8">
         <v>84</v>
       </c>
-      <c r="F10" s="9">
-        <v>5</v>
-      </c>
-      <c r="G10" s="9">
+      <c r="F10" s="8">
+        <v>5</v>
+      </c>
+      <c r="G10" s="8">
         <f t="shared" si="0"/>
         <v>89</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="9">
         <f t="shared" si="1"/>
         <v>29.666666666666668</v>
       </c>
-      <c r="I10" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J10" s="11">
+      <c r="I10" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J10" s="10">
         <f t="shared" si="2"/>
         <v>45</v>
       </c>
-      <c r="K10" s="10">
+      <c r="K10" s="9">
         <f t="shared" si="3"/>
         <v>19</v>
       </c>
-      <c r="L10" s="12">
+      <c r="L10" s="11">
         <v>50</v>
       </c>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -1418,41 +1416,41 @@
       <c r="C11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="8">
         <v>78</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="8">
         <v>253</v>
       </c>
-      <c r="F11" s="9">
-        <v>5</v>
-      </c>
-      <c r="G11" s="9">
+      <c r="F11" s="8">
+        <v>5</v>
+      </c>
+      <c r="G11" s="8">
         <f t="shared" si="0"/>
         <v>258</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H11" s="9">
         <f t="shared" si="1"/>
         <v>86</v>
       </c>
-      <c r="I11" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J11" s="11">
+      <c r="I11" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J11" s="10">
         <f t="shared" si="2"/>
         <v>129</v>
       </c>
-      <c r="K11" s="10">
+      <c r="K11" s="9">
         <f t="shared" si="3"/>
         <v>51</v>
       </c>
-      <c r="L11" s="13">
+      <c r="L11" s="12">
         <v>80</v>
       </c>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
@@ -1464,41 +1462,41 @@
       <c r="C12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="8">
         <v>100</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="8">
         <v>193</v>
       </c>
-      <c r="F12" s="9">
-        <v>5</v>
-      </c>
-      <c r="G12" s="9">
+      <c r="F12" s="8">
+        <v>5</v>
+      </c>
+      <c r="G12" s="8">
         <f t="shared" si="0"/>
         <v>198</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="9">
         <f t="shared" si="1"/>
         <v>66</v>
       </c>
-      <c r="I12" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J12" s="11">
+      <c r="I12" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J12" s="10">
         <f t="shared" si="2"/>
         <v>99</v>
       </c>
-      <c r="K12" s="10">
+      <c r="K12" s="9">
         <f t="shared" si="3"/>
         <v>-1</v>
       </c>
-      <c r="L12" s="12">
+      <c r="L12" s="11">
         <v>30</v>
       </c>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
@@ -1510,41 +1508,41 @@
       <c r="C13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="8">
         <v>137</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="8">
         <v>637</v>
       </c>
-      <c r="F13" s="9">
-        <v>5</v>
-      </c>
-      <c r="G13" s="9">
+      <c r="F13" s="8">
+        <v>5</v>
+      </c>
+      <c r="G13" s="8">
         <f t="shared" si="0"/>
         <v>642</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="9">
         <f t="shared" si="1"/>
         <v>214</v>
       </c>
-      <c r="I13" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J13" s="11">
+      <c r="I13" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J13" s="10">
         <f t="shared" si="2"/>
         <v>321</v>
       </c>
-      <c r="K13" s="10">
+      <c r="K13" s="9">
         <f t="shared" si="3"/>
         <v>184</v>
       </c>
-      <c r="L13" s="12">
+      <c r="L13" s="11">
         <v>160</v>
       </c>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
@@ -1556,41 +1554,41 @@
       <c r="C14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="8">
         <v>34</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="8">
         <v>72</v>
       </c>
-      <c r="F14" s="9">
-        <v>5</v>
-      </c>
-      <c r="G14" s="9">
+      <c r="F14" s="8">
+        <v>5</v>
+      </c>
+      <c r="G14" s="8">
         <f t="shared" si="0"/>
         <v>77</v>
       </c>
-      <c r="H14" s="10">
+      <c r="H14" s="9">
         <f t="shared" si="1"/>
         <v>25.666666666666668</v>
       </c>
-      <c r="I14" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J14" s="11">
+      <c r="I14" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J14" s="10">
         <f t="shared" si="2"/>
         <v>39</v>
       </c>
-      <c r="K14" s="10">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="L14" s="12">
+      <c r="K14" s="9">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="L14" s="11">
         <v>20</v>
       </c>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="9"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
@@ -1602,41 +1600,41 @@
       <c r="C15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="8">
         <v>13</v>
       </c>
-      <c r="E15" s="9">
+      <c r="E15" s="8">
         <v>31</v>
       </c>
-      <c r="F15" s="9">
-        <v>5</v>
-      </c>
-      <c r="G15" s="9">
+      <c r="F15" s="8">
+        <v>5</v>
+      </c>
+      <c r="G15" s="8">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="9">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="I15" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J15" s="11">
+      <c r="I15" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J15" s="10">
         <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="K15" s="10">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="L15" s="12">
+      <c r="K15" s="9">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="L15" s="11">
         <v>10</v>
       </c>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="9"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -1648,41 +1646,41 @@
       <c r="C16" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="8">
         <v>21</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16" s="8">
         <v>27</v>
       </c>
-      <c r="F16" s="9">
-        <v>5</v>
-      </c>
-      <c r="G16" s="9">
+      <c r="F16" s="8">
+        <v>5</v>
+      </c>
+      <c r="G16" s="8">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="H16" s="10">
+      <c r="H16" s="9">
         <f t="shared" si="1"/>
         <v>10.666666666666666</v>
       </c>
-      <c r="I16" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J16" s="11">
+      <c r="I16" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J16" s="10">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="K16" s="10">
+      <c r="K16" s="9">
         <f t="shared" si="3"/>
         <v>-5</v>
       </c>
-      <c r="L16" s="12">
+      <c r="L16" s="11">
         <v>20</v>
       </c>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="9"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
@@ -1694,41 +1692,41 @@
       <c r="C17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="8">
         <v>21</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="8">
         <v>32</v>
       </c>
-      <c r="F17" s="9">
-        <v>5</v>
-      </c>
-      <c r="G17" s="9">
+      <c r="F17" s="8">
+        <v>5</v>
+      </c>
+      <c r="G17" s="8">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="H17" s="10">
+      <c r="H17" s="9">
         <f t="shared" si="1"/>
         <v>12.333333333333334</v>
       </c>
-      <c r="I17" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J17" s="11">
+      <c r="I17" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J17" s="10">
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="K17" s="10">
+      <c r="K17" s="9">
         <f t="shared" si="3"/>
         <v>-2</v>
       </c>
-      <c r="L17" s="12">
+      <c r="L17" s="11">
         <v>10</v>
       </c>
-      <c r="M17" s="9"/>
-      <c r="N17" s="9"/>
-      <c r="O17" s="9"/>
-      <c r="P17" s="9"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
@@ -1740,41 +1738,41 @@
       <c r="C18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="8">
         <v>10</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="8">
         <v>29</v>
       </c>
-      <c r="F18" s="9">
-        <v>5</v>
-      </c>
-      <c r="G18" s="9">
+      <c r="F18" s="8">
+        <v>5</v>
+      </c>
+      <c r="G18" s="8">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="H18" s="10">
+      <c r="H18" s="9">
         <f t="shared" si="1"/>
         <v>11.333333333333334</v>
       </c>
-      <c r="I18" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J18" s="11">
+      <c r="I18" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J18" s="10">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="K18" s="10">
+      <c r="K18" s="9">
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="L18" s="12">
+      <c r="L18" s="11">
         <v>20</v>
       </c>
-      <c r="M18" s="9"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="9"/>
-      <c r="P18" s="9"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="8"/>
+      <c r="P18" s="8"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
@@ -1786,41 +1784,41 @@
       <c r="C19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="8">
         <v>106</v>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="8">
         <v>344</v>
       </c>
-      <c r="F19" s="9">
-        <v>5</v>
-      </c>
-      <c r="G19" s="9">
+      <c r="F19" s="8">
+        <v>5</v>
+      </c>
+      <c r="G19" s="8">
         <f t="shared" si="0"/>
         <v>349</v>
       </c>
-      <c r="H19" s="10">
+      <c r="H19" s="9">
         <f t="shared" si="1"/>
         <v>116.33333333333333</v>
       </c>
-      <c r="I19" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J19" s="11">
+      <c r="I19" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J19" s="10">
         <f t="shared" si="2"/>
         <v>175</v>
       </c>
-      <c r="K19" s="10">
+      <c r="K19" s="9">
         <f t="shared" si="3"/>
         <v>69</v>
       </c>
-      <c r="L19" s="12">
+      <c r="L19" s="11">
         <v>30</v>
       </c>
-      <c r="M19" s="9"/>
-      <c r="N19" s="9"/>
-      <c r="O19" s="9"/>
-      <c r="P19" s="9"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="8"/>
+      <c r="P19" s="8"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
@@ -1832,41 +1830,41 @@
       <c r="C20" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="8">
         <v>31</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="8">
         <v>84</v>
       </c>
-      <c r="F20" s="9">
-        <v>5</v>
-      </c>
-      <c r="G20" s="9">
+      <c r="F20" s="8">
+        <v>5</v>
+      </c>
+      <c r="G20" s="8">
         <f t="shared" si="0"/>
         <v>89</v>
       </c>
-      <c r="H20" s="10">
+      <c r="H20" s="9">
         <f t="shared" si="1"/>
         <v>29.666666666666668</v>
       </c>
-      <c r="I20" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J20" s="11">
+      <c r="I20" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J20" s="10">
         <f t="shared" si="2"/>
         <v>45</v>
       </c>
-      <c r="K20" s="10">
+      <c r="K20" s="9">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="L20" s="12">
+      <c r="L20" s="11">
         <v>20</v>
       </c>
-      <c r="M20" s="9"/>
-      <c r="N20" s="9"/>
-      <c r="O20" s="9"/>
-      <c r="P20" s="9"/>
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
+      <c r="O20" s="8"/>
+      <c r="P20" s="8"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -1878,41 +1876,41 @@
       <c r="C21" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="8">
         <v>42</v>
       </c>
-      <c r="E21" s="9">
+      <c r="E21" s="8">
         <v>86</v>
       </c>
-      <c r="F21" s="9">
-        <v>5</v>
-      </c>
-      <c r="G21" s="9">
+      <c r="F21" s="8">
+        <v>5</v>
+      </c>
+      <c r="G21" s="8">
         <f t="shared" si="0"/>
         <v>91</v>
       </c>
-      <c r="H21" s="10">
+      <c r="H21" s="9">
         <f t="shared" si="1"/>
         <v>30.333333333333332</v>
       </c>
-      <c r="I21" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J21" s="11">
+      <c r="I21" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J21" s="10">
         <f t="shared" si="2"/>
         <v>46</v>
       </c>
-      <c r="K21" s="10">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="L21" s="12">
+      <c r="K21" s="9">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="L21" s="11">
         <v>20</v>
       </c>
-      <c r="M21" s="9"/>
-      <c r="N21" s="9"/>
-      <c r="O21" s="9"/>
-      <c r="P21" s="9"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
+      <c r="O21" s="8"/>
+      <c r="P21" s="8"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
@@ -1924,41 +1922,41 @@
       <c r="C22" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D22" s="9">
+      <c r="D22" s="8">
         <v>39</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="8">
         <v>67</v>
       </c>
-      <c r="F22" s="9">
-        <v>5</v>
-      </c>
-      <c r="G22" s="9">
+      <c r="F22" s="8">
+        <v>5</v>
+      </c>
+      <c r="G22" s="8">
         <f t="shared" si="0"/>
         <v>72</v>
       </c>
-      <c r="H22" s="10">
+      <c r="H22" s="9">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="I22" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J22" s="11">
+      <c r="I22" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J22" s="10">
         <f t="shared" si="2"/>
         <v>36</v>
       </c>
-      <c r="K22" s="10">
+      <c r="K22" s="9">
         <f t="shared" si="3"/>
         <v>-3</v>
       </c>
-      <c r="L22" s="12">
+      <c r="L22" s="11">
         <v>10</v>
       </c>
-      <c r="M22" s="9"/>
-      <c r="N22" s="9"/>
-      <c r="O22" s="9"/>
-      <c r="P22" s="9"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
@@ -1970,41 +1968,41 @@
       <c r="C23" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="8">
         <v>30</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="8">
         <v>53</v>
       </c>
-      <c r="F23" s="9">
-        <v>5</v>
-      </c>
-      <c r="G23" s="9">
+      <c r="F23" s="8">
+        <v>5</v>
+      </c>
+      <c r="G23" s="8">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="H23" s="10">
+      <c r="H23" s="9">
         <f t="shared" si="1"/>
         <v>19.333333333333332</v>
       </c>
-      <c r="I23" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J23" s="11">
+      <c r="I23" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J23" s="10">
         <f t="shared" si="2"/>
         <v>29</v>
       </c>
-      <c r="K23" s="10">
+      <c r="K23" s="9">
         <f t="shared" si="3"/>
         <v>-1</v>
       </c>
-      <c r="L23" s="12">
+      <c r="L23" s="11">
         <v>20</v>
       </c>
-      <c r="M23" s="9"/>
-      <c r="N23" s="9"/>
-      <c r="O23" s="9"/>
-      <c r="P23" s="9"/>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="8"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
@@ -2016,43 +2014,43 @@
       <c r="C24" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="8">
         <v>35</v>
       </c>
-      <c r="E24" s="9">
+      <c r="E24" s="8">
         <v>19</v>
       </c>
-      <c r="F24" s="9">
-        <v>5</v>
-      </c>
-      <c r="G24" s="9">
+      <c r="F24" s="8">
+        <v>5</v>
+      </c>
+      <c r="G24" s="8">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="H24" s="10">
+      <c r="H24" s="9">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="I24" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J24" s="11">
+      <c r="I24" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J24" s="10">
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="K24" s="10">
+      <c r="K24" s="9">
         <f t="shared" si="3"/>
         <v>-23</v>
       </c>
-      <c r="L24" s="12">
+      <c r="L24" s="11">
         <v>30</v>
       </c>
-      <c r="M24" s="9" t="s">
+      <c r="M24" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="N24" s="9"/>
-      <c r="O24" s="9"/>
-      <c r="P24" s="9"/>
+      <c r="N24" s="8"/>
+      <c r="O24" s="8"/>
+      <c r="P24" s="8"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
@@ -2064,41 +2062,41 @@
       <c r="C25" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="8">
         <v>49</v>
       </c>
-      <c r="E25" s="9">
+      <c r="E25" s="8">
         <v>141</v>
       </c>
-      <c r="F25" s="9">
-        <v>5</v>
-      </c>
-      <c r="G25" s="9">
+      <c r="F25" s="8">
+        <v>5</v>
+      </c>
+      <c r="G25" s="8">
         <f t="shared" si="0"/>
         <v>146</v>
       </c>
-      <c r="H25" s="10">
+      <c r="H25" s="9">
         <f t="shared" si="1"/>
         <v>48.666666666666664</v>
       </c>
-      <c r="I25" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J25" s="11">
+      <c r="I25" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J25" s="10">
         <f t="shared" si="2"/>
         <v>73</v>
       </c>
-      <c r="K25" s="10">
+      <c r="K25" s="9">
         <f t="shared" si="3"/>
         <v>24</v>
       </c>
-      <c r="L25" s="12">
+      <c r="L25" s="11">
         <v>20</v>
       </c>
-      <c r="M25" s="9"/>
-      <c r="N25" s="9"/>
-      <c r="O25" s="9"/>
-      <c r="P25" s="9"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
@@ -2110,41 +2108,41 @@
       <c r="C26" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="8">
         <v>53</v>
       </c>
-      <c r="E26" s="9">
+      <c r="E26" s="8">
         <v>149</v>
       </c>
-      <c r="F26" s="9">
-        <v>5</v>
-      </c>
-      <c r="G26" s="9">
+      <c r="F26" s="8">
+        <v>5</v>
+      </c>
+      <c r="G26" s="8">
         <f t="shared" si="0"/>
         <v>154</v>
       </c>
-      <c r="H26" s="10">
+      <c r="H26" s="9">
         <f t="shared" si="1"/>
         <v>51.333333333333336</v>
       </c>
-      <c r="I26" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J26" s="11">
+      <c r="I26" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J26" s="10">
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
-      <c r="K26" s="10">
+      <c r="K26" s="9">
         <f t="shared" si="3"/>
         <v>24</v>
       </c>
-      <c r="L26" s="12">
+      <c r="L26" s="11">
         <v>50</v>
       </c>
-      <c r="M26" s="9"/>
-      <c r="N26" s="9"/>
-      <c r="O26" s="9"/>
-      <c r="P26" s="9"/>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
+      <c r="O26" s="8"/>
+      <c r="P26" s="8"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
@@ -2156,41 +2154,41 @@
       <c r="C27" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="8">
         <v>43</v>
       </c>
-      <c r="E27" s="9">
+      <c r="E27" s="8">
         <v>107</v>
       </c>
-      <c r="F27" s="9">
-        <v>5</v>
-      </c>
-      <c r="G27" s="9">
+      <c r="F27" s="8">
+        <v>5</v>
+      </c>
+      <c r="G27" s="8">
         <f t="shared" si="0"/>
         <v>112</v>
       </c>
-      <c r="H27" s="10">
+      <c r="H27" s="9">
         <f t="shared" si="1"/>
         <v>37.333333333333336</v>
       </c>
-      <c r="I27" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J27" s="11">
+      <c r="I27" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J27" s="10">
         <f t="shared" si="2"/>
         <v>56</v>
       </c>
-      <c r="K27" s="10">
+      <c r="K27" s="9">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="L27" s="12">
+      <c r="L27" s="11">
         <v>20</v>
       </c>
-      <c r="M27" s="9"/>
-      <c r="N27" s="9"/>
-      <c r="O27" s="9"/>
-      <c r="P27" s="9"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="8"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
@@ -2202,41 +2200,41 @@
       <c r="C28" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D28" s="9">
+      <c r="D28" s="8">
         <v>21</v>
       </c>
-      <c r="E28" s="9">
+      <c r="E28" s="8">
         <v>48</v>
       </c>
-      <c r="F28" s="9">
-        <v>5</v>
-      </c>
-      <c r="G28" s="9">
+      <c r="F28" s="8">
+        <v>5</v>
+      </c>
+      <c r="G28" s="8">
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
-      <c r="H28" s="10">
+      <c r="H28" s="9">
         <f t="shared" si="1"/>
         <v>17.666666666666668</v>
       </c>
-      <c r="I28" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J28" s="11">
+      <c r="I28" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J28" s="10">
         <f t="shared" si="2"/>
         <v>27</v>
       </c>
-      <c r="K28" s="10">
+      <c r="K28" s="9">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L28" s="12">
+      <c r="L28" s="11">
         <v>10</v>
       </c>
-      <c r="M28" s="9"/>
-      <c r="N28" s="9"/>
-      <c r="O28" s="9"/>
-      <c r="P28" s="9"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="8"/>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -2248,41 +2246,41 @@
       <c r="C29" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D29" s="9">
+      <c r="D29" s="8">
         <v>27</v>
       </c>
-      <c r="E29" s="9">
+      <c r="E29" s="8">
         <v>78</v>
       </c>
-      <c r="F29" s="9">
-        <v>5</v>
-      </c>
-      <c r="G29" s="9">
+      <c r="F29" s="8">
+        <v>5</v>
+      </c>
+      <c r="G29" s="8">
         <f t="shared" si="0"/>
         <v>83</v>
       </c>
-      <c r="H29" s="10">
+      <c r="H29" s="9">
         <f t="shared" si="1"/>
         <v>27.666666666666668</v>
       </c>
-      <c r="I29" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J29" s="11">
+      <c r="I29" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J29" s="10">
         <f t="shared" si="2"/>
         <v>42</v>
       </c>
-      <c r="K29" s="10">
+      <c r="K29" s="9">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="L29" s="12">
+      <c r="L29" s="11">
         <v>10</v>
       </c>
-      <c r="M29" s="9"/>
-      <c r="N29" s="9"/>
-      <c r="O29" s="9"/>
-      <c r="P29" s="9"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="8"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="8"/>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
@@ -2294,41 +2292,41 @@
       <c r="C30" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="8">
         <v>2</v>
       </c>
-      <c r="E30" s="9">
+      <c r="E30" s="8">
         <v>3</v>
       </c>
-      <c r="F30" s="9">
-        <v>5</v>
-      </c>
-      <c r="G30" s="9">
+      <c r="F30" s="8">
+        <v>5</v>
+      </c>
+      <c r="G30" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="H30" s="10">
+      <c r="H30" s="9">
         <f t="shared" si="1"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="I30" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J30" s="11">
-        <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="K30" s="10">
+      <c r="I30" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J30" s="10">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="K30" s="9">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="L30" s="12">
+      <c r="L30" s="11">
         <v>10</v>
       </c>
-      <c r="M30" s="9"/>
-      <c r="N30" s="9"/>
-      <c r="O30" s="9"/>
-      <c r="P30" s="9"/>
+      <c r="M30" s="8"/>
+      <c r="N30" s="8"/>
+      <c r="O30" s="8"/>
+      <c r="P30" s="8"/>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
@@ -2340,43 +2338,43 @@
       <c r="C31" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D31" s="9">
-        <v>5</v>
-      </c>
-      <c r="E31" s="9">
+      <c r="D31" s="8">
+        <v>5</v>
+      </c>
+      <c r="E31" s="8">
         <v>17</v>
       </c>
-      <c r="F31" s="9">
-        <v>5</v>
-      </c>
-      <c r="G31" s="9">
+      <c r="F31" s="8">
+        <v>5</v>
+      </c>
+      <c r="G31" s="8">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="H31" s="10">
+      <c r="H31" s="9">
         <f t="shared" si="1"/>
         <v>7.333333333333333</v>
       </c>
-      <c r="I31" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J31" s="11">
+      <c r="I31" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J31" s="10">
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="K31" s="10">
+      <c r="K31" s="9">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L31" s="12">
+      <c r="L31" s="11">
         <v>20</v>
       </c>
-      <c r="M31" s="9" t="s">
+      <c r="M31" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="N31" s="9"/>
-      <c r="O31" s="9"/>
-      <c r="P31" s="9"/>
+      <c r="N31" s="8"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="8"/>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
@@ -2388,41 +2386,41 @@
       <c r="C32" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D32" s="9">
-        <v>5</v>
-      </c>
-      <c r="E32" s="9">
-        <v>5</v>
-      </c>
-      <c r="F32" s="9">
-        <v>5</v>
-      </c>
-      <c r="G32" s="9">
+      <c r="D32" s="8">
+        <v>5</v>
+      </c>
+      <c r="E32" s="8">
+        <v>5</v>
+      </c>
+      <c r="F32" s="8">
+        <v>5</v>
+      </c>
+      <c r="G32" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="H32" s="10">
+      <c r="H32" s="9">
         <f t="shared" si="1"/>
         <v>3.3333333333333335</v>
       </c>
-      <c r="I32" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J32" s="11">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="K32" s="10">
+      <c r="I32" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J32" s="10">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="K32" s="9">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L32" s="12">
+      <c r="L32" s="11">
         <v>10</v>
       </c>
-      <c r="M32" s="9"/>
-      <c r="N32" s="9"/>
-      <c r="O32" s="9"/>
-      <c r="P32" s="9"/>
+      <c r="M32" s="8"/>
+      <c r="N32" s="8"/>
+      <c r="O32" s="8"/>
+      <c r="P32" s="8"/>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
@@ -2434,41 +2432,41 @@
       <c r="C33" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D33" s="9">
+      <c r="D33" s="8">
         <v>45</v>
       </c>
-      <c r="E33" s="9">
+      <c r="E33" s="8">
         <v>118</v>
       </c>
-      <c r="F33" s="9">
-        <v>5</v>
-      </c>
-      <c r="G33" s="9">
+      <c r="F33" s="8">
+        <v>5</v>
+      </c>
+      <c r="G33" s="8">
         <f t="shared" si="0"/>
         <v>123</v>
       </c>
-      <c r="H33" s="10">
+      <c r="H33" s="9">
         <f t="shared" si="1"/>
         <v>41</v>
       </c>
-      <c r="I33" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J33" s="11">
+      <c r="I33" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J33" s="10">
         <f t="shared" si="2"/>
         <v>62</v>
       </c>
-      <c r="K33" s="10">
+      <c r="K33" s="9">
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="L33" s="12">
+      <c r="L33" s="11">
         <v>20</v>
       </c>
-      <c r="M33" s="9"/>
-      <c r="N33" s="9"/>
-      <c r="O33" s="9"/>
-      <c r="P33" s="9"/>
+      <c r="M33" s="8"/>
+      <c r="N33" s="8"/>
+      <c r="O33" s="8"/>
+      <c r="P33" s="8"/>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
@@ -2480,41 +2478,41 @@
       <c r="C34" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D34" s="9">
+      <c r="D34" s="8">
         <v>13</v>
       </c>
-      <c r="E34" s="9">
+      <c r="E34" s="8">
         <v>28</v>
       </c>
-      <c r="F34" s="9">
-        <v>5</v>
-      </c>
-      <c r="G34" s="9">
+      <c r="F34" s="8">
+        <v>5</v>
+      </c>
+      <c r="G34" s="8">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="H34" s="10">
+      <c r="H34" s="9">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="I34" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J34" s="11">
+      <c r="I34" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J34" s="10">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="K34" s="10">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="L34" s="12">
+      <c r="K34" s="9">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="L34" s="11">
         <v>10</v>
       </c>
-      <c r="M34" s="9"/>
-      <c r="N34" s="9"/>
-      <c r="O34" s="9"/>
-      <c r="P34" s="9"/>
+      <c r="M34" s="8"/>
+      <c r="N34" s="8"/>
+      <c r="O34" s="8"/>
+      <c r="P34" s="8"/>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -2526,43 +2524,43 @@
       <c r="C35" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D35" s="9">
+      <c r="D35" s="8">
         <v>6</v>
       </c>
-      <c r="E35" s="9">
+      <c r="E35" s="8">
         <v>10</v>
       </c>
-      <c r="F35" s="9">
-        <v>5</v>
-      </c>
-      <c r="G35" s="9">
+      <c r="F35" s="8">
+        <v>5</v>
+      </c>
+      <c r="G35" s="8">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="H35" s="10">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="I35" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J35" s="11">
+      <c r="H35" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="I35" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J35" s="10">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="K35" s="10">
+      <c r="K35" s="9">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="L35" s="12">
+      <c r="L35" s="11">
         <v>20</v>
       </c>
-      <c r="M35" s="9" t="s">
+      <c r="M35" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="N35" s="9"/>
-      <c r="O35" s="9"/>
-      <c r="P35" s="9"/>
+      <c r="N35" s="8"/>
+      <c r="O35" s="8"/>
+      <c r="P35" s="8"/>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
@@ -2574,43 +2572,43 @@
       <c r="C36" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D36" s="9">
+      <c r="D36" s="8">
         <v>223</v>
       </c>
-      <c r="E36" s="9">
+      <c r="E36" s="8">
         <v>654</v>
       </c>
-      <c r="F36" s="9">
-        <v>5</v>
-      </c>
-      <c r="G36" s="9">
+      <c r="F36" s="8">
+        <v>5</v>
+      </c>
+      <c r="G36" s="8">
         <f t="shared" si="0"/>
         <v>659</v>
       </c>
-      <c r="H36" s="10">
+      <c r="H36" s="9">
         <f t="shared" si="1"/>
         <v>219.66666666666666</v>
       </c>
-      <c r="I36" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J36" s="11">
+      <c r="I36" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J36" s="10">
         <f t="shared" si="2"/>
         <v>330</v>
       </c>
-      <c r="K36" s="10">
+      <c r="K36" s="9">
         <f t="shared" si="3"/>
         <v>107</v>
       </c>
-      <c r="L36" s="12">
+      <c r="L36" s="11">
         <v>150</v>
       </c>
-      <c r="M36" s="9" t="s">
+      <c r="M36" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="N36" s="9"/>
-      <c r="O36" s="9"/>
-      <c r="P36" s="9"/>
+      <c r="N36" s="8"/>
+      <c r="O36" s="8"/>
+      <c r="P36" s="8"/>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
@@ -2622,41 +2620,41 @@
       <c r="C37" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D37" s="9">
+      <c r="D37" s="8">
         <v>0</v>
       </c>
-      <c r="E37" s="9">
+      <c r="E37" s="8">
         <v>7</v>
       </c>
-      <c r="F37" s="9">
-        <v>5</v>
-      </c>
-      <c r="G37" s="9">
+      <c r="F37" s="8">
+        <v>5</v>
+      </c>
+      <c r="G37" s="8">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="H37" s="10">
-        <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="I37" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J37" s="11">
+      <c r="H37" s="9">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="I37" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J37" s="10">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="K37" s="10">
+      <c r="K37" s="9">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L37" s="12">
+      <c r="L37" s="11">
         <v>10</v>
       </c>
-      <c r="M37" s="9"/>
-      <c r="N37" s="9"/>
-      <c r="O37" s="9"/>
-      <c r="P37" s="9"/>
+      <c r="M37" s="8"/>
+      <c r="N37" s="8"/>
+      <c r="O37" s="8"/>
+      <c r="P37" s="8"/>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
@@ -2668,43 +2666,43 @@
       <c r="C38" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="8">
         <v>23</v>
       </c>
-      <c r="E38" s="9">
+      <c r="E38" s="8">
         <v>32</v>
       </c>
-      <c r="F38" s="9">
-        <v>5</v>
-      </c>
-      <c r="G38" s="9">
+      <c r="F38" s="8">
+        <v>5</v>
+      </c>
+      <c r="G38" s="8">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="H38" s="10">
+      <c r="H38" s="9">
         <f t="shared" si="1"/>
         <v>12.333333333333334</v>
       </c>
-      <c r="I38" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J38" s="11">
+      <c r="I38" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J38" s="10">
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="K38" s="10">
+      <c r="K38" s="9">
         <f t="shared" si="3"/>
         <v>-4</v>
       </c>
-      <c r="L38" s="12">
+      <c r="L38" s="11">
         <v>100</v>
       </c>
-      <c r="M38" s="9" t="s">
+      <c r="M38" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="N38" s="9"/>
-      <c r="O38" s="9"/>
-      <c r="P38" s="9"/>
+      <c r="N38" s="8"/>
+      <c r="O38" s="8"/>
+      <c r="P38" s="8"/>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
@@ -2716,41 +2714,41 @@
       <c r="C39" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D39" s="9">
+      <c r="D39" s="8">
         <v>16</v>
       </c>
-      <c r="E39" s="9">
+      <c r="E39" s="8">
         <v>38</v>
       </c>
-      <c r="F39" s="9">
-        <v>5</v>
-      </c>
-      <c r="G39" s="9">
+      <c r="F39" s="8">
+        <v>5</v>
+      </c>
+      <c r="G39" s="8">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="H39" s="10">
+      <c r="H39" s="9">
         <f t="shared" si="1"/>
         <v>14.333333333333334</v>
       </c>
-      <c r="I39" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J39" s="11">
+      <c r="I39" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J39" s="10">
         <f t="shared" si="2"/>
         <v>22</v>
       </c>
-      <c r="K39" s="10">
+      <c r="K39" s="9">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L39" s="12">
+      <c r="L39" s="11">
         <v>10</v>
       </c>
-      <c r="M39" s="9"/>
-      <c r="N39" s="9"/>
-      <c r="O39" s="9"/>
-      <c r="P39" s="9"/>
+      <c r="M39" s="8"/>
+      <c r="N39" s="8"/>
+      <c r="O39" s="8"/>
+      <c r="P39" s="8"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
@@ -2762,41 +2760,41 @@
       <c r="C40" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="8">
         <v>35</v>
       </c>
-      <c r="E40" s="9">
+      <c r="E40" s="8">
         <v>75</v>
       </c>
-      <c r="F40" s="9">
-        <v>5</v>
-      </c>
-      <c r="G40" s="9">
+      <c r="F40" s="8">
+        <v>5</v>
+      </c>
+      <c r="G40" s="8">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="H40" s="10">
+      <c r="H40" s="9">
         <f t="shared" si="1"/>
         <v>26.666666666666668</v>
       </c>
-      <c r="I40" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J40" s="11">
+      <c r="I40" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J40" s="10">
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="K40" s="10">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="L40" s="12">
+      <c r="K40" s="9">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="L40" s="11">
         <v>20</v>
       </c>
-      <c r="M40" s="9"/>
-      <c r="N40" s="9"/>
-      <c r="O40" s="9"/>
-      <c r="P40" s="9"/>
+      <c r="M40" s="8"/>
+      <c r="N40" s="8"/>
+      <c r="O40" s="8"/>
+      <c r="P40" s="8"/>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -2808,41 +2806,41 @@
       <c r="C41" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D41" s="9">
+      <c r="D41" s="8">
         <v>14</v>
       </c>
-      <c r="E41" s="9">
+      <c r="E41" s="8">
         <v>47</v>
       </c>
-      <c r="F41" s="9">
-        <v>5</v>
-      </c>
-      <c r="G41" s="9">
+      <c r="F41" s="8">
+        <v>5</v>
+      </c>
+      <c r="G41" s="8">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="H41" s="10">
+      <c r="H41" s="9">
         <f t="shared" si="1"/>
         <v>17.333333333333332</v>
       </c>
-      <c r="I41" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J41" s="11">
+      <c r="I41" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J41" s="10">
         <f t="shared" si="2"/>
         <v>26</v>
       </c>
-      <c r="K41" s="10">
+      <c r="K41" s="9">
         <f t="shared" si="3"/>
         <v>12</v>
       </c>
-      <c r="L41" s="12">
+      <c r="L41" s="11">
         <v>20</v>
       </c>
-      <c r="M41" s="9"/>
-      <c r="N41" s="9"/>
-      <c r="O41" s="9"/>
-      <c r="P41" s="9"/>
+      <c r="M41" s="8"/>
+      <c r="N41" s="8"/>
+      <c r="O41" s="8"/>
+      <c r="P41" s="8"/>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
@@ -2854,41 +2852,41 @@
       <c r="C42" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D42" s="9">
+      <c r="D42" s="8">
         <v>40</v>
       </c>
-      <c r="E42" s="9">
+      <c r="E42" s="8">
         <v>91</v>
       </c>
-      <c r="F42" s="9">
-        <v>5</v>
-      </c>
-      <c r="G42" s="9">
+      <c r="F42" s="8">
+        <v>5</v>
+      </c>
+      <c r="G42" s="8">
         <f t="shared" si="0"/>
         <v>96</v>
       </c>
-      <c r="H42" s="10">
+      <c r="H42" s="9">
         <f t="shared" si="1"/>
         <v>32</v>
       </c>
-      <c r="I42" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J42" s="11">
+      <c r="I42" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J42" s="10">
         <f t="shared" si="2"/>
         <v>48</v>
       </c>
-      <c r="K42" s="10">
+      <c r="K42" s="9">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="L42" s="12">
+      <c r="L42" s="11">
         <v>40</v>
       </c>
-      <c r="M42" s="9"/>
-      <c r="N42" s="9"/>
-      <c r="O42" s="9"/>
-      <c r="P42" s="9"/>
+      <c r="M42" s="8"/>
+      <c r="N42" s="8"/>
+      <c r="O42" s="8"/>
+      <c r="P42" s="8"/>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
@@ -2900,41 +2898,41 @@
       <c r="C43" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D43" s="9">
+      <c r="D43" s="8">
         <v>13</v>
       </c>
-      <c r="E43" s="9">
+      <c r="E43" s="8">
         <v>42</v>
       </c>
-      <c r="F43" s="9">
-        <v>5</v>
-      </c>
-      <c r="G43" s="9">
+      <c r="F43" s="8">
+        <v>5</v>
+      </c>
+      <c r="G43" s="8">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-      <c r="H43" s="10">
+      <c r="H43" s="9">
         <f t="shared" si="1"/>
         <v>15.666666666666666</v>
       </c>
-      <c r="I43" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J43" s="11">
+      <c r="I43" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J43" s="10">
         <f t="shared" si="2"/>
         <v>24</v>
       </c>
-      <c r="K43" s="10">
+      <c r="K43" s="9">
         <f t="shared" si="3"/>
         <v>11</v>
       </c>
-      <c r="L43" s="12">
+      <c r="L43" s="11">
         <v>10</v>
       </c>
-      <c r="M43" s="9"/>
-      <c r="N43" s="9"/>
-      <c r="O43" s="9"/>
-      <c r="P43" s="9"/>
+      <c r="M43" s="8"/>
+      <c r="N43" s="8"/>
+      <c r="O43" s="8"/>
+      <c r="P43" s="8"/>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
@@ -2946,41 +2944,41 @@
       <c r="C44" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D44" s="9">
-        <v>5</v>
-      </c>
-      <c r="E44" s="9">
+      <c r="D44" s="8">
+        <v>5</v>
+      </c>
+      <c r="E44" s="8">
         <v>17</v>
       </c>
-      <c r="F44" s="9">
-        <v>5</v>
-      </c>
-      <c r="G44" s="9">
+      <c r="F44" s="8">
+        <v>5</v>
+      </c>
+      <c r="G44" s="8">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="H44" s="10">
+      <c r="H44" s="9">
         <f t="shared" si="1"/>
         <v>7.333333333333333</v>
       </c>
-      <c r="I44" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J44" s="11">
+      <c r="I44" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J44" s="10">
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="K44" s="10">
+      <c r="K44" s="9">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L44" s="12">
+      <c r="L44" s="11">
         <v>10</v>
       </c>
-      <c r="M44" s="9"/>
-      <c r="N44" s="9"/>
-      <c r="O44" s="9"/>
-      <c r="P44" s="9"/>
+      <c r="M44" s="8"/>
+      <c r="N44" s="8"/>
+      <c r="O44" s="8"/>
+      <c r="P44" s="8"/>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
@@ -2992,41 +2990,41 @@
       <c r="C45" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D45" s="9">
+      <c r="D45" s="8">
         <v>2</v>
       </c>
-      <c r="E45" s="9">
+      <c r="E45" s="8">
         <v>10</v>
       </c>
-      <c r="F45" s="9">
-        <v>5</v>
-      </c>
-      <c r="G45" s="9">
+      <c r="F45" s="8">
+        <v>5</v>
+      </c>
+      <c r="G45" s="8">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="H45" s="10">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="I45" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J45" s="11">
+      <c r="H45" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="I45" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J45" s="10">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="K45" s="10">
+      <c r="K45" s="9">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L45" s="12">
-        <v>5</v>
-      </c>
-      <c r="M45" s="9"/>
-      <c r="N45" s="9"/>
-      <c r="O45" s="9"/>
-      <c r="P45" s="9"/>
+      <c r="L45" s="11">
+        <v>5</v>
+      </c>
+      <c r="M45" s="8"/>
+      <c r="N45" s="8"/>
+      <c r="O45" s="8"/>
+      <c r="P45" s="8"/>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
@@ -3038,41 +3036,41 @@
       <c r="C46" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D46" s="9">
+      <c r="D46" s="8">
         <v>56</v>
       </c>
-      <c r="E46" s="9">
+      <c r="E46" s="8">
         <v>143</v>
       </c>
-      <c r="F46" s="9">
-        <v>5</v>
-      </c>
-      <c r="G46" s="9">
+      <c r="F46" s="8">
+        <v>5</v>
+      </c>
+      <c r="G46" s="8">
         <f t="shared" si="0"/>
         <v>148</v>
       </c>
-      <c r="H46" s="10">
+      <c r="H46" s="9">
         <f t="shared" si="1"/>
         <v>49.333333333333336</v>
       </c>
-      <c r="I46" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J46" s="11">
+      <c r="I46" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J46" s="10">
         <f t="shared" si="2"/>
         <v>74</v>
       </c>
-      <c r="K46" s="10">
+      <c r="K46" s="9">
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="L46" s="12">
+      <c r="L46" s="11">
         <v>40</v>
       </c>
-      <c r="M46" s="9"/>
-      <c r="N46" s="9"/>
-      <c r="O46" s="9"/>
-      <c r="P46" s="9"/>
+      <c r="M46" s="8"/>
+      <c r="N46" s="8"/>
+      <c r="O46" s="8"/>
+      <c r="P46" s="8"/>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
@@ -3084,41 +3082,41 @@
       <c r="C47" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D47" s="9">
+      <c r="D47" s="8">
         <v>0</v>
       </c>
-      <c r="E47" s="9">
+      <c r="E47" s="8">
         <v>0</v>
       </c>
-      <c r="F47" s="9">
-        <v>5</v>
-      </c>
-      <c r="G47" s="9">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H47" s="10">
+      <c r="F47" s="8">
+        <v>5</v>
+      </c>
+      <c r="G47" s="8">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H47" s="9">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I47" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J47" s="11">
+      <c r="I47" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J47" s="10">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K47" s="10">
+      <c r="K47" s="9">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L47" s="12">
+      <c r="L47" s="11">
         <v>10</v>
       </c>
-      <c r="M47" s="9"/>
-      <c r="N47" s="9"/>
-      <c r="O47" s="9"/>
-      <c r="P47" s="9"/>
+      <c r="M47" s="8"/>
+      <c r="N47" s="8"/>
+      <c r="O47" s="8"/>
+      <c r="P47" s="8"/>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
@@ -3130,41 +3128,41 @@
       <c r="C48" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D48" s="9">
+      <c r="D48" s="8">
         <v>0</v>
       </c>
-      <c r="E48" s="9">
+      <c r="E48" s="8">
         <v>0</v>
       </c>
-      <c r="F48" s="9">
-        <v>5</v>
-      </c>
-      <c r="G48" s="9">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H48" s="10">
+      <c r="F48" s="8">
+        <v>5</v>
+      </c>
+      <c r="G48" s="8">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H48" s="9">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I48" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J48" s="11">
+      <c r="I48" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J48" s="10">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K48" s="10">
+      <c r="K48" s="9">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L48" s="12">
+      <c r="L48" s="11">
         <v>10</v>
       </c>
-      <c r="M48" s="9"/>
-      <c r="N48" s="9"/>
-      <c r="O48" s="9"/>
-      <c r="P48" s="9"/>
+      <c r="M48" s="8"/>
+      <c r="N48" s="8"/>
+      <c r="O48" s="8"/>
+      <c r="P48" s="8"/>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
@@ -3176,41 +3174,41 @@
       <c r="C49" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D49" s="9">
+      <c r="D49" s="8">
         <v>1</v>
       </c>
-      <c r="E49" s="9">
+      <c r="E49" s="8">
         <v>10</v>
       </c>
-      <c r="F49" s="9">
-        <v>5</v>
-      </c>
-      <c r="G49" s="9">
+      <c r="F49" s="8">
+        <v>5</v>
+      </c>
+      <c r="G49" s="8">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="H49" s="10">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="I49" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J49" s="11">
+      <c r="H49" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="I49" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J49" s="10">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="K49" s="10">
+      <c r="K49" s="9">
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="L49" s="12">
-        <v>5</v>
-      </c>
-      <c r="M49" s="9"/>
-      <c r="N49" s="9"/>
-      <c r="O49" s="9"/>
-      <c r="P49" s="9"/>
+      <c r="L49" s="11">
+        <v>5</v>
+      </c>
+      <c r="M49" s="8"/>
+      <c r="N49" s="8"/>
+      <c r="O49" s="8"/>
+      <c r="P49" s="8"/>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
@@ -3222,41 +3220,41 @@
       <c r="C50" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D50" s="9">
+      <c r="D50" s="8">
         <v>2</v>
       </c>
-      <c r="E50" s="9">
+      <c r="E50" s="8">
         <v>14</v>
       </c>
-      <c r="F50" s="9">
-        <v>5</v>
-      </c>
-      <c r="G50" s="9">
+      <c r="F50" s="8">
+        <v>5</v>
+      </c>
+      <c r="G50" s="8">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="H50" s="10">
+      <c r="H50" s="9">
         <f t="shared" si="1"/>
         <v>6.333333333333333</v>
       </c>
-      <c r="I50" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J50" s="11">
+      <c r="I50" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J50" s="10">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="K50" s="10">
+      <c r="K50" s="9">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="L50" s="12">
+      <c r="L50" s="11">
         <v>10</v>
       </c>
-      <c r="M50" s="9"/>
-      <c r="N50" s="9"/>
-      <c r="O50" s="9"/>
-      <c r="P50" s="9"/>
+      <c r="M50" s="8"/>
+      <c r="N50" s="8"/>
+      <c r="O50" s="8"/>
+      <c r="P50" s="8"/>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
@@ -3268,41 +3266,41 @@
       <c r="C51" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D51" s="9">
+      <c r="D51" s="8">
         <v>8</v>
       </c>
-      <c r="E51" s="9">
+      <c r="E51" s="8">
         <v>11</v>
       </c>
-      <c r="F51" s="9">
-        <v>5</v>
-      </c>
-      <c r="G51" s="9">
+      <c r="F51" s="8">
+        <v>5</v>
+      </c>
+      <c r="G51" s="8">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="H51" s="10">
+      <c r="H51" s="9">
         <f t="shared" si="1"/>
         <v>5.333333333333333</v>
       </c>
-      <c r="I51" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J51" s="11">
+      <c r="I51" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J51" s="10">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="K51" s="10">
+      <c r="K51" s="9">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L51" s="12">
+      <c r="L51" s="11">
         <v>10</v>
       </c>
-      <c r="M51" s="9"/>
-      <c r="N51" s="9"/>
-      <c r="O51" s="9"/>
-      <c r="P51" s="9"/>
+      <c r="M51" s="8"/>
+      <c r="N51" s="8"/>
+      <c r="O51" s="8"/>
+      <c r="P51" s="8"/>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
@@ -3314,41 +3312,41 @@
       <c r="C52" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D52" s="9">
+      <c r="D52" s="8">
         <v>0</v>
       </c>
-      <c r="E52" s="9">
+      <c r="E52" s="8">
         <v>0</v>
       </c>
-      <c r="F52" s="9">
-        <v>5</v>
-      </c>
-      <c r="G52" s="9">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H52" s="10">
+      <c r="F52" s="8">
+        <v>5</v>
+      </c>
+      <c r="G52" s="8">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H52" s="9">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I52" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J52" s="11">
+      <c r="I52" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J52" s="10">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K52" s="10">
+      <c r="K52" s="9">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L52" s="12">
-        <v>5</v>
-      </c>
-      <c r="M52" s="9"/>
-      <c r="N52" s="9"/>
-      <c r="O52" s="9"/>
-      <c r="P52" s="9"/>
+      <c r="L52" s="11">
+        <v>5</v>
+      </c>
+      <c r="M52" s="8"/>
+      <c r="N52" s="8"/>
+      <c r="O52" s="8"/>
+      <c r="P52" s="8"/>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
@@ -3360,43 +3358,43 @@
       <c r="C53" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D53" s="9">
+      <c r="D53" s="8">
         <v>2</v>
       </c>
-      <c r="E53" s="9">
+      <c r="E53" s="8">
         <v>3</v>
       </c>
-      <c r="F53" s="9">
-        <v>5</v>
-      </c>
-      <c r="G53" s="9">
+      <c r="F53" s="8">
+        <v>5</v>
+      </c>
+      <c r="G53" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="H53" s="10">
+      <c r="H53" s="9">
         <f t="shared" si="1"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="I53" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J53" s="11">
-        <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="K53" s="10">
+      <c r="I53" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J53" s="10">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="K53" s="9">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="L53" s="12">
+      <c r="L53" s="11">
         <v>10</v>
       </c>
-      <c r="M53" s="9"/>
-      <c r="N53" s="9" t="s">
+      <c r="M53" s="8"/>
+      <c r="N53" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="O53" s="9"/>
-      <c r="P53" s="9"/>
+      <c r="O53" s="8"/>
+      <c r="P53" s="8"/>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
@@ -3408,43 +3406,43 @@
       <c r="C54" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D54" s="9">
+      <c r="D54" s="8">
         <v>197</v>
       </c>
-      <c r="E54" s="9">
+      <c r="E54" s="8">
         <v>348</v>
       </c>
-      <c r="F54" s="9">
-        <v>5</v>
-      </c>
-      <c r="G54" s="9">
+      <c r="F54" s="8">
+        <v>5</v>
+      </c>
+      <c r="G54" s="8">
         <f t="shared" si="0"/>
         <v>353</v>
       </c>
-      <c r="H54" s="10">
+      <c r="H54" s="9">
         <f t="shared" si="1"/>
         <v>117.66666666666667</v>
       </c>
-      <c r="I54" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J54" s="11">
+      <c r="I54" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J54" s="10">
         <f t="shared" si="2"/>
         <v>177</v>
       </c>
-      <c r="K54" s="10">
+      <c r="K54" s="9">
         <f t="shared" si="3"/>
         <v>-20</v>
       </c>
-      <c r="L54" s="12">
+      <c r="L54" s="11">
         <v>120</v>
       </c>
-      <c r="M54" s="9" t="s">
+      <c r="M54" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="N54" s="9"/>
-      <c r="O54" s="9"/>
-      <c r="P54" s="9"/>
+      <c r="N54" s="8"/>
+      <c r="O54" s="8"/>
+      <c r="P54" s="8"/>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
@@ -3456,43 +3454,43 @@
       <c r="C55" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D55" s="9">
+      <c r="D55" s="8">
         <v>104</v>
       </c>
-      <c r="E55" s="9">
+      <c r="E55" s="8">
         <v>296</v>
       </c>
-      <c r="F55" s="9">
-        <v>5</v>
-      </c>
-      <c r="G55" s="9">
+      <c r="F55" s="8">
+        <v>5</v>
+      </c>
+      <c r="G55" s="8">
         <f t="shared" si="0"/>
         <v>301</v>
       </c>
-      <c r="H55" s="10">
+      <c r="H55" s="9">
         <f t="shared" si="1"/>
         <v>100.33333333333333</v>
       </c>
-      <c r="I55" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J55" s="11">
+      <c r="I55" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J55" s="10">
         <f t="shared" si="2"/>
         <v>151</v>
       </c>
-      <c r="K55" s="10">
+      <c r="K55" s="9">
         <f t="shared" si="3"/>
         <v>47</v>
       </c>
-      <c r="L55" s="12">
+      <c r="L55" s="11">
         <v>100</v>
       </c>
-      <c r="M55" s="9" t="s">
+      <c r="M55" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="N55" s="9"/>
-      <c r="O55" s="9"/>
-      <c r="P55" s="9"/>
+      <c r="N55" s="8"/>
+      <c r="O55" s="8"/>
+      <c r="P55" s="8"/>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
@@ -3504,41 +3502,41 @@
       <c r="C56" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D56" s="9">
+      <c r="D56" s="8">
         <v>29</v>
       </c>
-      <c r="E56" s="9">
+      <c r="E56" s="8">
         <v>61</v>
       </c>
-      <c r="F56" s="9">
-        <v>5</v>
-      </c>
-      <c r="G56" s="9">
+      <c r="F56" s="8">
+        <v>5</v>
+      </c>
+      <c r="G56" s="8">
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
-      <c r="H56" s="10">
+      <c r="H56" s="9">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="I56" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J56" s="11">
+      <c r="I56" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J56" s="10">
         <f t="shared" si="2"/>
         <v>33</v>
       </c>
-      <c r="K56" s="10">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="L56" s="12">
+      <c r="K56" s="9">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="L56" s="11">
         <v>10</v>
       </c>
-      <c r="M56" s="9"/>
-      <c r="N56" s="9"/>
-      <c r="O56" s="9"/>
-      <c r="P56" s="9"/>
+      <c r="M56" s="8"/>
+      <c r="N56" s="8"/>
+      <c r="O56" s="8"/>
+      <c r="P56" s="8"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
@@ -3550,43 +3548,43 @@
       <c r="C57" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D57" s="9">
+      <c r="D57" s="8">
         <v>6</v>
       </c>
-      <c r="E57" s="9">
+      <c r="E57" s="8">
         <v>27</v>
       </c>
-      <c r="F57" s="9">
-        <v>5</v>
-      </c>
-      <c r="G57" s="9">
+      <c r="F57" s="8">
+        <v>5</v>
+      </c>
+      <c r="G57" s="8">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="H57" s="10">
+      <c r="H57" s="9">
         <f t="shared" si="1"/>
         <v>10.666666666666666</v>
       </c>
-      <c r="I57" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J57" s="11">
+      <c r="I57" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J57" s="10">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="K57" s="10">
+      <c r="K57" s="9">
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="L57" s="12">
+      <c r="L57" s="11">
         <v>30</v>
       </c>
-      <c r="M57" s="9" t="s">
+      <c r="M57" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="N57" s="9"/>
-      <c r="O57" s="9"/>
-      <c r="P57" s="9"/>
+      <c r="N57" s="8"/>
+      <c r="O57" s="8"/>
+      <c r="P57" s="8"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
@@ -3598,41 +3596,41 @@
       <c r="C58" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D58" s="9">
+      <c r="D58" s="8">
         <v>0</v>
       </c>
-      <c r="E58" s="9">
+      <c r="E58" s="8">
         <v>0</v>
       </c>
-      <c r="F58" s="9">
-        <v>5</v>
-      </c>
-      <c r="G58" s="9">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H58" s="10">
+      <c r="F58" s="8">
+        <v>5</v>
+      </c>
+      <c r="G58" s="8">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H58" s="9">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I58" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J58" s="11">
+      <c r="I58" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J58" s="10">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K58" s="10">
+      <c r="K58" s="9">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L58" s="12">
+      <c r="L58" s="11">
         <v>10</v>
       </c>
-      <c r="M58" s="9"/>
-      <c r="N58" s="9"/>
-      <c r="O58" s="9"/>
-      <c r="P58" s="9"/>
+      <c r="M58" s="8"/>
+      <c r="N58" s="8"/>
+      <c r="O58" s="8"/>
+      <c r="P58" s="8"/>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
@@ -3644,41 +3642,41 @@
       <c r="C59" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D59" s="9">
+      <c r="D59" s="8">
         <v>0</v>
       </c>
-      <c r="E59" s="9">
+      <c r="E59" s="8">
         <v>0</v>
       </c>
-      <c r="F59" s="9">
-        <v>5</v>
-      </c>
-      <c r="G59" s="9">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H59" s="10">
+      <c r="F59" s="8">
+        <v>5</v>
+      </c>
+      <c r="G59" s="8">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H59" s="9">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I59" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J59" s="11">
+      <c r="I59" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J59" s="10">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K59" s="10">
+      <c r="K59" s="9">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L59" s="12">
+      <c r="L59" s="11">
         <v>30</v>
       </c>
-      <c r="M59" s="9"/>
-      <c r="N59" s="9"/>
-      <c r="O59" s="9"/>
-      <c r="P59" s="9"/>
+      <c r="M59" s="8"/>
+      <c r="N59" s="8"/>
+      <c r="O59" s="8"/>
+      <c r="P59" s="8"/>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
@@ -3690,41 +3688,41 @@
       <c r="C60" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D60" s="9">
+      <c r="D60" s="8">
         <v>0</v>
       </c>
-      <c r="E60" s="9">
+      <c r="E60" s="8">
         <v>0</v>
       </c>
-      <c r="F60" s="9">
-        <v>5</v>
-      </c>
-      <c r="G60" s="9">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H60" s="10">
+      <c r="F60" s="8">
+        <v>5</v>
+      </c>
+      <c r="G60" s="8">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H60" s="9">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I60" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J60" s="11">
+      <c r="I60" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J60" s="10">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K60" s="10">
+      <c r="K60" s="9">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L60" s="12">
+      <c r="L60" s="11">
         <v>30</v>
       </c>
-      <c r="M60" s="9"/>
-      <c r="N60" s="9"/>
-      <c r="O60" s="9"/>
-      <c r="P60" s="9"/>
+      <c r="M60" s="8"/>
+      <c r="N60" s="8"/>
+      <c r="O60" s="8"/>
+      <c r="P60" s="8"/>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
@@ -3736,43 +3734,43 @@
       <c r="C61" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D61" s="9">
+      <c r="D61" s="8">
         <v>27</v>
       </c>
-      <c r="E61" s="9">
+      <c r="E61" s="8">
         <v>74</v>
       </c>
-      <c r="F61" s="9">
-        <v>5</v>
-      </c>
-      <c r="G61" s="9">
+      <c r="F61" s="8">
+        <v>5</v>
+      </c>
+      <c r="G61" s="8">
         <f t="shared" si="0"/>
         <v>79</v>
       </c>
-      <c r="H61" s="10">
+      <c r="H61" s="9">
         <f t="shared" si="1"/>
         <v>26.333333333333332</v>
       </c>
-      <c r="I61" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J61" s="11">
+      <c r="I61" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J61" s="10">
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="K61" s="10">
+      <c r="K61" s="9">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="L61" s="12">
+      <c r="L61" s="11">
         <v>150</v>
       </c>
-      <c r="M61" s="9" t="s">
+      <c r="M61" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="N61" s="9"/>
-      <c r="O61" s="9"/>
-      <c r="P61" s="9"/>
+      <c r="N61" s="8"/>
+      <c r="O61" s="8"/>
+      <c r="P61" s="8"/>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
@@ -3784,46 +3782,45 @@
       <c r="C62" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D62" s="9">
+      <c r="D62" s="8">
         <v>2</v>
       </c>
-      <c r="E62" s="9">
+      <c r="E62" s="8">
         <v>2</v>
       </c>
-      <c r="F62" s="9">
-        <v>5</v>
-      </c>
-      <c r="G62" s="9">
+      <c r="F62" s="8">
+        <v>5</v>
+      </c>
+      <c r="G62" s="8">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="H62" s="10">
+      <c r="H62" s="9">
         <f t="shared" si="1"/>
         <v>2.3333333333333335</v>
       </c>
-      <c r="I62" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="J62" s="11">
-        <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="K62" s="10">
+      <c r="I62" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="J62" s="10">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="K62" s="9">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="L62" s="12">
+      <c r="L62" s="11">
         <v>20</v>
       </c>
-      <c r="M62" s="9" t="s">
+      <c r="M62" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="N62" s="9"/>
-      <c r="O62" s="9"/>
-      <c r="P62" s="9"/>
+      <c r="N62" s="8"/>
+      <c r="O62" s="8"/>
+      <c r="P62" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1" xr:uid="{96666041-4A3A-42C1-A22D-86A52389C7E2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add po requirement and remarks column in CB UI
</commit_message>
<xml_diff>
--- a/data/input/CB Replenishment_Master.xlsx
+++ b/data/input/CB Replenishment_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5EDE381-5347-4E11-9779-2217E51CC726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7ED1B49-A6D7-4797-8965-4C8E34D6B581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CFE25F1-D4D7-4072-B0D8-85CA58EF1A1A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$N$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$P$62</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -513,7 +513,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -535,6 +535,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -583,9 +589,6 @@
     <xf numFmtId="10" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -603,6 +606,9 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -970,19 +976,19 @@
       <c r="K1" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="M1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="N1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="O1" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="P1" s="6" t="s">
         <v>144</v>
       </c>
     </row>
@@ -996,43 +1002,43 @@
       <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D2" s="7">
         <v>624</v>
       </c>
-      <c r="E2" s="8">
+      <c r="E2" s="7">
         <v>1910</v>
       </c>
-      <c r="F2" s="8">
+      <c r="F2" s="7">
         <v>25</v>
       </c>
-      <c r="G2" s="8">
+      <c r="G2" s="7">
         <f>E2+F2</f>
         <v>1935</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="8">
         <f>G2/3</f>
         <v>645</v>
       </c>
-      <c r="I2" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J2" s="10">
+      <c r="I2" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J2" s="9">
         <f>ROUNDUP(H2*I2,0)</f>
         <v>968</v>
       </c>
-      <c r="K2" s="9">
+      <c r="K2" s="8">
         <f>J2-D2</f>
         <v>344</v>
       </c>
-      <c r="L2" s="11">
+      <c r="L2" s="10">
         <v>300</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="M2" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -1044,41 +1050,41 @@
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="7">
         <v>89</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="7">
         <v>240</v>
       </c>
-      <c r="F3" s="8">
-        <v>5</v>
-      </c>
-      <c r="G3" s="8">
+      <c r="F3" s="7">
+        <v>5</v>
+      </c>
+      <c r="G3" s="7">
         <f t="shared" ref="G3:G62" si="0">E3+F3</f>
         <v>245</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="8">
         <f t="shared" ref="H3:H62" si="1">G3/3</f>
         <v>81.666666666666671</v>
       </c>
-      <c r="I3" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J3" s="10">
+      <c r="I3" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J3" s="9">
         <f t="shared" ref="J3:J62" si="2">ROUNDUP(H3*I3,0)</f>
         <v>123</v>
       </c>
-      <c r="K3" s="9">
+      <c r="K3" s="8">
         <f t="shared" ref="K3:K62" si="3">J3-D3</f>
         <v>34</v>
       </c>
-      <c r="L3" s="11">
+      <c r="L3" s="10">
         <v>30</v>
       </c>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="8"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -1090,43 +1096,43 @@
       <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="7">
         <v>230</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="7">
         <v>731</v>
       </c>
-      <c r="F4" s="8">
-        <v>5</v>
-      </c>
-      <c r="G4" s="8">
+      <c r="F4" s="7">
+        <v>5</v>
+      </c>
+      <c r="G4" s="7">
         <f t="shared" si="0"/>
         <v>736</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="8">
         <f t="shared" si="1"/>
         <v>245.33333333333334</v>
       </c>
-      <c r="I4" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J4" s="10">
+      <c r="I4" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J4" s="9">
         <f t="shared" si="2"/>
         <v>368</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="8">
         <f t="shared" si="3"/>
         <v>138</v>
       </c>
-      <c r="L4" s="11">
+      <c r="L4" s="10">
         <v>100</v>
       </c>
-      <c r="M4" s="8" t="s">
+      <c r="M4" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
-      <c r="P4" s="8"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -1138,41 +1144,41 @@
       <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="7">
         <v>8</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="7">
         <v>37</v>
       </c>
-      <c r="F5" s="8">
-        <v>5</v>
-      </c>
-      <c r="G5" s="8">
+      <c r="F5" s="7">
+        <v>5</v>
+      </c>
+      <c r="G5" s="7">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="8">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
-      <c r="I5" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J5" s="10">
+      <c r="I5" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J5" s="9">
         <f t="shared" si="2"/>
         <v>21</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="8">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="10">
         <v>50</v>
       </c>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -1184,41 +1190,41 @@
       <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="7">
         <v>2</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="7">
         <v>1</v>
       </c>
-      <c r="F6" s="8">
-        <v>5</v>
-      </c>
-      <c r="G6" s="8">
+      <c r="F6" s="7">
+        <v>5</v>
+      </c>
+      <c r="G6" s="7">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="8">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="I6" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J6" s="10">
+      <c r="I6" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J6" s="9">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K6" s="9">
+      <c r="K6" s="8">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="L6" s="11">
+      <c r="L6" s="10">
         <v>20</v>
       </c>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="7"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
@@ -1230,43 +1236,43 @@
       <c r="C7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="7">
         <v>47</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="7">
         <v>202</v>
       </c>
-      <c r="F7" s="8">
-        <v>5</v>
-      </c>
-      <c r="G7" s="8">
+      <c r="F7" s="7">
+        <v>5</v>
+      </c>
+      <c r="G7" s="7">
         <f t="shared" si="0"/>
         <v>207</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="8">
         <f t="shared" si="1"/>
         <v>69</v>
       </c>
-      <c r="I7" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J7" s="10">
+      <c r="I7" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J7" s="9">
         <f t="shared" si="2"/>
         <v>104</v>
       </c>
-      <c r="K7" s="9">
+      <c r="K7" s="8">
         <f t="shared" si="3"/>
         <v>57</v>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="10">
         <v>120</v>
       </c>
-      <c r="M7" s="8" t="s">
+      <c r="M7" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="N7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -1278,41 +1284,41 @@
       <c r="C8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="7">
         <v>165</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="7">
         <v>662</v>
       </c>
-      <c r="F8" s="8">
-        <v>5</v>
-      </c>
-      <c r="G8" s="8">
+      <c r="F8" s="7">
+        <v>5</v>
+      </c>
+      <c r="G8" s="7">
         <f t="shared" si="0"/>
         <v>667</v>
       </c>
-      <c r="H8" s="9">
+      <c r="H8" s="8">
         <f t="shared" si="1"/>
         <v>222.33333333333334</v>
       </c>
-      <c r="I8" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J8" s="10">
+      <c r="I8" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J8" s="9">
         <f t="shared" si="2"/>
         <v>334</v>
       </c>
-      <c r="K8" s="9">
+      <c r="K8" s="8">
         <f t="shared" si="3"/>
         <v>169</v>
       </c>
-      <c r="L8" s="11">
+      <c r="L8" s="10">
         <v>120</v>
       </c>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -1324,41 +1330,41 @@
       <c r="C9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="7">
         <v>72</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="7">
         <v>175</v>
       </c>
-      <c r="F9" s="8">
-        <v>5</v>
-      </c>
-      <c r="G9" s="8">
+      <c r="F9" s="7">
+        <v>5</v>
+      </c>
+      <c r="G9" s="7">
         <f t="shared" si="0"/>
         <v>180</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="8">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
-      <c r="I9" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J9" s="10">
+      <c r="I9" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J9" s="9">
         <f t="shared" si="2"/>
         <v>90</v>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="8">
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="L9" s="11">
+      <c r="L9" s="10">
         <v>10</v>
       </c>
-      <c r="M9" s="8"/>
-      <c r="N9" s="8"/>
-      <c r="O9" s="8"/>
-      <c r="P9" s="8"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
@@ -1370,41 +1376,41 @@
       <c r="C10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="7">
         <v>26</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="7">
         <v>84</v>
       </c>
-      <c r="F10" s="8">
-        <v>5</v>
-      </c>
-      <c r="G10" s="8">
+      <c r="F10" s="7">
+        <v>5</v>
+      </c>
+      <c r="G10" s="7">
         <f t="shared" si="0"/>
         <v>89</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="8">
         <f t="shared" si="1"/>
         <v>29.666666666666668</v>
       </c>
-      <c r="I10" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J10" s="10">
+      <c r="I10" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J10" s="9">
         <f t="shared" si="2"/>
         <v>45</v>
       </c>
-      <c r="K10" s="9">
+      <c r="K10" s="8">
         <f t="shared" si="3"/>
         <v>19</v>
       </c>
-      <c r="L10" s="11">
+      <c r="L10" s="10">
         <v>50</v>
       </c>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -1416,41 +1422,41 @@
       <c r="C11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="7">
         <v>78</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="7">
         <v>253</v>
       </c>
-      <c r="F11" s="8">
-        <v>5</v>
-      </c>
-      <c r="G11" s="8">
+      <c r="F11" s="7">
+        <v>5</v>
+      </c>
+      <c r="G11" s="7">
         <f t="shared" si="0"/>
         <v>258</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="8">
         <f t="shared" si="1"/>
         <v>86</v>
       </c>
-      <c r="I11" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J11" s="10">
+      <c r="I11" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J11" s="9">
         <f t="shared" si="2"/>
         <v>129</v>
       </c>
-      <c r="K11" s="9">
+      <c r="K11" s="8">
         <f t="shared" si="3"/>
         <v>51</v>
       </c>
-      <c r="L11" s="12">
+      <c r="L11" s="11">
         <v>80</v>
       </c>
-      <c r="M11" s="8"/>
-      <c r="N11" s="8"/>
-      <c r="O11" s="8"/>
-      <c r="P11" s="8"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
@@ -1462,41 +1468,41 @@
       <c r="C12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="7">
         <v>100</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="7">
         <v>193</v>
       </c>
-      <c r="F12" s="8">
-        <v>5</v>
-      </c>
-      <c r="G12" s="8">
+      <c r="F12" s="7">
+        <v>5</v>
+      </c>
+      <c r="G12" s="7">
         <f t="shared" si="0"/>
         <v>198</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="8">
         <f t="shared" si="1"/>
         <v>66</v>
       </c>
-      <c r="I12" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J12" s="10">
+      <c r="I12" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J12" s="9">
         <f t="shared" si="2"/>
         <v>99</v>
       </c>
-      <c r="K12" s="9">
+      <c r="K12" s="8">
         <f t="shared" si="3"/>
         <v>-1</v>
       </c>
-      <c r="L12" s="11">
+      <c r="L12" s="10">
         <v>30</v>
       </c>
-      <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="8"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
@@ -1508,41 +1514,41 @@
       <c r="C13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="7">
         <v>137</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="7">
         <v>637</v>
       </c>
-      <c r="F13" s="8">
-        <v>5</v>
-      </c>
-      <c r="G13" s="8">
+      <c r="F13" s="7">
+        <v>5</v>
+      </c>
+      <c r="G13" s="7">
         <f t="shared" si="0"/>
         <v>642</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="8">
         <f t="shared" si="1"/>
         <v>214</v>
       </c>
-      <c r="I13" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J13" s="10">
+      <c r="I13" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J13" s="9">
         <f t="shared" si="2"/>
         <v>321</v>
       </c>
-      <c r="K13" s="9">
+      <c r="K13" s="8">
         <f t="shared" si="3"/>
         <v>184</v>
       </c>
-      <c r="L13" s="11">
+      <c r="L13" s="10">
         <v>160</v>
       </c>
-      <c r="M13" s="8"/>
-      <c r="N13" s="8"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="8"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
@@ -1554,41 +1560,41 @@
       <c r="C14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="7">
         <v>34</v>
       </c>
-      <c r="E14" s="8">
+      <c r="E14" s="7">
         <v>72</v>
       </c>
-      <c r="F14" s="8">
-        <v>5</v>
-      </c>
-      <c r="G14" s="8">
+      <c r="F14" s="7">
+        <v>5</v>
+      </c>
+      <c r="G14" s="7">
         <f t="shared" si="0"/>
         <v>77</v>
       </c>
-      <c r="H14" s="9">
+      <c r="H14" s="8">
         <f t="shared" si="1"/>
         <v>25.666666666666668</v>
       </c>
-      <c r="I14" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J14" s="10">
+      <c r="I14" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J14" s="9">
         <f t="shared" si="2"/>
         <v>39</v>
       </c>
-      <c r="K14" s="9">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="L14" s="11">
+      <c r="K14" s="8">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="L14" s="10">
         <v>20</v>
       </c>
-      <c r="M14" s="8"/>
-      <c r="N14" s="8"/>
-      <c r="O14" s="8"/>
-      <c r="P14" s="8"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
@@ -1600,41 +1606,41 @@
       <c r="C15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="7">
         <v>13</v>
       </c>
-      <c r="E15" s="8">
+      <c r="E15" s="7">
         <v>31</v>
       </c>
-      <c r="F15" s="8">
-        <v>5</v>
-      </c>
-      <c r="G15" s="8">
+      <c r="F15" s="7">
+        <v>5</v>
+      </c>
+      <c r="G15" s="7">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="H15" s="9">
+      <c r="H15" s="8">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="I15" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J15" s="10">
+      <c r="I15" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J15" s="9">
         <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="K15" s="9">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="L15" s="11">
+      <c r="K15" s="8">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="L15" s="10">
         <v>10</v>
       </c>
-      <c r="M15" s="8"/>
-      <c r="N15" s="8"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="8"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -1646,41 +1652,41 @@
       <c r="C16" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="7">
         <v>21</v>
       </c>
-      <c r="E16" s="8">
+      <c r="E16" s="7">
         <v>27</v>
       </c>
-      <c r="F16" s="8">
-        <v>5</v>
-      </c>
-      <c r="G16" s="8">
+      <c r="F16" s="7">
+        <v>5</v>
+      </c>
+      <c r="G16" s="7">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="H16" s="9">
+      <c r="H16" s="8">
         <f t="shared" si="1"/>
         <v>10.666666666666666</v>
       </c>
-      <c r="I16" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J16" s="10">
+      <c r="I16" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J16" s="9">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="K16" s="9">
+      <c r="K16" s="8">
         <f t="shared" si="3"/>
         <v>-5</v>
       </c>
-      <c r="L16" s="11">
+      <c r="L16" s="10">
         <v>20</v>
       </c>
-      <c r="M16" s="8"/>
-      <c r="N16" s="8"/>
-      <c r="O16" s="8"/>
-      <c r="P16" s="8"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
@@ -1692,41 +1698,41 @@
       <c r="C17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="7">
         <v>21</v>
       </c>
-      <c r="E17" s="8">
+      <c r="E17" s="7">
         <v>32</v>
       </c>
-      <c r="F17" s="8">
-        <v>5</v>
-      </c>
-      <c r="G17" s="8">
+      <c r="F17" s="7">
+        <v>5</v>
+      </c>
+      <c r="G17" s="7">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="H17" s="9">
+      <c r="H17" s="8">
         <f t="shared" si="1"/>
         <v>12.333333333333334</v>
       </c>
-      <c r="I17" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J17" s="10">
+      <c r="I17" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J17" s="9">
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="K17" s="9">
+      <c r="K17" s="8">
         <f t="shared" si="3"/>
         <v>-2</v>
       </c>
-      <c r="L17" s="11">
+      <c r="L17" s="10">
         <v>10</v>
       </c>
-      <c r="M17" s="8"/>
-      <c r="N17" s="8"/>
-      <c r="O17" s="8"/>
-      <c r="P17" s="8"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
@@ -1738,41 +1744,41 @@
       <c r="C18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="7">
         <v>10</v>
       </c>
-      <c r="E18" s="8">
+      <c r="E18" s="7">
         <v>29</v>
       </c>
-      <c r="F18" s="8">
-        <v>5</v>
-      </c>
-      <c r="G18" s="8">
+      <c r="F18" s="7">
+        <v>5</v>
+      </c>
+      <c r="G18" s="7">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="H18" s="9">
+      <c r="H18" s="8">
         <f t="shared" si="1"/>
         <v>11.333333333333334</v>
       </c>
-      <c r="I18" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J18" s="10">
+      <c r="I18" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J18" s="9">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="K18" s="9">
+      <c r="K18" s="8">
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="L18" s="11">
+      <c r="L18" s="10">
         <v>20</v>
       </c>
-      <c r="M18" s="8"/>
-      <c r="N18" s="8"/>
-      <c r="O18" s="8"/>
-      <c r="P18" s="8"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
@@ -1784,41 +1790,41 @@
       <c r="C19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="7">
         <v>106</v>
       </c>
-      <c r="E19" s="8">
+      <c r="E19" s="7">
         <v>344</v>
       </c>
-      <c r="F19" s="8">
-        <v>5</v>
-      </c>
-      <c r="G19" s="8">
+      <c r="F19" s="7">
+        <v>5</v>
+      </c>
+      <c r="G19" s="7">
         <f t="shared" si="0"/>
         <v>349</v>
       </c>
-      <c r="H19" s="9">
+      <c r="H19" s="8">
         <f t="shared" si="1"/>
         <v>116.33333333333333</v>
       </c>
-      <c r="I19" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J19" s="10">
+      <c r="I19" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J19" s="9">
         <f t="shared" si="2"/>
         <v>175</v>
       </c>
-      <c r="K19" s="9">
+      <c r="K19" s="8">
         <f t="shared" si="3"/>
         <v>69</v>
       </c>
-      <c r="L19" s="11">
+      <c r="L19" s="10">
         <v>30</v>
       </c>
-      <c r="M19" s="8"/>
-      <c r="N19" s="8"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="8"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="7"/>
+      <c r="O19" s="7"/>
+      <c r="P19" s="7"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
@@ -1830,41 +1836,41 @@
       <c r="C20" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="7">
         <v>31</v>
       </c>
-      <c r="E20" s="8">
+      <c r="E20" s="7">
         <v>84</v>
       </c>
-      <c r="F20" s="8">
-        <v>5</v>
-      </c>
-      <c r="G20" s="8">
+      <c r="F20" s="7">
+        <v>5</v>
+      </c>
+      <c r="G20" s="7">
         <f t="shared" si="0"/>
         <v>89</v>
       </c>
-      <c r="H20" s="9">
+      <c r="H20" s="8">
         <f t="shared" si="1"/>
         <v>29.666666666666668</v>
       </c>
-      <c r="I20" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J20" s="10">
+      <c r="I20" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J20" s="9">
         <f t="shared" si="2"/>
         <v>45</v>
       </c>
-      <c r="K20" s="9">
+      <c r="K20" s="8">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="L20" s="11">
+      <c r="L20" s="10">
         <v>20</v>
       </c>
-      <c r="M20" s="8"/>
-      <c r="N20" s="8"/>
-      <c r="O20" s="8"/>
-      <c r="P20" s="8"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="7"/>
+      <c r="O20" s="7"/>
+      <c r="P20" s="7"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
@@ -1876,41 +1882,41 @@
       <c r="C21" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="8">
+      <c r="D21" s="7">
         <v>42</v>
       </c>
-      <c r="E21" s="8">
+      <c r="E21" s="7">
         <v>86</v>
       </c>
-      <c r="F21" s="8">
-        <v>5</v>
-      </c>
-      <c r="G21" s="8">
+      <c r="F21" s="7">
+        <v>5</v>
+      </c>
+      <c r="G21" s="7">
         <f t="shared" si="0"/>
         <v>91</v>
       </c>
-      <c r="H21" s="9">
+      <c r="H21" s="8">
         <f t="shared" si="1"/>
         <v>30.333333333333332</v>
       </c>
-      <c r="I21" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J21" s="10">
+      <c r="I21" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J21" s="9">
         <f t="shared" si="2"/>
         <v>46</v>
       </c>
-      <c r="K21" s="9">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="L21" s="11">
+      <c r="K21" s="8">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="L21" s="10">
         <v>20</v>
       </c>
-      <c r="M21" s="8"/>
-      <c r="N21" s="8"/>
-      <c r="O21" s="8"/>
-      <c r="P21" s="8"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="7"/>
+      <c r="P21" s="7"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
@@ -1922,41 +1928,41 @@
       <c r="C22" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D22" s="8">
+      <c r="D22" s="7">
         <v>39</v>
       </c>
-      <c r="E22" s="8">
+      <c r="E22" s="7">
         <v>67</v>
       </c>
-      <c r="F22" s="8">
-        <v>5</v>
-      </c>
-      <c r="G22" s="8">
+      <c r="F22" s="7">
+        <v>5</v>
+      </c>
+      <c r="G22" s="7">
         <f t="shared" si="0"/>
         <v>72</v>
       </c>
-      <c r="H22" s="9">
+      <c r="H22" s="8">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="I22" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J22" s="10">
+      <c r="I22" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J22" s="9">
         <f t="shared" si="2"/>
         <v>36</v>
       </c>
-      <c r="K22" s="9">
+      <c r="K22" s="8">
         <f t="shared" si="3"/>
         <v>-3</v>
       </c>
-      <c r="L22" s="11">
+      <c r="L22" s="10">
         <v>10</v>
       </c>
-      <c r="M22" s="8"/>
-      <c r="N22" s="8"/>
-      <c r="O22" s="8"/>
-      <c r="P22" s="8"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="7"/>
+      <c r="O22" s="7"/>
+      <c r="P22" s="7"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
@@ -1968,41 +1974,41 @@
       <c r="C23" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="7">
         <v>30</v>
       </c>
-      <c r="E23" s="8">
+      <c r="E23" s="7">
         <v>53</v>
       </c>
-      <c r="F23" s="8">
-        <v>5</v>
-      </c>
-      <c r="G23" s="8">
+      <c r="F23" s="7">
+        <v>5</v>
+      </c>
+      <c r="G23" s="7">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="8">
         <f t="shared" si="1"/>
         <v>19.333333333333332</v>
       </c>
-      <c r="I23" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J23" s="10">
+      <c r="I23" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J23" s="9">
         <f t="shared" si="2"/>
         <v>29</v>
       </c>
-      <c r="K23" s="9">
+      <c r="K23" s="8">
         <f t="shared" si="3"/>
         <v>-1</v>
       </c>
-      <c r="L23" s="11">
+      <c r="L23" s="10">
         <v>20</v>
       </c>
-      <c r="M23" s="8"/>
-      <c r="N23" s="8"/>
-      <c r="O23" s="8"/>
-      <c r="P23" s="8"/>
+      <c r="M23" s="7"/>
+      <c r="N23" s="7"/>
+      <c r="O23" s="7"/>
+      <c r="P23" s="7"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
@@ -2014,43 +2020,43 @@
       <c r="C24" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="7">
         <v>35</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E24" s="7">
         <v>19</v>
       </c>
-      <c r="F24" s="8">
-        <v>5</v>
-      </c>
-      <c r="G24" s="8">
+      <c r="F24" s="7">
+        <v>5</v>
+      </c>
+      <c r="G24" s="7">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="H24" s="9">
+      <c r="H24" s="8">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="I24" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J24" s="10">
+      <c r="I24" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J24" s="9">
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="K24" s="9">
+      <c r="K24" s="8">
         <f t="shared" si="3"/>
         <v>-23</v>
       </c>
-      <c r="L24" s="11">
+      <c r="L24" s="10">
         <v>30</v>
       </c>
-      <c r="M24" s="8" t="s">
+      <c r="M24" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="N24" s="8"/>
-      <c r="O24" s="8"/>
-      <c r="P24" s="8"/>
+      <c r="N24" s="7"/>
+      <c r="O24" s="7"/>
+      <c r="P24" s="7"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
@@ -2062,41 +2068,41 @@
       <c r="C25" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="7">
         <v>49</v>
       </c>
-      <c r="E25" s="8">
+      <c r="E25" s="7">
         <v>141</v>
       </c>
-      <c r="F25" s="8">
-        <v>5</v>
-      </c>
-      <c r="G25" s="8">
+      <c r="F25" s="7">
+        <v>5</v>
+      </c>
+      <c r="G25" s="7">
         <f t="shared" si="0"/>
         <v>146</v>
       </c>
-      <c r="H25" s="9">
+      <c r="H25" s="8">
         <f t="shared" si="1"/>
         <v>48.666666666666664</v>
       </c>
-      <c r="I25" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J25" s="10">
+      <c r="I25" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J25" s="9">
         <f t="shared" si="2"/>
         <v>73</v>
       </c>
-      <c r="K25" s="9">
+      <c r="K25" s="8">
         <f t="shared" si="3"/>
         <v>24</v>
       </c>
-      <c r="L25" s="11">
+      <c r="L25" s="10">
         <v>20</v>
       </c>
-      <c r="M25" s="8"/>
-      <c r="N25" s="8"/>
-      <c r="O25" s="8"/>
-      <c r="P25" s="8"/>
+      <c r="M25" s="7"/>
+      <c r="N25" s="7"/>
+      <c r="O25" s="7"/>
+      <c r="P25" s="7"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
@@ -2108,41 +2114,41 @@
       <c r="C26" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="7">
         <v>53</v>
       </c>
-      <c r="E26" s="8">
+      <c r="E26" s="7">
         <v>149</v>
       </c>
-      <c r="F26" s="8">
-        <v>5</v>
-      </c>
-      <c r="G26" s="8">
+      <c r="F26" s="7">
+        <v>5</v>
+      </c>
+      <c r="G26" s="7">
         <f t="shared" si="0"/>
         <v>154</v>
       </c>
-      <c r="H26" s="9">
+      <c r="H26" s="8">
         <f t="shared" si="1"/>
         <v>51.333333333333336</v>
       </c>
-      <c r="I26" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J26" s="10">
+      <c r="I26" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J26" s="9">
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
-      <c r="K26" s="9">
+      <c r="K26" s="8">
         <f t="shared" si="3"/>
         <v>24</v>
       </c>
-      <c r="L26" s="11">
+      <c r="L26" s="10">
         <v>50</v>
       </c>
-      <c r="M26" s="8"/>
-      <c r="N26" s="8"/>
-      <c r="O26" s="8"/>
-      <c r="P26" s="8"/>
+      <c r="M26" s="7"/>
+      <c r="N26" s="7"/>
+      <c r="O26" s="7"/>
+      <c r="P26" s="7"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
@@ -2154,41 +2160,41 @@
       <c r="C27" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="7">
         <v>43</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E27" s="7">
         <v>107</v>
       </c>
-      <c r="F27" s="8">
-        <v>5</v>
-      </c>
-      <c r="G27" s="8">
+      <c r="F27" s="7">
+        <v>5</v>
+      </c>
+      <c r="G27" s="7">
         <f t="shared" si="0"/>
         <v>112</v>
       </c>
-      <c r="H27" s="9">
+      <c r="H27" s="8">
         <f t="shared" si="1"/>
         <v>37.333333333333336</v>
       </c>
-      <c r="I27" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J27" s="10">
+      <c r="I27" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J27" s="9">
         <f t="shared" si="2"/>
         <v>56</v>
       </c>
-      <c r="K27" s="9">
+      <c r="K27" s="8">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="L27" s="11">
+      <c r="L27" s="10">
         <v>20</v>
       </c>
-      <c r="M27" s="8"/>
-      <c r="N27" s="8"/>
-      <c r="O27" s="8"/>
-      <c r="P27" s="8"/>
+      <c r="M27" s="7"/>
+      <c r="N27" s="7"/>
+      <c r="O27" s="7"/>
+      <c r="P27" s="7"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
@@ -2200,41 +2206,41 @@
       <c r="C28" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D28" s="8">
+      <c r="D28" s="7">
         <v>21</v>
       </c>
-      <c r="E28" s="8">
+      <c r="E28" s="7">
         <v>48</v>
       </c>
-      <c r="F28" s="8">
-        <v>5</v>
-      </c>
-      <c r="G28" s="8">
+      <c r="F28" s="7">
+        <v>5</v>
+      </c>
+      <c r="G28" s="7">
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
-      <c r="H28" s="9">
+      <c r="H28" s="8">
         <f t="shared" si="1"/>
         <v>17.666666666666668</v>
       </c>
-      <c r="I28" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J28" s="10">
+      <c r="I28" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J28" s="9">
         <f t="shared" si="2"/>
         <v>27</v>
       </c>
-      <c r="K28" s="9">
+      <c r="K28" s="8">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L28" s="11">
+      <c r="L28" s="10">
         <v>10</v>
       </c>
-      <c r="M28" s="8"/>
-      <c r="N28" s="8"/>
-      <c r="O28" s="8"/>
-      <c r="P28" s="8"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="7"/>
+      <c r="O28" s="7"/>
+      <c r="P28" s="7"/>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -2246,41 +2252,41 @@
       <c r="C29" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="7">
         <v>27</v>
       </c>
-      <c r="E29" s="8">
+      <c r="E29" s="7">
         <v>78</v>
       </c>
-      <c r="F29" s="8">
-        <v>5</v>
-      </c>
-      <c r="G29" s="8">
+      <c r="F29" s="7">
+        <v>5</v>
+      </c>
+      <c r="G29" s="7">
         <f t="shared" si="0"/>
         <v>83</v>
       </c>
-      <c r="H29" s="9">
+      <c r="H29" s="8">
         <f t="shared" si="1"/>
         <v>27.666666666666668</v>
       </c>
-      <c r="I29" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J29" s="10">
+      <c r="I29" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J29" s="9">
         <f t="shared" si="2"/>
         <v>42</v>
       </c>
-      <c r="K29" s="9">
+      <c r="K29" s="8">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="L29" s="11">
+      <c r="L29" s="10">
         <v>10</v>
       </c>
-      <c r="M29" s="8"/>
-      <c r="N29" s="8"/>
-      <c r="O29" s="8"/>
-      <c r="P29" s="8"/>
+      <c r="M29" s="7"/>
+      <c r="N29" s="7"/>
+      <c r="O29" s="7"/>
+      <c r="P29" s="7"/>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
@@ -2292,41 +2298,41 @@
       <c r="C30" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D30" s="8">
+      <c r="D30" s="7">
         <v>2</v>
       </c>
-      <c r="E30" s="8">
+      <c r="E30" s="7">
         <v>3</v>
       </c>
-      <c r="F30" s="8">
-        <v>5</v>
-      </c>
-      <c r="G30" s="8">
+      <c r="F30" s="7">
+        <v>5</v>
+      </c>
+      <c r="G30" s="7">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="H30" s="9">
+      <c r="H30" s="8">
         <f t="shared" si="1"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="I30" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J30" s="10">
-        <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="K30" s="9">
+      <c r="I30" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J30" s="9">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="K30" s="8">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="L30" s="11">
+      <c r="L30" s="10">
         <v>10</v>
       </c>
-      <c r="M30" s="8"/>
-      <c r="N30" s="8"/>
-      <c r="O30" s="8"/>
-      <c r="P30" s="8"/>
+      <c r="M30" s="7"/>
+      <c r="N30" s="7"/>
+      <c r="O30" s="7"/>
+      <c r="P30" s="7"/>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
@@ -2338,43 +2344,43 @@
       <c r="C31" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D31" s="8">
-        <v>5</v>
-      </c>
-      <c r="E31" s="8">
+      <c r="D31" s="7">
+        <v>5</v>
+      </c>
+      <c r="E31" s="7">
         <v>17</v>
       </c>
-      <c r="F31" s="8">
-        <v>5</v>
-      </c>
-      <c r="G31" s="8">
+      <c r="F31" s="7">
+        <v>5</v>
+      </c>
+      <c r="G31" s="7">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="H31" s="9">
+      <c r="H31" s="8">
         <f t="shared" si="1"/>
         <v>7.333333333333333</v>
       </c>
-      <c r="I31" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J31" s="10">
+      <c r="I31" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J31" s="9">
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="K31" s="9">
+      <c r="K31" s="8">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L31" s="11">
+      <c r="L31" s="10">
         <v>20</v>
       </c>
-      <c r="M31" s="8" t="s">
+      <c r="M31" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="N31" s="8"/>
-      <c r="O31" s="8"/>
-      <c r="P31" s="8"/>
+      <c r="N31" s="7"/>
+      <c r="O31" s="7"/>
+      <c r="P31" s="7"/>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
@@ -2386,41 +2392,41 @@
       <c r="C32" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D32" s="8">
-        <v>5</v>
-      </c>
-      <c r="E32" s="8">
-        <v>5</v>
-      </c>
-      <c r="F32" s="8">
-        <v>5</v>
-      </c>
-      <c r="G32" s="8">
+      <c r="D32" s="7">
+        <v>5</v>
+      </c>
+      <c r="E32" s="7">
+        <v>5</v>
+      </c>
+      <c r="F32" s="7">
+        <v>5</v>
+      </c>
+      <c r="G32" s="7">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="H32" s="9">
+      <c r="H32" s="8">
         <f t="shared" si="1"/>
         <v>3.3333333333333335</v>
       </c>
-      <c r="I32" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J32" s="10">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="K32" s="9">
+      <c r="I32" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J32" s="9">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="K32" s="8">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L32" s="11">
+      <c r="L32" s="10">
         <v>10</v>
       </c>
-      <c r="M32" s="8"/>
-      <c r="N32" s="8"/>
-      <c r="O32" s="8"/>
-      <c r="P32" s="8"/>
+      <c r="M32" s="7"/>
+      <c r="N32" s="7"/>
+      <c r="O32" s="7"/>
+      <c r="P32" s="7"/>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
@@ -2432,41 +2438,41 @@
       <c r="C33" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D33" s="8">
+      <c r="D33" s="7">
         <v>45</v>
       </c>
-      <c r="E33" s="8">
+      <c r="E33" s="7">
         <v>118</v>
       </c>
-      <c r="F33" s="8">
-        <v>5</v>
-      </c>
-      <c r="G33" s="8">
+      <c r="F33" s="7">
+        <v>5</v>
+      </c>
+      <c r="G33" s="7">
         <f t="shared" si="0"/>
         <v>123</v>
       </c>
-      <c r="H33" s="9">
+      <c r="H33" s="8">
         <f t="shared" si="1"/>
         <v>41</v>
       </c>
-      <c r="I33" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J33" s="10">
+      <c r="I33" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J33" s="9">
         <f t="shared" si="2"/>
         <v>62</v>
       </c>
-      <c r="K33" s="9">
+      <c r="K33" s="8">
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="L33" s="11">
+      <c r="L33" s="10">
         <v>20</v>
       </c>
-      <c r="M33" s="8"/>
-      <c r="N33" s="8"/>
-      <c r="O33" s="8"/>
-      <c r="P33" s="8"/>
+      <c r="M33" s="7"/>
+      <c r="N33" s="7"/>
+      <c r="O33" s="7"/>
+      <c r="P33" s="7"/>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
@@ -2478,41 +2484,41 @@
       <c r="C34" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D34" s="8">
+      <c r="D34" s="7">
         <v>13</v>
       </c>
-      <c r="E34" s="8">
+      <c r="E34" s="7">
         <v>28</v>
       </c>
-      <c r="F34" s="8">
-        <v>5</v>
-      </c>
-      <c r="G34" s="8">
+      <c r="F34" s="7">
+        <v>5</v>
+      </c>
+      <c r="G34" s="7">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="H34" s="9">
+      <c r="H34" s="8">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="I34" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J34" s="10">
+      <c r="I34" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J34" s="9">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="K34" s="9">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="L34" s="11">
+      <c r="K34" s="8">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="L34" s="10">
         <v>10</v>
       </c>
-      <c r="M34" s="8"/>
-      <c r="N34" s="8"/>
-      <c r="O34" s="8"/>
-      <c r="P34" s="8"/>
+      <c r="M34" s="7"/>
+      <c r="N34" s="7"/>
+      <c r="O34" s="7"/>
+      <c r="P34" s="7"/>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -2524,43 +2530,43 @@
       <c r="C35" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D35" s="8">
+      <c r="D35" s="7">
         <v>6</v>
       </c>
-      <c r="E35" s="8">
+      <c r="E35" s="7">
         <v>10</v>
       </c>
-      <c r="F35" s="8">
-        <v>5</v>
-      </c>
-      <c r="G35" s="8">
+      <c r="F35" s="7">
+        <v>5</v>
+      </c>
+      <c r="G35" s="7">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="H35" s="9">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="I35" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J35" s="10">
+      <c r="H35" s="8">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="I35" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J35" s="9">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="K35" s="9">
+      <c r="K35" s="8">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="L35" s="11">
+      <c r="L35" s="10">
         <v>20</v>
       </c>
-      <c r="M35" s="8" t="s">
+      <c r="M35" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
-      <c r="P35" s="8"/>
+      <c r="N35" s="7"/>
+      <c r="O35" s="7"/>
+      <c r="P35" s="7"/>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
@@ -2572,43 +2578,43 @@
       <c r="C36" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D36" s="8">
+      <c r="D36" s="7">
         <v>223</v>
       </c>
-      <c r="E36" s="8">
+      <c r="E36" s="7">
         <v>654</v>
       </c>
-      <c r="F36" s="8">
-        <v>5</v>
-      </c>
-      <c r="G36" s="8">
+      <c r="F36" s="7">
+        <v>5</v>
+      </c>
+      <c r="G36" s="7">
         <f t="shared" si="0"/>
         <v>659</v>
       </c>
-      <c r="H36" s="9">
+      <c r="H36" s="8">
         <f t="shared" si="1"/>
         <v>219.66666666666666</v>
       </c>
-      <c r="I36" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J36" s="10">
+      <c r="I36" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J36" s="9">
         <f t="shared" si="2"/>
         <v>330</v>
       </c>
-      <c r="K36" s="9">
+      <c r="K36" s="8">
         <f t="shared" si="3"/>
         <v>107</v>
       </c>
-      <c r="L36" s="11">
+      <c r="L36" s="10">
         <v>150</v>
       </c>
-      <c r="M36" s="8" t="s">
+      <c r="M36" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="N36" s="8"/>
-      <c r="O36" s="8"/>
-      <c r="P36" s="8"/>
+      <c r="N36" s="7"/>
+      <c r="O36" s="7"/>
+      <c r="P36" s="7"/>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
@@ -2620,41 +2626,41 @@
       <c r="C37" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D37" s="8">
+      <c r="D37" s="7">
         <v>0</v>
       </c>
-      <c r="E37" s="8">
+      <c r="E37" s="7">
         <v>7</v>
       </c>
-      <c r="F37" s="8">
-        <v>5</v>
-      </c>
-      <c r="G37" s="8">
+      <c r="F37" s="7">
+        <v>5</v>
+      </c>
+      <c r="G37" s="7">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="H37" s="9">
-        <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="I37" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J37" s="10">
+      <c r="H37" s="8">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="I37" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J37" s="9">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="K37" s="9">
+      <c r="K37" s="8">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L37" s="11">
+      <c r="L37" s="10">
         <v>10</v>
       </c>
-      <c r="M37" s="8"/>
-      <c r="N37" s="8"/>
-      <c r="O37" s="8"/>
-      <c r="P37" s="8"/>
+      <c r="M37" s="7"/>
+      <c r="N37" s="7"/>
+      <c r="O37" s="7"/>
+      <c r="P37" s="7"/>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
@@ -2666,43 +2672,43 @@
       <c r="C38" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D38" s="8">
+      <c r="D38" s="7">
         <v>23</v>
       </c>
-      <c r="E38" s="8">
+      <c r="E38" s="7">
         <v>32</v>
       </c>
-      <c r="F38" s="8">
-        <v>5</v>
-      </c>
-      <c r="G38" s="8">
+      <c r="F38" s="7">
+        <v>5</v>
+      </c>
+      <c r="G38" s="7">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="H38" s="9">
+      <c r="H38" s="8">
         <f t="shared" si="1"/>
         <v>12.333333333333334</v>
       </c>
-      <c r="I38" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J38" s="10">
+      <c r="I38" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J38" s="9">
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="K38" s="9">
+      <c r="K38" s="8">
         <f t="shared" si="3"/>
         <v>-4</v>
       </c>
-      <c r="L38" s="11">
+      <c r="L38" s="10">
         <v>100</v>
       </c>
-      <c r="M38" s="8" t="s">
+      <c r="M38" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="N38" s="8"/>
-      <c r="O38" s="8"/>
-      <c r="P38" s="8"/>
+      <c r="N38" s="7"/>
+      <c r="O38" s="7"/>
+      <c r="P38" s="7"/>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
@@ -2714,41 +2720,41 @@
       <c r="C39" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D39" s="8">
+      <c r="D39" s="7">
         <v>16</v>
       </c>
-      <c r="E39" s="8">
+      <c r="E39" s="7">
         <v>38</v>
       </c>
-      <c r="F39" s="8">
-        <v>5</v>
-      </c>
-      <c r="G39" s="8">
+      <c r="F39" s="7">
+        <v>5</v>
+      </c>
+      <c r="G39" s="7">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="H39" s="9">
+      <c r="H39" s="8">
         <f t="shared" si="1"/>
         <v>14.333333333333334</v>
       </c>
-      <c r="I39" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J39" s="10">
+      <c r="I39" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J39" s="9">
         <f t="shared" si="2"/>
         <v>22</v>
       </c>
-      <c r="K39" s="9">
+      <c r="K39" s="8">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L39" s="11">
+      <c r="L39" s="10">
         <v>10</v>
       </c>
-      <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="8"/>
-      <c r="P39" s="8"/>
+      <c r="M39" s="7"/>
+      <c r="N39" s="7"/>
+      <c r="O39" s="7"/>
+      <c r="P39" s="7"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
@@ -2760,41 +2766,41 @@
       <c r="C40" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D40" s="8">
+      <c r="D40" s="7">
         <v>35</v>
       </c>
-      <c r="E40" s="8">
+      <c r="E40" s="7">
         <v>75</v>
       </c>
-      <c r="F40" s="8">
-        <v>5</v>
-      </c>
-      <c r="G40" s="8">
+      <c r="F40" s="7">
+        <v>5</v>
+      </c>
+      <c r="G40" s="7">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="H40" s="9">
+      <c r="H40" s="8">
         <f t="shared" si="1"/>
         <v>26.666666666666668</v>
       </c>
-      <c r="I40" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J40" s="10">
+      <c r="I40" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J40" s="9">
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="K40" s="9">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="L40" s="11">
+      <c r="K40" s="8">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="L40" s="10">
         <v>20</v>
       </c>
-      <c r="M40" s="8"/>
-      <c r="N40" s="8"/>
-      <c r="O40" s="8"/>
-      <c r="P40" s="8"/>
+      <c r="M40" s="7"/>
+      <c r="N40" s="7"/>
+      <c r="O40" s="7"/>
+      <c r="P40" s="7"/>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -2806,41 +2812,41 @@
       <c r="C41" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D41" s="8">
+      <c r="D41" s="7">
         <v>14</v>
       </c>
-      <c r="E41" s="8">
+      <c r="E41" s="7">
         <v>47</v>
       </c>
-      <c r="F41" s="8">
-        <v>5</v>
-      </c>
-      <c r="G41" s="8">
+      <c r="F41" s="7">
+        <v>5</v>
+      </c>
+      <c r="G41" s="7">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="H41" s="9">
+      <c r="H41" s="8">
         <f t="shared" si="1"/>
         <v>17.333333333333332</v>
       </c>
-      <c r="I41" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J41" s="10">
+      <c r="I41" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J41" s="9">
         <f t="shared" si="2"/>
         <v>26</v>
       </c>
-      <c r="K41" s="9">
+      <c r="K41" s="8">
         <f t="shared" si="3"/>
         <v>12</v>
       </c>
-      <c r="L41" s="11">
+      <c r="L41" s="10">
         <v>20</v>
       </c>
-      <c r="M41" s="8"/>
-      <c r="N41" s="8"/>
-      <c r="O41" s="8"/>
-      <c r="P41" s="8"/>
+      <c r="M41" s="7"/>
+      <c r="N41" s="7"/>
+      <c r="O41" s="7"/>
+      <c r="P41" s="7"/>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
@@ -2852,41 +2858,41 @@
       <c r="C42" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D42" s="8">
+      <c r="D42" s="7">
         <v>40</v>
       </c>
-      <c r="E42" s="8">
+      <c r="E42" s="7">
         <v>91</v>
       </c>
-      <c r="F42" s="8">
-        <v>5</v>
-      </c>
-      <c r="G42" s="8">
+      <c r="F42" s="7">
+        <v>5</v>
+      </c>
+      <c r="G42" s="7">
         <f t="shared" si="0"/>
         <v>96</v>
       </c>
-      <c r="H42" s="9">
+      <c r="H42" s="8">
         <f t="shared" si="1"/>
         <v>32</v>
       </c>
-      <c r="I42" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J42" s="10">
+      <c r="I42" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J42" s="9">
         <f t="shared" si="2"/>
         <v>48</v>
       </c>
-      <c r="K42" s="9">
+      <c r="K42" s="8">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="L42" s="11">
+      <c r="L42" s="10">
         <v>40</v>
       </c>
-      <c r="M42" s="8"/>
-      <c r="N42" s="8"/>
-      <c r="O42" s="8"/>
-      <c r="P42" s="8"/>
+      <c r="M42" s="7"/>
+      <c r="N42" s="7"/>
+      <c r="O42" s="7"/>
+      <c r="P42" s="7"/>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
@@ -2898,41 +2904,41 @@
       <c r="C43" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D43" s="8">
+      <c r="D43" s="7">
         <v>13</v>
       </c>
-      <c r="E43" s="8">
+      <c r="E43" s="7">
         <v>42</v>
       </c>
-      <c r="F43" s="8">
-        <v>5</v>
-      </c>
-      <c r="G43" s="8">
+      <c r="F43" s="7">
+        <v>5</v>
+      </c>
+      <c r="G43" s="7">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-      <c r="H43" s="9">
+      <c r="H43" s="8">
         <f t="shared" si="1"/>
         <v>15.666666666666666</v>
       </c>
-      <c r="I43" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J43" s="10">
+      <c r="I43" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J43" s="9">
         <f t="shared" si="2"/>
         <v>24</v>
       </c>
-      <c r="K43" s="9">
+      <c r="K43" s="8">
         <f t="shared" si="3"/>
         <v>11</v>
       </c>
-      <c r="L43" s="11">
+      <c r="L43" s="10">
         <v>10</v>
       </c>
-      <c r="M43" s="8"/>
-      <c r="N43" s="8"/>
-      <c r="O43" s="8"/>
-      <c r="P43" s="8"/>
+      <c r="M43" s="7"/>
+      <c r="N43" s="7"/>
+      <c r="O43" s="7"/>
+      <c r="P43" s="7"/>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
@@ -2944,41 +2950,41 @@
       <c r="C44" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D44" s="8">
-        <v>5</v>
-      </c>
-      <c r="E44" s="8">
+      <c r="D44" s="7">
+        <v>5</v>
+      </c>
+      <c r="E44" s="7">
         <v>17</v>
       </c>
-      <c r="F44" s="8">
-        <v>5</v>
-      </c>
-      <c r="G44" s="8">
+      <c r="F44" s="7">
+        <v>5</v>
+      </c>
+      <c r="G44" s="7">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="H44" s="9">
+      <c r="H44" s="8">
         <f t="shared" si="1"/>
         <v>7.333333333333333</v>
       </c>
-      <c r="I44" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J44" s="10">
+      <c r="I44" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J44" s="9">
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="K44" s="9">
+      <c r="K44" s="8">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L44" s="11">
+      <c r="L44" s="10">
         <v>10</v>
       </c>
-      <c r="M44" s="8"/>
-      <c r="N44" s="8"/>
-      <c r="O44" s="8"/>
-      <c r="P44" s="8"/>
+      <c r="M44" s="7"/>
+      <c r="N44" s="7"/>
+      <c r="O44" s="7"/>
+      <c r="P44" s="7"/>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
@@ -2990,41 +2996,41 @@
       <c r="C45" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D45" s="8">
+      <c r="D45" s="7">
         <v>2</v>
       </c>
-      <c r="E45" s="8">
+      <c r="E45" s="7">
         <v>10</v>
       </c>
-      <c r="F45" s="8">
-        <v>5</v>
-      </c>
-      <c r="G45" s="8">
+      <c r="F45" s="7">
+        <v>5</v>
+      </c>
+      <c r="G45" s="7">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="H45" s="9">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="I45" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J45" s="10">
+      <c r="H45" s="8">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="I45" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J45" s="9">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="K45" s="9">
+      <c r="K45" s="8">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="L45" s="11">
-        <v>5</v>
-      </c>
-      <c r="M45" s="8"/>
-      <c r="N45" s="8"/>
-      <c r="O45" s="8"/>
-      <c r="P45" s="8"/>
+      <c r="L45" s="10">
+        <v>5</v>
+      </c>
+      <c r="M45" s="7"/>
+      <c r="N45" s="7"/>
+      <c r="O45" s="7"/>
+      <c r="P45" s="7"/>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
@@ -3036,41 +3042,41 @@
       <c r="C46" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D46" s="8">
+      <c r="D46" s="7">
         <v>56</v>
       </c>
-      <c r="E46" s="8">
+      <c r="E46" s="7">
         <v>143</v>
       </c>
-      <c r="F46" s="8">
-        <v>5</v>
-      </c>
-      <c r="G46" s="8">
+      <c r="F46" s="7">
+        <v>5</v>
+      </c>
+      <c r="G46" s="7">
         <f t="shared" si="0"/>
         <v>148</v>
       </c>
-      <c r="H46" s="9">
+      <c r="H46" s="8">
         <f t="shared" si="1"/>
         <v>49.333333333333336</v>
       </c>
-      <c r="I46" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J46" s="10">
+      <c r="I46" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J46" s="9">
         <f t="shared" si="2"/>
         <v>74</v>
       </c>
-      <c r="K46" s="9">
+      <c r="K46" s="8">
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="L46" s="11">
+      <c r="L46" s="10">
         <v>40</v>
       </c>
-      <c r="M46" s="8"/>
-      <c r="N46" s="8"/>
-      <c r="O46" s="8"/>
-      <c r="P46" s="8"/>
+      <c r="M46" s="7"/>
+      <c r="N46" s="7"/>
+      <c r="O46" s="7"/>
+      <c r="P46" s="7"/>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
@@ -3082,41 +3088,41 @@
       <c r="C47" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D47" s="8">
+      <c r="D47" s="7">
         <v>0</v>
       </c>
-      <c r="E47" s="8">
+      <c r="E47" s="7">
         <v>0</v>
       </c>
-      <c r="F47" s="8">
-        <v>5</v>
-      </c>
-      <c r="G47" s="8">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H47" s="9">
+      <c r="F47" s="7">
+        <v>5</v>
+      </c>
+      <c r="G47" s="7">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H47" s="8">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I47" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J47" s="10">
+      <c r="I47" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J47" s="9">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K47" s="9">
+      <c r="K47" s="8">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L47" s="11">
+      <c r="L47" s="10">
         <v>10</v>
       </c>
-      <c r="M47" s="8"/>
-      <c r="N47" s="8"/>
-      <c r="O47" s="8"/>
-      <c r="P47" s="8"/>
+      <c r="M47" s="7"/>
+      <c r="N47" s="7"/>
+      <c r="O47" s="7"/>
+      <c r="P47" s="7"/>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
@@ -3128,41 +3134,41 @@
       <c r="C48" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D48" s="8">
+      <c r="D48" s="7">
         <v>0</v>
       </c>
-      <c r="E48" s="8">
+      <c r="E48" s="7">
         <v>0</v>
       </c>
-      <c r="F48" s="8">
-        <v>5</v>
-      </c>
-      <c r="G48" s="8">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H48" s="9">
+      <c r="F48" s="7">
+        <v>5</v>
+      </c>
+      <c r="G48" s="7">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H48" s="8">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I48" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J48" s="10">
+      <c r="I48" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J48" s="9">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K48" s="9">
+      <c r="K48" s="8">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L48" s="11">
+      <c r="L48" s="10">
         <v>10</v>
       </c>
-      <c r="M48" s="8"/>
-      <c r="N48" s="8"/>
-      <c r="O48" s="8"/>
-      <c r="P48" s="8"/>
+      <c r="M48" s="7"/>
+      <c r="N48" s="7"/>
+      <c r="O48" s="7"/>
+      <c r="P48" s="7"/>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
@@ -3174,41 +3180,41 @@
       <c r="C49" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D49" s="8">
+      <c r="D49" s="7">
         <v>1</v>
       </c>
-      <c r="E49" s="8">
+      <c r="E49" s="7">
         <v>10</v>
       </c>
-      <c r="F49" s="8">
-        <v>5</v>
-      </c>
-      <c r="G49" s="8">
+      <c r="F49" s="7">
+        <v>5</v>
+      </c>
+      <c r="G49" s="7">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="H49" s="9">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="I49" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J49" s="10">
+      <c r="H49" s="8">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="I49" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J49" s="9">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="K49" s="9">
+      <c r="K49" s="8">
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="L49" s="11">
-        <v>5</v>
-      </c>
-      <c r="M49" s="8"/>
-      <c r="N49" s="8"/>
-      <c r="O49" s="8"/>
-      <c r="P49" s="8"/>
+      <c r="L49" s="10">
+        <v>5</v>
+      </c>
+      <c r="M49" s="7"/>
+      <c r="N49" s="7"/>
+      <c r="O49" s="7"/>
+      <c r="P49" s="7"/>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
@@ -3220,41 +3226,41 @@
       <c r="C50" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D50" s="8">
+      <c r="D50" s="7">
         <v>2</v>
       </c>
-      <c r="E50" s="8">
+      <c r="E50" s="7">
         <v>14</v>
       </c>
-      <c r="F50" s="8">
-        <v>5</v>
-      </c>
-      <c r="G50" s="8">
+      <c r="F50" s="7">
+        <v>5</v>
+      </c>
+      <c r="G50" s="7">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="H50" s="9">
+      <c r="H50" s="8">
         <f t="shared" si="1"/>
         <v>6.333333333333333</v>
       </c>
-      <c r="I50" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J50" s="10">
+      <c r="I50" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J50" s="9">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="K50" s="9">
+      <c r="K50" s="8">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="L50" s="11">
+      <c r="L50" s="10">
         <v>10</v>
       </c>
-      <c r="M50" s="8"/>
-      <c r="N50" s="8"/>
-      <c r="O50" s="8"/>
-      <c r="P50" s="8"/>
+      <c r="M50" s="7"/>
+      <c r="N50" s="7"/>
+      <c r="O50" s="7"/>
+      <c r="P50" s="7"/>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
@@ -3266,41 +3272,41 @@
       <c r="C51" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D51" s="8">
+      <c r="D51" s="7">
         <v>8</v>
       </c>
-      <c r="E51" s="8">
+      <c r="E51" s="7">
         <v>11</v>
       </c>
-      <c r="F51" s="8">
-        <v>5</v>
-      </c>
-      <c r="G51" s="8">
+      <c r="F51" s="7">
+        <v>5</v>
+      </c>
+      <c r="G51" s="7">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="H51" s="9">
+      <c r="H51" s="8">
         <f t="shared" si="1"/>
         <v>5.333333333333333</v>
       </c>
-      <c r="I51" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J51" s="10">
+      <c r="I51" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J51" s="9">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="K51" s="9">
+      <c r="K51" s="8">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L51" s="11">
+      <c r="L51" s="10">
         <v>10</v>
       </c>
-      <c r="M51" s="8"/>
-      <c r="N51" s="8"/>
-      <c r="O51" s="8"/>
-      <c r="P51" s="8"/>
+      <c r="M51" s="7"/>
+      <c r="N51" s="7"/>
+      <c r="O51" s="7"/>
+      <c r="P51" s="7"/>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
@@ -3312,41 +3318,41 @@
       <c r="C52" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D52" s="8">
+      <c r="D52" s="7">
         <v>0</v>
       </c>
-      <c r="E52" s="8">
+      <c r="E52" s="7">
         <v>0</v>
       </c>
-      <c r="F52" s="8">
-        <v>5</v>
-      </c>
-      <c r="G52" s="8">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H52" s="9">
+      <c r="F52" s="7">
+        <v>5</v>
+      </c>
+      <c r="G52" s="7">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H52" s="8">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I52" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J52" s="10">
+      <c r="I52" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J52" s="9">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K52" s="9">
+      <c r="K52" s="8">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L52" s="11">
-        <v>5</v>
-      </c>
-      <c r="M52" s="8"/>
-      <c r="N52" s="8"/>
-      <c r="O52" s="8"/>
-      <c r="P52" s="8"/>
+      <c r="L52" s="10">
+        <v>5</v>
+      </c>
+      <c r="M52" s="7"/>
+      <c r="N52" s="7"/>
+      <c r="O52" s="7"/>
+      <c r="P52" s="7"/>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
@@ -3358,43 +3364,43 @@
       <c r="C53" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D53" s="8">
+      <c r="D53" s="7">
         <v>2</v>
       </c>
-      <c r="E53" s="8">
+      <c r="E53" s="7">
         <v>3</v>
       </c>
-      <c r="F53" s="8">
-        <v>5</v>
-      </c>
-      <c r="G53" s="8">
+      <c r="F53" s="7">
+        <v>5</v>
+      </c>
+      <c r="G53" s="7">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="H53" s="9">
+      <c r="H53" s="8">
         <f t="shared" si="1"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="I53" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J53" s="10">
-        <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="K53" s="9">
+      <c r="I53" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J53" s="9">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="K53" s="8">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="L53" s="11">
+      <c r="L53" s="10">
         <v>10</v>
       </c>
-      <c r="M53" s="8"/>
-      <c r="N53" s="8" t="s">
+      <c r="M53" s="7"/>
+      <c r="N53" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="O53" s="8"/>
-      <c r="P53" s="8"/>
+      <c r="O53" s="7"/>
+      <c r="P53" s="7"/>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
@@ -3406,43 +3412,43 @@
       <c r="C54" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D54" s="8">
+      <c r="D54" s="7">
         <v>197</v>
       </c>
-      <c r="E54" s="8">
+      <c r="E54" s="7">
         <v>348</v>
       </c>
-      <c r="F54" s="8">
-        <v>5</v>
-      </c>
-      <c r="G54" s="8">
+      <c r="F54" s="7">
+        <v>5</v>
+      </c>
+      <c r="G54" s="7">
         <f t="shared" si="0"/>
         <v>353</v>
       </c>
-      <c r="H54" s="9">
+      <c r="H54" s="8">
         <f t="shared" si="1"/>
         <v>117.66666666666667</v>
       </c>
-      <c r="I54" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J54" s="10">
+      <c r="I54" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J54" s="9">
         <f t="shared" si="2"/>
         <v>177</v>
       </c>
-      <c r="K54" s="9">
+      <c r="K54" s="8">
         <f t="shared" si="3"/>
         <v>-20</v>
       </c>
-      <c r="L54" s="11">
+      <c r="L54" s="10">
         <v>120</v>
       </c>
-      <c r="M54" s="8" t="s">
+      <c r="M54" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="N54" s="8"/>
-      <c r="O54" s="8"/>
-      <c r="P54" s="8"/>
+      <c r="N54" s="7"/>
+      <c r="O54" s="7"/>
+      <c r="P54" s="7"/>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
@@ -3454,43 +3460,43 @@
       <c r="C55" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D55" s="8">
+      <c r="D55" s="7">
         <v>104</v>
       </c>
-      <c r="E55" s="8">
+      <c r="E55" s="7">
         <v>296</v>
       </c>
-      <c r="F55" s="8">
-        <v>5</v>
-      </c>
-      <c r="G55" s="8">
+      <c r="F55" s="7">
+        <v>5</v>
+      </c>
+      <c r="G55" s="7">
         <f t="shared" si="0"/>
         <v>301</v>
       </c>
-      <c r="H55" s="9">
+      <c r="H55" s="8">
         <f t="shared" si="1"/>
         <v>100.33333333333333</v>
       </c>
-      <c r="I55" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J55" s="10">
+      <c r="I55" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J55" s="9">
         <f t="shared" si="2"/>
         <v>151</v>
       </c>
-      <c r="K55" s="9">
+      <c r="K55" s="8">
         <f t="shared" si="3"/>
         <v>47</v>
       </c>
-      <c r="L55" s="11">
+      <c r="L55" s="10">
         <v>100</v>
       </c>
-      <c r="M55" s="8" t="s">
+      <c r="M55" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="N55" s="8"/>
-      <c r="O55" s="8"/>
-      <c r="P55" s="8"/>
+      <c r="N55" s="7"/>
+      <c r="O55" s="7"/>
+      <c r="P55" s="7"/>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
@@ -3502,41 +3508,41 @@
       <c r="C56" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D56" s="8">
+      <c r="D56" s="7">
         <v>29</v>
       </c>
-      <c r="E56" s="8">
+      <c r="E56" s="7">
         <v>61</v>
       </c>
-      <c r="F56" s="8">
-        <v>5</v>
-      </c>
-      <c r="G56" s="8">
+      <c r="F56" s="7">
+        <v>5</v>
+      </c>
+      <c r="G56" s="7">
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
-      <c r="H56" s="9">
+      <c r="H56" s="8">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="I56" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J56" s="10">
+      <c r="I56" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J56" s="9">
         <f t="shared" si="2"/>
         <v>33</v>
       </c>
-      <c r="K56" s="9">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="L56" s="11">
+      <c r="K56" s="8">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="L56" s="10">
         <v>10</v>
       </c>
-      <c r="M56" s="8"/>
-      <c r="N56" s="8"/>
-      <c r="O56" s="8"/>
-      <c r="P56" s="8"/>
+      <c r="M56" s="7"/>
+      <c r="N56" s="7"/>
+      <c r="O56" s="7"/>
+      <c r="P56" s="7"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
@@ -3548,43 +3554,43 @@
       <c r="C57" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D57" s="8">
+      <c r="D57" s="7">
         <v>6</v>
       </c>
-      <c r="E57" s="8">
+      <c r="E57" s="7">
         <v>27</v>
       </c>
-      <c r="F57" s="8">
-        <v>5</v>
-      </c>
-      <c r="G57" s="8">
+      <c r="F57" s="7">
+        <v>5</v>
+      </c>
+      <c r="G57" s="7">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="H57" s="9">
+      <c r="H57" s="8">
         <f t="shared" si="1"/>
         <v>10.666666666666666</v>
       </c>
-      <c r="I57" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J57" s="10">
+      <c r="I57" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J57" s="9">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="K57" s="9">
+      <c r="K57" s="8">
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="L57" s="11">
+      <c r="L57" s="10">
         <v>30</v>
       </c>
-      <c r="M57" s="8" t="s">
+      <c r="M57" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="N57" s="8"/>
-      <c r="O57" s="8"/>
-      <c r="P57" s="8"/>
+      <c r="N57" s="7"/>
+      <c r="O57" s="7"/>
+      <c r="P57" s="7"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
@@ -3596,41 +3602,41 @@
       <c r="C58" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D58" s="8">
+      <c r="D58" s="7">
         <v>0</v>
       </c>
-      <c r="E58" s="8">
+      <c r="E58" s="7">
         <v>0</v>
       </c>
-      <c r="F58" s="8">
-        <v>5</v>
-      </c>
-      <c r="G58" s="8">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H58" s="9">
+      <c r="F58" s="7">
+        <v>5</v>
+      </c>
+      <c r="G58" s="7">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H58" s="8">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I58" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J58" s="10">
+      <c r="I58" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J58" s="9">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K58" s="9">
+      <c r="K58" s="8">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L58" s="11">
+      <c r="L58" s="10">
         <v>10</v>
       </c>
-      <c r="M58" s="8"/>
-      <c r="N58" s="8"/>
-      <c r="O58" s="8"/>
-      <c r="P58" s="8"/>
+      <c r="M58" s="7"/>
+      <c r="N58" s="7"/>
+      <c r="O58" s="7"/>
+      <c r="P58" s="7"/>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
@@ -3642,41 +3648,41 @@
       <c r="C59" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D59" s="8">
+      <c r="D59" s="7">
         <v>0</v>
       </c>
-      <c r="E59" s="8">
+      <c r="E59" s="7">
         <v>0</v>
       </c>
-      <c r="F59" s="8">
-        <v>5</v>
-      </c>
-      <c r="G59" s="8">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H59" s="9">
+      <c r="F59" s="7">
+        <v>5</v>
+      </c>
+      <c r="G59" s="7">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H59" s="8">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I59" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J59" s="10">
+      <c r="I59" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J59" s="9">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K59" s="9">
+      <c r="K59" s="8">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L59" s="11">
+      <c r="L59" s="10">
         <v>30</v>
       </c>
-      <c r="M59" s="8"/>
-      <c r="N59" s="8"/>
-      <c r="O59" s="8"/>
-      <c r="P59" s="8"/>
+      <c r="M59" s="7"/>
+      <c r="N59" s="7"/>
+      <c r="O59" s="7"/>
+      <c r="P59" s="7"/>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
@@ -3688,41 +3694,41 @@
       <c r="C60" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D60" s="8">
+      <c r="D60" s="7">
         <v>0</v>
       </c>
-      <c r="E60" s="8">
+      <c r="E60" s="7">
         <v>0</v>
       </c>
-      <c r="F60" s="8">
-        <v>5</v>
-      </c>
-      <c r="G60" s="8">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H60" s="9">
+      <c r="F60" s="7">
+        <v>5</v>
+      </c>
+      <c r="G60" s="7">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H60" s="8">
         <f t="shared" si="1"/>
         <v>1.6666666666666667</v>
       </c>
-      <c r="I60" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J60" s="10">
+      <c r="I60" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J60" s="9">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K60" s="9">
+      <c r="K60" s="8">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L60" s="11">
+      <c r="L60" s="10">
         <v>30</v>
       </c>
-      <c r="M60" s="8"/>
-      <c r="N60" s="8"/>
-      <c r="O60" s="8"/>
-      <c r="P60" s="8"/>
+      <c r="M60" s="7"/>
+      <c r="N60" s="7"/>
+      <c r="O60" s="7"/>
+      <c r="P60" s="7"/>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
@@ -3734,43 +3740,43 @@
       <c r="C61" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D61" s="8">
+      <c r="D61" s="7">
         <v>27</v>
       </c>
-      <c r="E61" s="8">
+      <c r="E61" s="7">
         <v>74</v>
       </c>
-      <c r="F61" s="8">
-        <v>5</v>
-      </c>
-      <c r="G61" s="8">
+      <c r="F61" s="7">
+        <v>5</v>
+      </c>
+      <c r="G61" s="7">
         <f t="shared" si="0"/>
         <v>79</v>
       </c>
-      <c r="H61" s="9">
+      <c r="H61" s="8">
         <f t="shared" si="1"/>
         <v>26.333333333333332</v>
       </c>
-      <c r="I61" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J61" s="10">
+      <c r="I61" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J61" s="9">
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="K61" s="9">
+      <c r="K61" s="8">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="L61" s="11">
+      <c r="L61" s="10">
         <v>150</v>
       </c>
-      <c r="M61" s="8" t="s">
+      <c r="M61" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="N61" s="8"/>
-      <c r="O61" s="8"/>
-      <c r="P61" s="8"/>
+      <c r="N61" s="7"/>
+      <c r="O61" s="7"/>
+      <c r="P61" s="7"/>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
@@ -3782,45 +3788,46 @@
       <c r="C62" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D62" s="8">
+      <c r="D62" s="7">
         <v>2</v>
       </c>
-      <c r="E62" s="8">
+      <c r="E62" s="7">
         <v>2</v>
       </c>
-      <c r="F62" s="8">
-        <v>5</v>
-      </c>
-      <c r="G62" s="8">
+      <c r="F62" s="7">
+        <v>5</v>
+      </c>
+      <c r="G62" s="7">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="H62" s="9">
+      <c r="H62" s="8">
         <f t="shared" si="1"/>
         <v>2.3333333333333335</v>
       </c>
-      <c r="I62" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="J62" s="10">
-        <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="K62" s="9">
+      <c r="I62" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="J62" s="9">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="K62" s="8">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="L62" s="11">
+      <c r="L62" s="10">
         <v>20</v>
       </c>
-      <c r="M62" s="8" t="s">
+      <c r="M62" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="N62" s="8"/>
-      <c r="O62" s="8"/>
-      <c r="P62" s="8"/>
+      <c r="N62" s="7"/>
+      <c r="O62" s="7"/>
+      <c r="P62" s="7"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:P62" xr:uid="{96666041-4A3A-42C1-A22D-86A52389C7E2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CB replenishment update: added Open PO & In-Transit logic
</commit_message>
<xml_diff>
--- a/data/input/CB Replenishment_Master.xlsx
+++ b/data/input/CB Replenishment_Master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7ED1B49-A6D7-4797-8965-4C8E34D6B581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14013958-15C3-45E5-812D-AF5ABBDE08F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CFE25F1-D4D7-4072-B0D8-85CA58EF1A1A}"/>
   </bookViews>

</xml_diff>

<commit_message>
fix po edit override + service merge cleanup
</commit_message>
<xml_diff>
--- a/data/input/CB Replenishment_Master.xlsx
+++ b/data/input/CB Replenishment_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14013958-15C3-45E5-812D-AF5ABBDE08F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC616193-634F-41E4-8313-CE7D6E706326}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CFE25F1-D4D7-4072-B0D8-85CA58EF1A1A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="140">
   <si>
     <t>ASIN</t>
   </si>
@@ -198,9 +198,6 @@
     <t>AM-C5</t>
   </si>
   <si>
-    <t>Aggressive pricing</t>
-  </si>
-  <si>
     <t>B0FQJWWDVK</t>
   </si>
   <si>
@@ -396,9 +393,6 @@
     <t>PB-10</t>
   </si>
   <si>
-    <t>Was OOS</t>
-  </si>
-  <si>
     <t>B0FTVS34SD</t>
   </si>
   <si>
@@ -423,19 +417,10 @@
     <t>AI-13</t>
   </si>
   <si>
-    <t>DRR has increased</t>
-  </si>
-  <si>
     <t>B0GCP1J2HC</t>
   </si>
   <si>
     <t>M8</t>
-  </si>
-  <si>
-    <t>Head ASIN</t>
-  </si>
-  <si>
-    <t>Was OOS with Cambium</t>
   </si>
   <si>
     <t>3 Months CB Sales</t>
@@ -944,7 +929,7 @@
   <sheetData>
     <row r="1" spans="1:16" s="2" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
@@ -953,31 +938,31 @@
         <v>1</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="I1" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L1" s="12" t="s">
         <v>133</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="L1" s="12" t="s">
-        <v>138</v>
       </c>
       <c r="M1" s="12" t="s">
         <v>2</v>
@@ -986,10 +971,10 @@
         <v>3</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -1033,9 +1018,7 @@
       <c r="L2" s="10">
         <v>300</v>
       </c>
-      <c r="M2" s="7" t="s">
-        <v>131</v>
-      </c>
+      <c r="M2" s="7"/>
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
       <c r="P2" s="7"/>
@@ -1127,9 +1110,7 @@
       <c r="L4" s="10">
         <v>100</v>
       </c>
-      <c r="M4" s="7" t="s">
-        <v>131</v>
-      </c>
+      <c r="M4" s="7"/>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
       <c r="P4" s="7"/>
@@ -1267,9 +1248,7 @@
       <c r="L7" s="10">
         <v>120</v>
       </c>
-      <c r="M7" s="7" t="s">
-        <v>119</v>
-      </c>
+      <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
@@ -2051,9 +2030,7 @@
       <c r="L24" s="10">
         <v>30</v>
       </c>
-      <c r="M24" s="7" t="s">
-        <v>53</v>
-      </c>
+      <c r="M24" s="7"/>
       <c r="N24" s="7"/>
       <c r="O24" s="7"/>
       <c r="P24" s="7"/>
@@ -2109,10 +2086,10 @@
         <v>4</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="D26" s="7">
         <v>53</v>
@@ -2155,10 +2132,10 @@
         <v>4</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="D27" s="7">
         <v>43</v>
@@ -2201,10 +2178,10 @@
         <v>4</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="D28" s="7">
         <v>21</v>
@@ -2247,10 +2224,10 @@
         <v>4</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="D29" s="7">
         <v>27</v>
@@ -2293,10 +2270,10 @@
         <v>4</v>
       </c>
       <c r="B30" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="D30" s="7">
         <v>2</v>
@@ -2339,10 +2316,10 @@
         <v>4</v>
       </c>
       <c r="B31" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="D31" s="7">
         <v>5</v>
@@ -2375,9 +2352,7 @@
       <c r="L31" s="10">
         <v>20</v>
       </c>
-      <c r="M31" s="7" t="s">
-        <v>53</v>
-      </c>
+      <c r="M31" s="7"/>
       <c r="N31" s="7"/>
       <c r="O31" s="7"/>
       <c r="P31" s="7"/>
@@ -2387,10 +2362,10 @@
         <v>4</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="D32" s="7">
         <v>5</v>
@@ -2433,10 +2408,10 @@
         <v>4</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="D33" s="7">
         <v>45</v>
@@ -2479,10 +2454,10 @@
         <v>4</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="D34" s="7">
         <v>13</v>
@@ -2525,10 +2500,10 @@
         <v>4</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="D35" s="7">
         <v>6</v>
@@ -2561,9 +2536,7 @@
       <c r="L35" s="10">
         <v>20</v>
       </c>
-      <c r="M35" s="7" t="s">
-        <v>53</v>
-      </c>
+      <c r="M35" s="7"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
       <c r="P35" s="7"/>
@@ -2573,10 +2546,10 @@
         <v>4</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="D36" s="7">
         <v>223</v>
@@ -2609,9 +2582,7 @@
       <c r="L36" s="10">
         <v>150</v>
       </c>
-      <c r="M36" s="7" t="s">
-        <v>132</v>
-      </c>
+      <c r="M36" s="7"/>
       <c r="N36" s="7"/>
       <c r="O36" s="7"/>
       <c r="P36" s="7"/>
@@ -2621,10 +2592,10 @@
         <v>4</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D37" s="7">
         <v>0</v>
@@ -2667,10 +2638,10 @@
         <v>4</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>78</v>
       </c>
       <c r="D38" s="7">
         <v>23</v>
@@ -2703,9 +2674,7 @@
       <c r="L38" s="10">
         <v>100</v>
       </c>
-      <c r="M38" s="7" t="s">
-        <v>53</v>
-      </c>
+      <c r="M38" s="7"/>
       <c r="N38" s="7"/>
       <c r="O38" s="7"/>
       <c r="P38" s="7"/>
@@ -2715,10 +2684,10 @@
         <v>4</v>
       </c>
       <c r="B39" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="D39" s="7">
         <v>16</v>
@@ -2758,13 +2727,13 @@
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="C40" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="D40" s="7">
         <v>35</v>
@@ -2804,13 +2773,13 @@
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B41" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C41" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="D41" s="7">
         <v>14</v>
@@ -2850,13 +2819,13 @@
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B42" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>87</v>
       </c>
       <c r="D42" s="7">
         <v>40</v>
@@ -2896,13 +2865,13 @@
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B43" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="D43" s="7">
         <v>13</v>
@@ -2942,13 +2911,13 @@
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B44" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="D44" s="7">
         <v>5</v>
@@ -2988,13 +2957,13 @@
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B45" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C45" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="D45" s="7">
         <v>2</v>
@@ -3034,13 +3003,13 @@
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B46" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C46" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="D46" s="7">
         <v>56</v>
@@ -3080,13 +3049,13 @@
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B47" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="D47" s="7">
         <v>0</v>
@@ -3126,13 +3095,13 @@
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B48" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C48" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="D48" s="7">
         <v>0</v>
@@ -3175,10 +3144,10 @@
         <v>4</v>
       </c>
       <c r="B49" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="D49" s="7">
         <v>1</v>
@@ -3221,10 +3190,10 @@
         <v>4</v>
       </c>
       <c r="B50" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C50" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="D50" s="7">
         <v>2</v>
@@ -3267,10 +3236,10 @@
         <v>4</v>
       </c>
       <c r="B51" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C51" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="D51" s="7">
         <v>8</v>
@@ -3313,10 +3282,10 @@
         <v>4</v>
       </c>
       <c r="B52" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="D52" s="7">
         <v>0</v>
@@ -3359,10 +3328,10 @@
         <v>4</v>
       </c>
       <c r="B53" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="D53" s="7">
         <v>2</v>
@@ -3397,7 +3366,7 @@
       </c>
       <c r="M53" s="7"/>
       <c r="N53" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O53" s="7"/>
       <c r="P53" s="7"/>
@@ -3407,10 +3376,10 @@
         <v>4</v>
       </c>
       <c r="B54" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="D54" s="7">
         <v>197</v>
@@ -3443,9 +3412,7 @@
       <c r="L54" s="10">
         <v>120</v>
       </c>
-      <c r="M54" s="7" t="s">
-        <v>132</v>
-      </c>
+      <c r="M54" s="7"/>
       <c r="N54" s="7"/>
       <c r="O54" s="7"/>
       <c r="P54" s="7"/>
@@ -3455,10 +3422,10 @@
         <v>4</v>
       </c>
       <c r="B55" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C55" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>114</v>
       </c>
       <c r="D55" s="7">
         <v>104</v>
@@ -3491,9 +3458,7 @@
       <c r="L55" s="10">
         <v>100</v>
       </c>
-      <c r="M55" s="7" t="s">
-        <v>132</v>
-      </c>
+      <c r="M55" s="7"/>
       <c r="N55" s="7"/>
       <c r="O55" s="7"/>
       <c r="P55" s="7"/>
@@ -3503,10 +3468,10 @@
         <v>4</v>
       </c>
       <c r="B56" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C56" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="D56" s="7">
         <v>29</v>
@@ -3549,10 +3514,10 @@
         <v>4</v>
       </c>
       <c r="B57" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C57" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="D57" s="7">
         <v>6</v>
@@ -3585,9 +3550,7 @@
       <c r="L57" s="10">
         <v>30</v>
       </c>
-      <c r="M57" s="7" t="s">
-        <v>119</v>
-      </c>
+      <c r="M57" s="7"/>
       <c r="N57" s="7"/>
       <c r="O57" s="7"/>
       <c r="P57" s="7"/>
@@ -3597,10 +3560,10 @@
         <v>4</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D58" s="7">
         <v>0</v>
@@ -3643,10 +3606,10 @@
         <v>4</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D59" s="7">
         <v>0</v>
@@ -3689,10 +3652,10 @@
         <v>4</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D60" s="7">
         <v>0</v>
@@ -3735,10 +3698,10 @@
         <v>4</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D61" s="7">
         <v>27</v>
@@ -3771,9 +3734,7 @@
       <c r="L61" s="10">
         <v>150</v>
       </c>
-      <c r="M61" s="7" t="s">
-        <v>128</v>
-      </c>
+      <c r="M61" s="7"/>
       <c r="N61" s="7"/>
       <c r="O61" s="7"/>
       <c r="P61" s="7"/>
@@ -3783,10 +3744,10 @@
         <v>4</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D62" s="7">
         <v>2</v>
@@ -3819,15 +3780,12 @@
       <c r="L62" s="10">
         <v>20</v>
       </c>
-      <c r="M62" s="7" t="s">
-        <v>119</v>
-      </c>
+      <c r="M62" s="7"/>
       <c r="N62" s="7"/>
       <c r="O62" s="7"/>
       <c r="P62" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P62" xr:uid="{96666041-4A3A-42C1-A22D-86A52389C7E2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CB Master: add full bundle names (UB, PB, GB, KB, AB models)
</commit_message>
<xml_diff>
--- a/data/input/CB Replenishment_Master.xlsx
+++ b/data/input/CB Replenishment_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E83437AB-9B33-4961-AEA0-F6C5F9ED9899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCCF692-4CE0-4D46-8E52-1D87210420AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CFE25F1-D4D7-4072-B0D8-85CA58EF1A1A}"/>
   </bookViews>
@@ -321,33 +321,18 @@
     <t>B0FJ2DT13L</t>
   </si>
   <si>
-    <t>GB-02</t>
-  </si>
-  <si>
     <t>B0FJ8S5XJ8</t>
   </si>
   <si>
-    <t>PB-03</t>
-  </si>
-  <si>
     <t>B0FJ8PZ9H7</t>
   </si>
   <si>
-    <t>PB-04</t>
-  </si>
-  <si>
     <t>B0FJ8T4WXM</t>
   </si>
   <si>
-    <t>PB-05</t>
-  </si>
-  <si>
     <t>B0FN7B3KWS</t>
   </si>
   <si>
-    <t>UB-02</t>
-  </si>
-  <si>
     <t>B0FQBX8J17</t>
   </si>
   <si>
@@ -369,9 +354,6 @@
     <t>B0FTVQQVDC</t>
   </si>
   <si>
-    <t>PB-10</t>
-  </si>
-  <si>
     <t>B0FTVS34SD</t>
   </si>
   <si>
@@ -1245,60 +1227,15 @@
     <t>AM-C48</t>
   </si>
   <si>
-    <t>UB-01</t>
-  </si>
-  <si>
-    <t>KB-01</t>
-  </si>
-  <si>
-    <t>PB-01</t>
-  </si>
-  <si>
-    <t>GB-01</t>
-  </si>
-  <si>
-    <t>PB-02</t>
-  </si>
-  <si>
     <t>GB-03</t>
   </si>
   <si>
-    <t>GB-04</t>
-  </si>
-  <si>
-    <t>GB-05</t>
-  </si>
-  <si>
-    <t>PB-06</t>
-  </si>
-  <si>
-    <t>PB-07</t>
-  </si>
-  <si>
-    <t>PB-08</t>
-  </si>
-  <si>
     <t>AM-C11X Pro</t>
   </si>
   <si>
-    <t>PB-09</t>
-  </si>
-  <si>
     <t>AM-S2</t>
   </si>
   <si>
-    <t>PB-11</t>
-  </si>
-  <si>
-    <t>PB-12</t>
-  </si>
-  <si>
-    <t>PB-14</t>
-  </si>
-  <si>
-    <t>UB-03</t>
-  </si>
-  <si>
     <t>AM-W23</t>
   </si>
   <si>
@@ -2062,6 +1999,69 @@
   </si>
   <si>
     <t>FBA79983</t>
+  </si>
+  <si>
+    <t>UB-01 (AI-04, AM-S1, AA-21, AM-C2)</t>
+  </si>
+  <si>
+    <t>KB-01 (AM-W32 + AI-12)</t>
+  </si>
+  <si>
+    <t>PB-01 (AM-C11 + AI-04)</t>
+  </si>
+  <si>
+    <t>GB-01 (AM-C43 +AI-10)</t>
+  </si>
+  <si>
+    <t>GB-02 (AM-C43 + AI-11)</t>
+  </si>
+  <si>
+    <t>PB-02 (AI-04 Red + AM-C11 + AA-05)</t>
+  </si>
+  <si>
+    <t>PB-03 (AI-04 Red + AM-C11 x 2)</t>
+  </si>
+  <si>
+    <t>GB-04 (AM-C45 + AI-06)</t>
+  </si>
+  <si>
+    <t>GB-05 (AM-C43 + AI-06)</t>
+  </si>
+  <si>
+    <t>PB-04 (AI-04 Red + AM-C44 x 2)</t>
+  </si>
+  <si>
+    <t>PB-05 (AA-05 + AM-C11 + AI-04)</t>
+  </si>
+  <si>
+    <t>PB-06 (AA-05 + AM-C44 + AI-04)</t>
+  </si>
+  <si>
+    <t>PB-07 (AA-05 + AM-C45 + AI-04)</t>
+  </si>
+  <si>
+    <t>PB-08 (AM-C1 + AI-04)</t>
+  </si>
+  <si>
+    <t>UB-02 (AM-S1 + AA-21)</t>
+  </si>
+  <si>
+    <t>PB-09 (AM-C45 + AI-06 + AA-05)</t>
+  </si>
+  <si>
+    <t>PB-10 (AM-C2+AI-04+AH-60-BL)</t>
+  </si>
+  <si>
+    <t>PB-11 (AM-C44+AA-05+AH-45-BK)</t>
+  </si>
+  <si>
+    <t>PB-12 (AM-C11+AA-05+AI-04+AH-60-RD)</t>
+  </si>
+  <si>
+    <t>PB-14 (AM-C43+AH-40-SL+AI-12)</t>
+  </si>
+  <si>
+    <t>UB-03 (AM-S1 + AA-22)</t>
   </si>
 </sst>
 </file>
@@ -2529,49 +2529,49 @@
   <sheetData>
     <row r="1" spans="1:19" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>464</v>
+        <v>443</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>460</v>
+        <v>439</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>461</v>
+        <v>440</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="I1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="J1" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>128</v>
-      </c>
       <c r="N1" s="3" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="P1" s="5" t="s">
         <v>2</v>
@@ -2580,10 +2580,10 @@
         <v>3</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="S1" s="6" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2591,16 +2591,16 @@
         <v>4</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>465</v>
+        <v>444</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F2" s="9">
         <v>0</v>
@@ -2627,13 +2627,13 @@
         <v>5</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>466</v>
+        <v>445</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F3" s="9">
         <v>2010</v>
@@ -2660,13 +2660,13 @@
         <v>7</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>467</v>
+        <v>446</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>8</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F4" s="9">
         <v>0</v>
@@ -2693,13 +2693,13 @@
         <v>9</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>468</v>
+        <v>447</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F5" s="9">
         <v>0</v>
@@ -2726,13 +2726,13 @@
         <v>11</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>469</v>
+        <v>448</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F6" s="9">
         <v>0</v>
@@ -2759,13 +2759,13 @@
         <v>13</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>470</v>
+        <v>449</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>14</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F7" s="9">
         <v>0</v>
@@ -2789,16 +2789,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>471</v>
+        <v>450</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F8" s="9">
         <v>0</v>
@@ -2825,13 +2825,13 @@
         <v>15</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>472</v>
+        <v>451</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F9" s="9">
         <v>0</v>
@@ -2858,13 +2858,13 @@
         <v>17</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>473</v>
+        <v>452</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>18</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F10" s="9">
         <v>0</v>
@@ -2891,13 +2891,13 @@
         <v>19</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>474</v>
+        <v>453</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>20</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F11" s="9">
         <v>0</v>
@@ -2921,16 +2921,16 @@
         <v>4</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>475</v>
+        <v>454</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F12" s="9">
         <v>0</v>
@@ -2954,16 +2954,16 @@
         <v>4</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>476</v>
+        <v>455</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F13" s="9">
         <v>0</v>
@@ -2990,13 +2990,13 @@
         <v>21</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>477</v>
+        <v>456</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F14" s="9">
         <v>0</v>
@@ -3023,13 +3023,13 @@
         <v>23</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>478</v>
+        <v>457</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>24</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F15" s="9">
         <v>0</v>
@@ -3056,13 +3056,13 @@
         <v>25</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>479</v>
+        <v>458</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F16" s="9">
         <v>0</v>
@@ -3089,13 +3089,13 @@
         <v>27</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>480</v>
+        <v>459</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F17" s="9">
         <v>520</v>
@@ -3122,13 +3122,13 @@
         <v>29</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>481</v>
+        <v>460</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>30</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F18" s="9">
         <v>0</v>
@@ -3155,13 +3155,13 @@
         <v>31</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>482</v>
+        <v>461</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>32</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F19" s="9">
         <v>0</v>
@@ -3188,13 +3188,13 @@
         <v>33</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>483</v>
+        <v>462</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>34</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F20" s="9">
         <v>0</v>
@@ -3218,16 +3218,16 @@
         <v>4</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>484</v>
+        <v>463</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F21" s="9">
         <v>0</v>
@@ -3254,13 +3254,13 @@
         <v>35</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>485</v>
+        <v>464</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F22" s="9">
         <v>0</v>
@@ -3287,13 +3287,13 @@
         <v>37</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>486</v>
+        <v>465</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>38</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F23" s="9">
         <v>0</v>
@@ -3317,16 +3317,16 @@
         <v>4</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>487</v>
+        <v>466</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F24" s="9">
         <v>0</v>
@@ -3353,13 +3353,13 @@
         <v>39</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>488</v>
+        <v>467</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>40</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F25" s="9">
         <v>0</v>
@@ -3386,13 +3386,13 @@
         <v>41</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>489</v>
+        <v>468</v>
       </c>
       <c r="D26" s="9" t="s">
         <v>42</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F26" s="9">
         <v>0</v>
@@ -3416,16 +3416,16 @@
         <v>4</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>490</v>
+        <v>469</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F27" s="9">
         <v>0</v>
@@ -3452,13 +3452,13 @@
         <v>43</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>491</v>
+        <v>470</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F28" s="9">
         <v>0</v>
@@ -3485,13 +3485,13 @@
         <v>45</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>492</v>
+        <v>471</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>46</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F29" s="9">
         <v>0</v>
@@ -3515,16 +3515,16 @@
         <v>4</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>493</v>
+        <v>472</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F30" s="9">
         <v>0</v>
@@ -3551,13 +3551,13 @@
         <v>47</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>494</v>
+        <v>473</v>
       </c>
       <c r="D31" s="9" t="s">
         <v>48</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F31" s="9">
         <v>0</v>
@@ -3584,13 +3584,13 @@
         <v>49</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>495</v>
+        <v>474</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>50</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F32" s="9">
         <v>0</v>
@@ -3617,13 +3617,13 @@
         <v>51</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>496</v>
+        <v>475</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>52</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F33" s="9">
         <v>0</v>
@@ -3647,16 +3647,16 @@
         <v>4</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>497</v>
+        <v>476</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F34" s="9">
         <v>0</v>
@@ -3680,16 +3680,16 @@
         <v>4</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>498</v>
+        <v>477</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F35" s="9">
         <v>0</v>
@@ -3713,16 +3713,16 @@
         <v>4</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>499</v>
+        <v>478</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F36" s="9">
         <v>0</v>
@@ -3749,13 +3749,13 @@
         <v>55</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>500</v>
+        <v>479</v>
       </c>
       <c r="D37" s="9" t="s">
         <v>56</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F37" s="9">
         <v>0</v>
@@ -3779,16 +3779,16 @@
         <v>4</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>501</v>
+        <v>480</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F38" s="9">
         <v>504</v>
@@ -3812,16 +3812,16 @@
         <v>4</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>502</v>
+        <v>481</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F39" s="9">
         <v>0</v>
@@ -3845,16 +3845,16 @@
         <v>4</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>503</v>
+        <v>482</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F40" s="9">
         <v>0</v>
@@ -3878,16 +3878,16 @@
         <v>4</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>504</v>
+        <v>483</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F41" s="9">
         <v>0</v>
@@ -3914,13 +3914,13 @@
         <v>57</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>505</v>
+        <v>484</v>
       </c>
       <c r="D42" s="9" t="s">
         <v>58</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F42" s="9">
         <v>0</v>
@@ -3944,16 +3944,16 @@
         <v>4</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>506</v>
+        <v>485</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F43" s="9">
         <v>0</v>
@@ -3977,16 +3977,16 @@
         <v>4</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>507</v>
+        <v>486</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F44" s="9">
         <v>0</v>
@@ -4010,16 +4010,16 @@
         <v>4</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>508</v>
+        <v>487</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F45" s="9">
         <v>0</v>
@@ -4043,16 +4043,16 @@
         <v>4</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>509</v>
+        <v>488</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F46" s="9">
         <v>0</v>
@@ -4076,16 +4076,16 @@
         <v>4</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>510</v>
+        <v>489</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F47" s="9">
         <v>0</v>
@@ -4109,16 +4109,16 @@
         <v>4</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>511</v>
+        <v>490</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F48" s="9">
         <v>0</v>
@@ -4145,13 +4145,13 @@
         <v>59</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>512</v>
+        <v>491</v>
       </c>
       <c r="D49" s="9" t="s">
         <v>60</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F49" s="9">
         <v>0</v>
@@ -4178,13 +4178,13 @@
         <v>61</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>513</v>
+        <v>492</v>
       </c>
       <c r="D50" s="9" t="s">
         <v>62</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F50" s="9">
         <v>0</v>
@@ -4211,13 +4211,13 @@
         <v>75</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>514</v>
+        <v>493</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F51" s="9">
         <v>0</v>
@@ -4241,16 +4241,16 @@
         <v>4</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>515</v>
+        <v>494</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F52" s="9">
         <v>0</v>
@@ -4274,16 +4274,16 @@
         <v>4</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>516</v>
+        <v>495</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F53" s="9">
         <v>0</v>
@@ -4307,16 +4307,16 @@
         <v>4</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>517</v>
+        <v>496</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F54" s="9">
         <v>0</v>
@@ -4343,13 +4343,13 @@
         <v>63</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>518</v>
+        <v>497</v>
       </c>
       <c r="D55" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F55" s="9">
         <v>0</v>
@@ -4373,16 +4373,16 @@
         <v>4</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>519</v>
+        <v>498</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F56" s="9">
         <v>0</v>
@@ -4406,16 +4406,16 @@
         <v>4</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>520</v>
+        <v>499</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F57" s="9">
         <v>0</v>
@@ -4439,16 +4439,16 @@
         <v>4</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>521</v>
+        <v>500</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F58" s="9">
         <v>0</v>
@@ -4472,16 +4472,16 @@
         <v>4</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>522</v>
+        <v>501</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F59" s="9">
         <v>0</v>
@@ -4505,16 +4505,16 @@
         <v>4</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>523</v>
+        <v>502</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F60" s="9">
         <v>0</v>
@@ -4541,13 +4541,13 @@
         <v>65</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>524</v>
+        <v>503</v>
       </c>
       <c r="D61" s="9" t="s">
         <v>66</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F61" s="9">
         <v>0</v>
@@ -4571,16 +4571,16 @@
         <v>4</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>525</v>
+        <v>504</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F62" s="9">
         <v>0</v>
@@ -4604,16 +4604,16 @@
         <v>4</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>526</v>
+        <v>505</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F63" s="9">
         <v>0</v>
@@ -4640,13 +4640,13 @@
         <v>67</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>527</v>
+        <v>506</v>
       </c>
       <c r="D64" s="9" t="s">
         <v>68</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F64" s="9">
         <v>0</v>
@@ -4670,16 +4670,16 @@
         <v>4</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C65" s="9" t="s">
-        <v>528</v>
+        <v>507</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F65" s="9">
         <v>0</v>
@@ -4703,16 +4703,16 @@
         <v>4</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C66" s="9" t="s">
-        <v>529</v>
+        <v>508</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="E66" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F66" s="9">
         <v>0</v>
@@ -4736,16 +4736,16 @@
         <v>4</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="C67" s="9" t="s">
-        <v>530</v>
+        <v>509</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F67" s="9">
         <v>0</v>
@@ -4772,13 +4772,13 @@
         <v>69</v>
       </c>
       <c r="C68" s="9" t="s">
-        <v>531</v>
+        <v>510</v>
       </c>
       <c r="D68" s="9" t="s">
         <v>70</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F68" s="9">
         <v>0</v>
@@ -4802,16 +4802,16 @@
         <v>4</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C69" s="9" t="s">
-        <v>532</v>
+        <v>511</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F69" s="9">
         <v>0</v>
@@ -4835,16 +4835,16 @@
         <v>4</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C70" s="9" t="s">
-        <v>533</v>
+        <v>512</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="E70" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F70" s="9">
         <v>0</v>
@@ -4871,13 +4871,13 @@
         <v>71</v>
       </c>
       <c r="C71" s="9" t="s">
-        <v>534</v>
+        <v>513</v>
       </c>
       <c r="D71" s="9" t="s">
         <v>72</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F71" s="9">
         <v>0</v>
@@ -4901,16 +4901,16 @@
         <v>4</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C72" s="9" t="s">
-        <v>535</v>
+        <v>514</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="E72" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F72" s="9">
         <v>0</v>
@@ -4934,16 +4934,16 @@
         <v>4</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C73" s="9" t="s">
-        <v>536</v>
+        <v>515</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F73" s="9">
         <v>0</v>
@@ -4967,16 +4967,16 @@
         <v>4</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C74" s="9" t="s">
-        <v>537</v>
+        <v>516</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F74" s="9">
         <v>0</v>
@@ -5000,16 +5000,16 @@
         <v>4</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C75" s="9" t="s">
-        <v>538</v>
+        <v>517</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F75" s="9">
         <v>0</v>
@@ -5033,16 +5033,16 @@
         <v>4</v>
       </c>
       <c r="B76" s="9" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C76" s="9" t="s">
-        <v>539</v>
+        <v>518</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="E76" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F76" s="9">
         <v>0</v>
@@ -5066,16 +5066,16 @@
         <v>4</v>
       </c>
       <c r="B77" s="9" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C77" s="9" t="s">
-        <v>540</v>
+        <v>519</v>
       </c>
       <c r="D77" s="9" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F77" s="9">
         <v>0</v>
@@ -5099,16 +5099,16 @@
         <v>4</v>
       </c>
       <c r="B78" s="9" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C78" s="9" t="s">
-        <v>541</v>
+        <v>520</v>
       </c>
       <c r="D78" s="9" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="E78" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F78" s="9">
         <v>0</v>
@@ -5132,16 +5132,16 @@
         <v>4</v>
       </c>
       <c r="B79" s="9" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C79" s="9" t="s">
-        <v>542</v>
+        <v>521</v>
       </c>
       <c r="D79" s="9" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F79" s="9">
         <v>0</v>
@@ -5165,16 +5165,16 @@
         <v>4</v>
       </c>
       <c r="B80" s="9" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C80" s="9" t="s">
-        <v>543</v>
+        <v>522</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="E80" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F80" s="9">
         <v>0</v>
@@ -5198,16 +5198,16 @@
         <v>4</v>
       </c>
       <c r="B81" s="9" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C81" s="9" t="s">
-        <v>544</v>
+        <v>523</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F81" s="9">
         <v>0</v>
@@ -5231,16 +5231,16 @@
         <v>4</v>
       </c>
       <c r="B82" s="9" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C82" s="9" t="s">
-        <v>545</v>
+        <v>524</v>
       </c>
       <c r="D82" s="9" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="E82" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F82" s="9">
         <v>0</v>
@@ -5264,16 +5264,16 @@
         <v>4</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C83" s="9" t="s">
-        <v>546</v>
+        <v>525</v>
       </c>
       <c r="D83" s="9" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="E83" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F83" s="9">
         <v>0</v>
@@ -5297,16 +5297,16 @@
         <v>4</v>
       </c>
       <c r="B84" s="9" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="C84" s="9" t="s">
-        <v>547</v>
+        <v>526</v>
       </c>
       <c r="D84" s="9" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="E84" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F84" s="9">
         <v>0</v>
@@ -5330,16 +5330,16 @@
         <v>4</v>
       </c>
       <c r="B85" s="9" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C85" s="9" t="s">
-        <v>548</v>
+        <v>527</v>
       </c>
       <c r="D85" s="9" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F85" s="9">
         <v>0</v>
@@ -5363,16 +5363,16 @@
         <v>4</v>
       </c>
       <c r="B86" s="9" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C86" s="9" t="s">
-        <v>549</v>
+        <v>528</v>
       </c>
       <c r="D86" s="9" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="E86" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F86" s="9">
         <v>0</v>
@@ -5396,16 +5396,16 @@
         <v>4</v>
       </c>
       <c r="B87" s="9" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="C87" s="9" t="s">
-        <v>550</v>
+        <v>529</v>
       </c>
       <c r="D87" s="9" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="E87" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F87" s="9">
         <v>0</v>
@@ -5429,16 +5429,16 @@
         <v>4</v>
       </c>
       <c r="B88" s="9" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C88" s="9" t="s">
-        <v>551</v>
+        <v>530</v>
       </c>
       <c r="D88" s="9" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="E88" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F88" s="9">
         <v>0</v>
@@ -5462,16 +5462,16 @@
         <v>4</v>
       </c>
       <c r="B89" s="9" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="C89" s="9" t="s">
-        <v>552</v>
+        <v>531</v>
       </c>
       <c r="D89" s="9" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="E89" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F89" s="9">
         <v>0</v>
@@ -5495,16 +5495,16 @@
         <v>4</v>
       </c>
       <c r="B90" s="9" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C90" s="9" t="s">
-        <v>553</v>
+        <v>532</v>
       </c>
       <c r="D90" s="9" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="E90" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F90" s="9">
         <v>0</v>
@@ -5528,16 +5528,16 @@
         <v>4</v>
       </c>
       <c r="B91" s="9" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="C91" s="9" t="s">
-        <v>554</v>
+        <v>533</v>
       </c>
       <c r="D91" s="9" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="E91" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F91" s="9">
         <v>0</v>
@@ -5561,16 +5561,16 @@
         <v>4</v>
       </c>
       <c r="B92" s="9" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C92" s="9" t="s">
-        <v>555</v>
+        <v>534</v>
       </c>
       <c r="D92" s="9" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="E92" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F92" s="9">
         <v>0</v>
@@ -5594,16 +5594,16 @@
         <v>4</v>
       </c>
       <c r="B93" s="9" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C93" s="9" t="s">
-        <v>556</v>
+        <v>535</v>
       </c>
       <c r="D93" s="9" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="E93" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F93" s="9">
         <v>0</v>
@@ -5627,16 +5627,16 @@
         <v>4</v>
       </c>
       <c r="B94" s="9" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="C94" s="9" t="s">
-        <v>557</v>
+        <v>536</v>
       </c>
       <c r="D94" s="9" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="E94" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F94" s="9">
         <v>0</v>
@@ -5660,16 +5660,16 @@
         <v>4</v>
       </c>
       <c r="B95" s="9" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="C95" s="9" t="s">
-        <v>558</v>
+        <v>537</v>
       </c>
       <c r="D95" s="9" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="E95" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F95" s="9">
         <v>0</v>
@@ -5693,16 +5693,16 @@
         <v>4</v>
       </c>
       <c r="B96" s="9" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C96" s="9" t="s">
-        <v>559</v>
+        <v>538</v>
       </c>
       <c r="D96" s="9" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="E96" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F96" s="9">
         <v>0</v>
@@ -5726,16 +5726,16 @@
         <v>4</v>
       </c>
       <c r="B97" s="9" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C97" s="9" t="s">
-        <v>560</v>
+        <v>539</v>
       </c>
       <c r="D97" s="9" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="E97" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F97" s="9">
         <v>0</v>
@@ -5759,16 +5759,16 @@
         <v>4</v>
       </c>
       <c r="B98" s="9" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C98" s="9" t="s">
-        <v>561</v>
+        <v>540</v>
       </c>
       <c r="D98" s="9" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="E98" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F98" s="9">
         <v>0</v>
@@ -5792,16 +5792,16 @@
         <v>4</v>
       </c>
       <c r="B99" s="9" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C99" s="9" t="s">
-        <v>562</v>
+        <v>541</v>
       </c>
       <c r="D99" s="9" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="E99" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F99" s="9">
         <v>0</v>
@@ -5825,16 +5825,16 @@
         <v>4</v>
       </c>
       <c r="B100" s="9" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C100" s="9" t="s">
-        <v>563</v>
+        <v>542</v>
       </c>
       <c r="D100" s="9" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
       <c r="E100" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F100" s="9">
         <v>0</v>
@@ -5858,16 +5858,16 @@
         <v>4</v>
       </c>
       <c r="B101" s="9" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C101" s="9" t="s">
-        <v>564</v>
+        <v>543</v>
       </c>
       <c r="D101" s="9" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
       <c r="E101" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F101" s="9">
         <v>0</v>
@@ -5891,16 +5891,16 @@
         <v>4</v>
       </c>
       <c r="B102" s="9" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="C102" s="9" t="s">
-        <v>565</v>
+        <v>544</v>
       </c>
       <c r="D102" s="9" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="E102" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F102" s="9">
         <v>0</v>
@@ -5924,16 +5924,16 @@
         <v>4</v>
       </c>
       <c r="B103" s="9" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="C103" s="9" t="s">
-        <v>566</v>
+        <v>545</v>
       </c>
       <c r="D103" s="9" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
       <c r="E103" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F103" s="9">
         <v>0</v>
@@ -5957,16 +5957,16 @@
         <v>4</v>
       </c>
       <c r="B104" s="9" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="C104" s="9" t="s">
-        <v>567</v>
+        <v>546</v>
       </c>
       <c r="D104" s="9" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="E104" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F104" s="9">
         <v>0</v>
@@ -5990,16 +5990,16 @@
         <v>4</v>
       </c>
       <c r="B105" s="9" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C105" s="9" t="s">
-        <v>568</v>
+        <v>547</v>
       </c>
       <c r="D105" s="9" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
       <c r="E105" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F105" s="9">
         <v>0</v>
@@ -6023,16 +6023,16 @@
         <v>4</v>
       </c>
       <c r="B106" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="C106" s="9" t="s">
-        <v>569</v>
+        <v>548</v>
       </c>
       <c r="D106" s="9" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="E106" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F106" s="9">
         <v>0</v>
@@ -6056,16 +6056,16 @@
         <v>4</v>
       </c>
       <c r="B107" s="9" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="C107" s="9" t="s">
-        <v>570</v>
+        <v>549</v>
       </c>
       <c r="D107" s="9" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
       <c r="E107" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F107" s="9">
         <v>0</v>
@@ -6089,16 +6089,16 @@
         <v>4</v>
       </c>
       <c r="B108" s="9" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="C108" s="9" t="s">
-        <v>571</v>
+        <v>550</v>
       </c>
       <c r="D108" s="9" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="E108" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F108" s="9">
         <v>0</v>
@@ -6122,16 +6122,16 @@
         <v>4</v>
       </c>
       <c r="B109" s="9" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="C109" s="9" t="s">
-        <v>572</v>
+        <v>551</v>
       </c>
       <c r="D109" s="9" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="E109" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F109" s="9">
         <v>0</v>
@@ -6155,16 +6155,16 @@
         <v>4</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C110" s="9" t="s">
-        <v>573</v>
+        <v>552</v>
       </c>
       <c r="D110" s="9" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="E110" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F110" s="9">
         <v>0</v>
@@ -6188,16 +6188,16 @@
         <v>4</v>
       </c>
       <c r="B111" s="9" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C111" s="9" t="s">
-        <v>574</v>
+        <v>553</v>
       </c>
       <c r="D111" s="9" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
       <c r="E111" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F111" s="9">
         <v>0</v>
@@ -6221,16 +6221,16 @@
         <v>4</v>
       </c>
       <c r="B112" s="9" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C112" s="9" t="s">
-        <v>575</v>
+        <v>554</v>
       </c>
       <c r="D112" s="9" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="E112" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F112" s="9">
         <v>0</v>
@@ -6254,16 +6254,16 @@
         <v>4</v>
       </c>
       <c r="B113" s="9" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="C113" s="9" t="s">
-        <v>576</v>
+        <v>555</v>
       </c>
       <c r="D113" s="9" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="E113" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F113" s="9">
         <v>0</v>
@@ -6287,16 +6287,16 @@
         <v>4</v>
       </c>
       <c r="B114" s="9" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="C114" s="9" t="s">
-        <v>577</v>
+        <v>556</v>
       </c>
       <c r="D114" s="9" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="E114" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F114" s="9">
         <v>500</v>
@@ -6320,16 +6320,16 @@
         <v>4</v>
       </c>
       <c r="B115" s="9" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="C115" s="9" t="s">
-        <v>578</v>
+        <v>557</v>
       </c>
       <c r="D115" s="9" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
       <c r="E115" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F115" s="9">
         <v>0</v>
@@ -6353,16 +6353,16 @@
         <v>4</v>
       </c>
       <c r="B116" s="9" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="C116" s="9" t="s">
-        <v>579</v>
+        <v>558</v>
       </c>
       <c r="D116" s="9" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="E116" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F116" s="9">
         <v>0</v>
@@ -6386,16 +6386,16 @@
         <v>4</v>
       </c>
       <c r="B117" s="9" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="C117" s="9" t="s">
-        <v>580</v>
+        <v>559</v>
       </c>
       <c r="D117" s="9" t="s">
-        <v>365</v>
+        <v>359</v>
       </c>
       <c r="E117" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F117" s="9">
         <v>0</v>
@@ -6419,16 +6419,16 @@
         <v>4</v>
       </c>
       <c r="B118" s="9" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C118" s="9" t="s">
-        <v>581</v>
+        <v>560</v>
       </c>
       <c r="D118" s="9" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
       <c r="E118" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F118" s="9">
         <v>0</v>
@@ -6452,16 +6452,16 @@
         <v>4</v>
       </c>
       <c r="B119" s="9" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="C119" s="9" t="s">
-        <v>582</v>
+        <v>561</v>
       </c>
       <c r="D119" s="9" t="s">
-        <v>367</v>
+        <v>361</v>
       </c>
       <c r="E119" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F119" s="9">
         <v>0</v>
@@ -6485,16 +6485,16 @@
         <v>4</v>
       </c>
       <c r="B120" s="9" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="C120" s="9" t="s">
-        <v>583</v>
+        <v>562</v>
       </c>
       <c r="D120" s="9" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="E120" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F120" s="9">
         <v>0</v>
@@ -6518,16 +6518,16 @@
         <v>80</v>
       </c>
       <c r="B121" s="9" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="C121" s="9" t="s">
-        <v>584</v>
+        <v>563</v>
       </c>
       <c r="D121" s="9" t="s">
-        <v>369</v>
+        <v>363</v>
       </c>
       <c r="E121" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F121" s="9">
         <v>0</v>
@@ -6551,16 +6551,16 @@
         <v>80</v>
       </c>
       <c r="B122" s="9" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="C122" s="9" t="s">
-        <v>585</v>
+        <v>564</v>
       </c>
       <c r="D122" s="9" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="E122" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F122" s="9">
         <v>0</v>
@@ -6587,13 +6587,13 @@
         <v>81</v>
       </c>
       <c r="C123" s="9" t="s">
-        <v>586</v>
+        <v>565</v>
       </c>
       <c r="D123" s="9" t="s">
         <v>82</v>
       </c>
       <c r="E123" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F123" s="9">
         <v>0</v>
@@ -6617,16 +6617,16 @@
         <v>80</v>
       </c>
       <c r="B124" s="9" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C124" s="9" t="s">
-        <v>587</v>
+        <v>566</v>
       </c>
       <c r="D124" s="9" t="s">
-        <v>371</v>
+        <v>365</v>
       </c>
       <c r="E124" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F124" s="9">
         <v>0</v>
@@ -6653,13 +6653,13 @@
         <v>83</v>
       </c>
       <c r="C125" s="9" t="s">
-        <v>588</v>
+        <v>567</v>
       </c>
       <c r="D125" s="9" t="s">
         <v>84</v>
       </c>
       <c r="E125" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F125" s="9">
         <v>0</v>
@@ -6686,13 +6686,13 @@
         <v>85</v>
       </c>
       <c r="C126" s="9" t="s">
-        <v>589</v>
+        <v>568</v>
       </c>
       <c r="D126" s="9" t="s">
         <v>86</v>
       </c>
       <c r="E126" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F126" s="9">
         <v>0</v>
@@ -6716,16 +6716,16 @@
         <v>80</v>
       </c>
       <c r="B127" s="9" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="C127" s="9" t="s">
-        <v>590</v>
+        <v>569</v>
       </c>
       <c r="D127" s="9" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
       <c r="E127" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F127" s="9">
         <v>0</v>
@@ -6752,13 +6752,13 @@
         <v>87</v>
       </c>
       <c r="C128" s="9" t="s">
-        <v>591</v>
+        <v>570</v>
       </c>
       <c r="D128" s="9" t="s">
         <v>88</v>
       </c>
       <c r="E128" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F128" s="9">
         <v>0</v>
@@ -6782,16 +6782,16 @@
         <v>80</v>
       </c>
       <c r="B129" s="9" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="C129" s="9" t="s">
-        <v>592</v>
+        <v>571</v>
       </c>
       <c r="D129" s="9" t="s">
-        <v>373</v>
+        <v>367</v>
       </c>
       <c r="E129" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F129" s="9">
         <v>0</v>
@@ -6815,16 +6815,16 @@
         <v>80</v>
       </c>
       <c r="B130" s="9" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="C130" s="9" t="s">
-        <v>593</v>
+        <v>572</v>
       </c>
       <c r="D130" s="9" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
       <c r="E130" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F130" s="9">
         <v>0</v>
@@ -6848,16 +6848,16 @@
         <v>80</v>
       </c>
       <c r="B131" s="9" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="C131" s="9" t="s">
-        <v>594</v>
+        <v>573</v>
       </c>
       <c r="D131" s="9" t="s">
-        <v>375</v>
+        <v>369</v>
       </c>
       <c r="E131" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F131" s="9">
         <v>0</v>
@@ -6881,16 +6881,16 @@
         <v>80</v>
       </c>
       <c r="B132" s="9" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="C132" s="9" t="s">
-        <v>595</v>
+        <v>574</v>
       </c>
       <c r="D132" s="9" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="E132" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F132" s="9">
         <v>0</v>
@@ -6914,16 +6914,16 @@
         <v>80</v>
       </c>
       <c r="B133" s="9" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="C133" s="9" t="s">
-        <v>596</v>
+        <v>575</v>
       </c>
       <c r="D133" s="9" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="E133" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F133" s="9">
         <v>0</v>
@@ -6947,16 +6947,16 @@
         <v>80</v>
       </c>
       <c r="B134" s="9" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="C134" s="9" t="s">
-        <v>597</v>
+        <v>576</v>
       </c>
       <c r="D134" s="9" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="E134" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F134" s="9">
         <v>0</v>
@@ -6980,16 +6980,16 @@
         <v>80</v>
       </c>
       <c r="B135" s="9" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C135" s="9" t="s">
-        <v>598</v>
+        <v>577</v>
       </c>
       <c r="D135" s="9" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="E135" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F135" s="9">
         <v>0</v>
@@ -7013,16 +7013,16 @@
         <v>80</v>
       </c>
       <c r="B136" s="9" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="C136" s="9" t="s">
-        <v>599</v>
+        <v>578</v>
       </c>
       <c r="D136" s="9" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="E136" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F136" s="9">
         <v>0</v>
@@ -7046,16 +7046,16 @@
         <v>80</v>
       </c>
       <c r="B137" s="9" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C137" s="9" t="s">
-        <v>600</v>
+        <v>579</v>
       </c>
       <c r="D137" s="9" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="E137" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F137" s="9">
         <v>0</v>
@@ -7082,13 +7082,13 @@
         <v>89</v>
       </c>
       <c r="C138" s="9" t="s">
-        <v>601</v>
+        <v>580</v>
       </c>
       <c r="D138" s="9" t="s">
         <v>90</v>
       </c>
       <c r="E138" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F138" s="9">
         <v>0</v>
@@ -7112,16 +7112,16 @@
         <v>80</v>
       </c>
       <c r="B139" s="9" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="C139" s="9" t="s">
-        <v>602</v>
+        <v>581</v>
       </c>
       <c r="D139" s="9" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="E139" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F139" s="9">
         <v>0</v>
@@ -7145,16 +7145,16 @@
         <v>80</v>
       </c>
       <c r="B140" s="9" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C140" s="9" t="s">
-        <v>603</v>
+        <v>582</v>
       </c>
       <c r="D140" s="9" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="E140" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F140" s="9">
         <v>0</v>
@@ -7181,13 +7181,13 @@
         <v>91</v>
       </c>
       <c r="C141" s="9" t="s">
-        <v>604</v>
+        <v>583</v>
       </c>
       <c r="D141" s="9" t="s">
         <v>92</v>
       </c>
       <c r="E141" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F141" s="9">
         <v>0</v>
@@ -7211,16 +7211,16 @@
         <v>80</v>
       </c>
       <c r="B142" s="9" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C142" s="9" t="s">
-        <v>605</v>
+        <v>584</v>
       </c>
       <c r="D142" s="9" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="E142" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F142" s="9">
         <v>0</v>
@@ -7244,16 +7244,16 @@
         <v>80</v>
       </c>
       <c r="B143" s="9" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="C143" s="9" t="s">
-        <v>606</v>
+        <v>585</v>
       </c>
       <c r="D143" s="9" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="E143" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F143" s="9">
         <v>0</v>
@@ -7277,16 +7277,16 @@
         <v>80</v>
       </c>
       <c r="B144" s="9" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C144" s="9" t="s">
-        <v>607</v>
+        <v>586</v>
       </c>
       <c r="D144" s="9" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="E144" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F144" s="9">
         <v>0</v>
@@ -7310,16 +7310,16 @@
         <v>80</v>
       </c>
       <c r="B145" s="9" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="C145" s="9" t="s">
-        <v>608</v>
+        <v>587</v>
       </c>
       <c r="D145" s="9" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="E145" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F145" s="9">
         <v>0</v>
@@ -7343,16 +7343,16 @@
         <v>80</v>
       </c>
       <c r="B146" s="9" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C146" s="9" t="s">
-        <v>609</v>
+        <v>588</v>
       </c>
       <c r="D146" s="9" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="E146" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F146" s="9">
         <v>0</v>
@@ -7376,16 +7376,16 @@
         <v>4</v>
       </c>
       <c r="B147" s="9" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="C147" s="9" t="s">
-        <v>610</v>
+        <v>589</v>
       </c>
       <c r="D147" s="9" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="E147" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F147" s="9">
         <v>0</v>
@@ -7409,16 +7409,16 @@
         <v>4</v>
       </c>
       <c r="B148" s="9" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="C148" s="9" t="s">
-        <v>611</v>
+        <v>590</v>
       </c>
       <c r="D148" s="9" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="E148" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F148" s="9">
         <v>0</v>
@@ -7442,16 +7442,16 @@
         <v>4</v>
       </c>
       <c r="B149" s="9" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="C149" s="9" t="s">
-        <v>612</v>
+        <v>591</v>
       </c>
       <c r="D149" s="9" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="E149" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F149" s="9">
         <v>0</v>
@@ -7478,13 +7478,13 @@
         <v>76</v>
       </c>
       <c r="C150" s="9" t="s">
-        <v>613</v>
+        <v>592</v>
       </c>
       <c r="D150" s="9" t="s">
         <v>77</v>
       </c>
       <c r="E150" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F150" s="9">
         <v>0</v>
@@ -7511,13 +7511,13 @@
         <v>78</v>
       </c>
       <c r="C151" s="9" t="s">
-        <v>614</v>
+        <v>593</v>
       </c>
       <c r="D151" s="9" t="s">
         <v>79</v>
       </c>
       <c r="E151" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F151" s="9">
         <v>0</v>
@@ -7544,13 +7544,13 @@
         <v>73</v>
       </c>
       <c r="C152" s="9" t="s">
-        <v>615</v>
+        <v>594</v>
       </c>
       <c r="D152" s="9" t="s">
         <v>74</v>
       </c>
       <c r="E152" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F152" s="9">
         <v>0</v>
@@ -7574,16 +7574,16 @@
         <v>4</v>
       </c>
       <c r="B153" s="9" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="C153" s="9" t="s">
-        <v>616</v>
+        <v>595</v>
       </c>
       <c r="D153" s="9" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="E153" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F153" s="9">
         <v>0</v>
@@ -7607,16 +7607,16 @@
         <v>4</v>
       </c>
       <c r="B154" s="9" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="C154" s="9" t="s">
-        <v>616</v>
+        <v>595</v>
       </c>
       <c r="D154" s="9" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="E154" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F154" s="9">
         <v>0</v>
@@ -7640,16 +7640,16 @@
         <v>4</v>
       </c>
       <c r="B155" s="9" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="C155" s="9" t="s">
-        <v>617</v>
+        <v>596</v>
       </c>
       <c r="D155" s="9" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="E155" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F155" s="9">
         <v>0</v>
@@ -7673,16 +7673,16 @@
         <v>4</v>
       </c>
       <c r="B156" s="9" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="C156" s="9" t="s">
-        <v>618</v>
+        <v>597</v>
       </c>
       <c r="D156" s="9" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="E156" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F156" s="9">
         <v>3000</v>
@@ -7706,16 +7706,16 @@
         <v>4</v>
       </c>
       <c r="B157" s="9" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="C157" s="9" t="s">
-        <v>619</v>
+        <v>598</v>
       </c>
       <c r="D157" s="9" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="E157" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F157" s="9">
         <v>0</v>
@@ -7739,16 +7739,16 @@
         <v>4</v>
       </c>
       <c r="B158" s="9" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="C158" s="9" t="s">
-        <v>620</v>
+        <v>599</v>
       </c>
       <c r="D158" s="9" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="E158" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F158" s="9">
         <v>0</v>
@@ -7772,16 +7772,16 @@
         <v>4</v>
       </c>
       <c r="B159" s="9" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="C159" s="9" t="s">
-        <v>621</v>
+        <v>600</v>
       </c>
       <c r="D159" s="9" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="E159" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F159" s="9">
         <v>0</v>
@@ -7805,16 +7805,16 @@
         <v>4</v>
       </c>
       <c r="B160" s="9" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="C160" s="9" t="s">
-        <v>622</v>
+        <v>601</v>
       </c>
       <c r="D160" s="9" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="E160" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F160" s="9">
         <v>0</v>
@@ -7838,16 +7838,16 @@
         <v>4</v>
       </c>
       <c r="B161" s="9" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="C161" s="9" t="s">
-        <v>623</v>
+        <v>602</v>
       </c>
       <c r="D161" s="9" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="E161" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F161" s="9">
         <v>0</v>
@@ -7874,13 +7874,13 @@
         <v>53</v>
       </c>
       <c r="C162" s="9" t="s">
-        <v>624</v>
+        <v>603</v>
       </c>
       <c r="D162" s="9" t="s">
         <v>54</v>
       </c>
       <c r="E162" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F162" s="9">
         <v>0</v>
@@ -7904,16 +7904,16 @@
         <v>4</v>
       </c>
       <c r="B163" s="9" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C163" s="9" t="s">
-        <v>625</v>
+        <v>604</v>
       </c>
       <c r="D163" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E163" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F163" s="9">
         <v>0</v>
@@ -7937,16 +7937,16 @@
         <v>4</v>
       </c>
       <c r="B164" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C164" s="9" t="s">
-        <v>626</v>
+        <v>605</v>
       </c>
       <c r="D164" s="9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E164" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F164" s="9">
         <v>0</v>
@@ -7970,16 +7970,16 @@
         <v>4</v>
       </c>
       <c r="B165" s="9" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="C165" s="9" t="s">
-        <v>627</v>
+        <v>606</v>
       </c>
       <c r="D165" s="9" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="E165" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F165" s="9">
         <v>0</v>
@@ -8003,16 +8003,16 @@
         <v>4</v>
       </c>
       <c r="B166" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C166" s="9" t="s">
-        <v>628</v>
+        <v>607</v>
       </c>
       <c r="D166" s="9" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E166" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F166" s="9">
         <v>0</v>
@@ -8036,16 +8036,16 @@
         <v>4</v>
       </c>
       <c r="B167" s="9" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="C167" s="9" t="s">
-        <v>629</v>
+        <v>608</v>
       </c>
       <c r="D167" s="9" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="E167" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F167" s="9">
         <v>0</v>
@@ -8069,16 +8069,16 @@
         <v>4</v>
       </c>
       <c r="B168" s="9" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="C168" s="9" t="s">
-        <v>630</v>
+        <v>609</v>
       </c>
       <c r="D168" s="9" t="s">
-        <v>402</v>
+        <v>654</v>
       </c>
       <c r="E168" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F168" s="9">
         <v>0</v>
@@ -8102,16 +8102,16 @@
         <v>4</v>
       </c>
       <c r="B169" s="9" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="C169" s="9" t="s">
-        <v>631</v>
+        <v>610</v>
       </c>
       <c r="D169" s="9" t="s">
-        <v>403</v>
+        <v>655</v>
       </c>
       <c r="E169" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F169" s="9">
         <v>0</v>
@@ -8135,16 +8135,16 @@
         <v>4</v>
       </c>
       <c r="B170" s="9" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="C170" s="9" t="s">
-        <v>632</v>
+        <v>611</v>
       </c>
       <c r="D170" s="9" t="s">
-        <v>404</v>
+        <v>656</v>
       </c>
       <c r="E170" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F170" s="9">
         <v>0</v>
@@ -8168,16 +8168,16 @@
         <v>4</v>
       </c>
       <c r="B171" s="9" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="C171" s="9" t="s">
-        <v>633</v>
+        <v>612</v>
       </c>
       <c r="D171" s="9" t="s">
-        <v>405</v>
+        <v>657</v>
       </c>
       <c r="E171" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F171" s="9">
         <v>0</v>
@@ -8204,13 +8204,13 @@
         <v>93</v>
       </c>
       <c r="C172" s="9" t="s">
-        <v>634</v>
+        <v>613</v>
       </c>
       <c r="D172" s="9" t="s">
-        <v>94</v>
+        <v>658</v>
       </c>
       <c r="E172" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F172" s="9">
         <v>0</v>
@@ -8234,16 +8234,16 @@
         <v>4</v>
       </c>
       <c r="B173" s="9" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="C173" s="9" t="s">
-        <v>635</v>
+        <v>614</v>
       </c>
       <c r="D173" s="9" t="s">
-        <v>406</v>
+        <v>659</v>
       </c>
       <c r="E173" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F173" s="9">
         <v>0</v>
@@ -8267,16 +8267,16 @@
         <v>4</v>
       </c>
       <c r="B174" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C174" s="9" t="s">
-        <v>636</v>
+        <v>615</v>
       </c>
       <c r="D174" s="9" t="s">
-        <v>96</v>
+        <v>660</v>
       </c>
       <c r="E174" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F174" s="9">
         <v>0</v>
@@ -8300,16 +8300,16 @@
         <v>4</v>
       </c>
       <c r="B175" s="9" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C175" s="9" t="s">
-        <v>637</v>
+        <v>616</v>
       </c>
       <c r="D175" s="9" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="E175" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F175" s="9">
         <v>0</v>
@@ -8333,16 +8333,16 @@
         <v>4</v>
       </c>
       <c r="B176" s="9" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="C176" s="9" t="s">
-        <v>638</v>
+        <v>617</v>
       </c>
       <c r="D176" s="9" t="s">
-        <v>408</v>
+        <v>661</v>
       </c>
       <c r="E176" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F176" s="9">
         <v>0</v>
@@ -8366,16 +8366,16 @@
         <v>4</v>
       </c>
       <c r="B177" s="9" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="C177" s="9" t="s">
-        <v>639</v>
+        <v>618</v>
       </c>
       <c r="D177" s="9" t="s">
-        <v>409</v>
+        <v>662</v>
       </c>
       <c r="E177" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F177" s="9">
         <v>0</v>
@@ -8399,16 +8399,16 @@
         <v>4</v>
       </c>
       <c r="B178" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C178" s="9" t="s">
-        <v>640</v>
+        <v>619</v>
       </c>
       <c r="D178" s="9" t="s">
-        <v>98</v>
+        <v>663</v>
       </c>
       <c r="E178" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F178" s="9">
         <v>0</v>
@@ -8432,16 +8432,16 @@
         <v>4</v>
       </c>
       <c r="B179" s="9" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C179" s="9" t="s">
-        <v>641</v>
+        <v>620</v>
       </c>
       <c r="D179" s="9" t="s">
-        <v>100</v>
+        <v>664</v>
       </c>
       <c r="E179" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F179" s="9">
         <v>0</v>
@@ -8465,16 +8465,16 @@
         <v>4</v>
       </c>
       <c r="B180" s="9" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="C180" s="9" t="s">
-        <v>642</v>
+        <v>621</v>
       </c>
       <c r="D180" s="9" t="s">
-        <v>410</v>
+        <v>665</v>
       </c>
       <c r="E180" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F180" s="9">
         <v>0</v>
@@ -8498,16 +8498,16 @@
         <v>4</v>
       </c>
       <c r="B181" s="9" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="C181" s="9" t="s">
-        <v>643</v>
+        <v>622</v>
       </c>
       <c r="D181" s="9" t="s">
-        <v>411</v>
+        <v>666</v>
       </c>
       <c r="E181" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F181" s="9">
         <v>0</v>
@@ -8531,16 +8531,16 @@
         <v>4</v>
       </c>
       <c r="B182" s="9" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="C182" s="9" t="s">
-        <v>644</v>
+        <v>623</v>
       </c>
       <c r="D182" s="9" t="s">
-        <v>412</v>
+        <v>667</v>
       </c>
       <c r="E182" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F182" s="9">
         <v>0</v>
@@ -8564,16 +8564,16 @@
         <v>4</v>
       </c>
       <c r="B183" s="9" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C183" s="9" t="s">
-        <v>645</v>
+        <v>624</v>
       </c>
       <c r="D183" s="9" t="s">
-        <v>102</v>
+        <v>668</v>
       </c>
       <c r="E183" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F183" s="9">
         <v>0</v>
@@ -8597,16 +8597,16 @@
         <v>4</v>
       </c>
       <c r="B184" s="9" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="C184" s="9" t="s">
-        <v>646</v>
+        <v>625</v>
       </c>
       <c r="D184" s="9" t="s">
-        <v>413</v>
+        <v>397</v>
       </c>
       <c r="E184" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F184" s="9">
         <v>0</v>
@@ -8630,16 +8630,16 @@
         <v>4</v>
       </c>
       <c r="B185" s="9" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C185" s="9" t="s">
-        <v>647</v>
+        <v>626</v>
       </c>
       <c r="D185" s="9" t="s">
-        <v>414</v>
+        <v>669</v>
       </c>
       <c r="E185" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F185" s="9">
         <v>0</v>
@@ -8663,16 +8663,16 @@
         <v>4</v>
       </c>
       <c r="B186" s="9" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="C186" s="9" t="s">
-        <v>648</v>
+        <v>627</v>
       </c>
       <c r="D186" s="9" t="s">
-        <v>415</v>
+        <v>398</v>
       </c>
       <c r="E186" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F186" s="9">
         <v>700</v>
@@ -8696,16 +8696,16 @@
         <v>4</v>
       </c>
       <c r="B187" s="9" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C187" s="9" t="s">
-        <v>649</v>
+        <v>628</v>
       </c>
       <c r="D187" s="9" t="s">
-        <v>110</v>
+        <v>670</v>
       </c>
       <c r="E187" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F187" s="9">
         <v>0</v>
@@ -8729,16 +8729,16 @@
         <v>4</v>
       </c>
       <c r="B188" s="9" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="C188" s="9" t="s">
-        <v>650</v>
+        <v>629</v>
       </c>
       <c r="D188" s="9" t="s">
-        <v>416</v>
+        <v>671</v>
       </c>
       <c r="E188" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F188" s="9">
         <v>0</v>
@@ -8762,16 +8762,16 @@
         <v>4</v>
       </c>
       <c r="B189" s="9" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="C189" s="9" t="s">
-        <v>651</v>
+        <v>630</v>
       </c>
       <c r="D189" s="9" t="s">
-        <v>417</v>
+        <v>672</v>
       </c>
       <c r="E189" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F189" s="9">
         <v>0</v>
@@ -8795,16 +8795,16 @@
         <v>4</v>
       </c>
       <c r="B190" s="9" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C190" s="9" t="s">
-        <v>652</v>
+        <v>631</v>
       </c>
       <c r="D190" s="9" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="E190" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F190" s="9">
         <v>0</v>
@@ -8828,16 +8828,16 @@
         <v>4</v>
       </c>
       <c r="B191" s="9" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="C191" s="9" t="s">
-        <v>653</v>
+        <v>632</v>
       </c>
       <c r="D191" s="9" t="s">
-        <v>418</v>
+        <v>673</v>
       </c>
       <c r="E191" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F191" s="9">
         <v>0</v>
@@ -8861,16 +8861,16 @@
         <v>4</v>
       </c>
       <c r="B192" s="9" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="C192" s="9" t="s">
-        <v>654</v>
+        <v>633</v>
       </c>
       <c r="D192" s="9" t="s">
-        <v>419</v>
+        <v>674</v>
       </c>
       <c r="E192" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F192" s="9">
         <v>0</v>
@@ -8894,16 +8894,16 @@
         <v>4</v>
       </c>
       <c r="B193" s="9" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C193" s="9" t="s">
-        <v>655</v>
+        <v>634</v>
       </c>
       <c r="D193" s="9" t="s">
-        <v>420</v>
+        <v>399</v>
       </c>
       <c r="E193" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F193" s="9">
         <v>0</v>
@@ -8927,16 +8927,16 @@
         <v>4</v>
       </c>
       <c r="B194" s="9" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="C194" s="9" t="s">
-        <v>656</v>
+        <v>635</v>
       </c>
       <c r="D194" s="9" t="s">
-        <v>421</v>
+        <v>400</v>
       </c>
       <c r="E194" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F194" s="9">
         <v>0</v>
@@ -8960,16 +8960,16 @@
         <v>4</v>
       </c>
       <c r="B195" s="9" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C195" s="9" t="s">
-        <v>657</v>
+        <v>636</v>
       </c>
       <c r="D195" s="9" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="E195" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F195" s="9">
         <v>0</v>
@@ -8993,16 +8993,16 @@
         <v>4</v>
       </c>
       <c r="B196" s="9" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="C196" s="9" t="s">
-        <v>658</v>
+        <v>637</v>
       </c>
       <c r="D196" s="9" t="s">
-        <v>422</v>
+        <v>401</v>
       </c>
       <c r="E196" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F196" s="9">
         <v>0</v>
@@ -9026,16 +9026,16 @@
         <v>4</v>
       </c>
       <c r="B197" s="9" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C197" s="9" t="s">
-        <v>659</v>
+        <v>638</v>
       </c>
       <c r="D197" s="9" t="s">
-        <v>423</v>
+        <v>402</v>
       </c>
       <c r="E197" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F197" s="9">
         <v>0</v>
@@ -9059,16 +9059,16 @@
         <v>4</v>
       </c>
       <c r="B198" s="9" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="C198" s="9" t="s">
-        <v>660</v>
+        <v>639</v>
       </c>
       <c r="D198" s="9" t="s">
-        <v>424</v>
+        <v>403</v>
       </c>
       <c r="E198" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F198" s="9">
         <v>0</v>
@@ -9092,16 +9092,16 @@
         <v>4</v>
       </c>
       <c r="B199" s="9" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="C199" s="9" t="s">
-        <v>661</v>
+        <v>640</v>
       </c>
       <c r="D199" s="9" t="s">
-        <v>425</v>
+        <v>404</v>
       </c>
       <c r="E199" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F199" s="9">
         <v>60</v>
@@ -9125,16 +9125,16 @@
         <v>4</v>
       </c>
       <c r="B200" s="9" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="C200" s="9" t="s">
-        <v>662</v>
+        <v>641</v>
       </c>
       <c r="D200" s="9" t="s">
-        <v>426</v>
+        <v>405</v>
       </c>
       <c r="E200" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F200" s="9">
         <v>50</v>
@@ -9158,16 +9158,16 @@
         <v>4</v>
       </c>
       <c r="B201" s="9" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="C201" s="9" t="s">
-        <v>663</v>
+        <v>642</v>
       </c>
       <c r="D201" s="9" t="s">
-        <v>427</v>
+        <v>406</v>
       </c>
       <c r="E201" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F201" s="9">
         <v>0</v>
@@ -9191,16 +9191,16 @@
         <v>4</v>
       </c>
       <c r="B202" s="9" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C202" s="9" t="s">
-        <v>664</v>
+        <v>643</v>
       </c>
       <c r="D202" s="9" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="E202" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F202" s="9">
         <v>0</v>
@@ -9224,16 +9224,16 @@
         <v>4</v>
       </c>
       <c r="B203" s="9" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="C203" s="9" t="s">
-        <v>665</v>
+        <v>644</v>
       </c>
       <c r="D203" s="9" t="s">
-        <v>428</v>
+        <v>407</v>
       </c>
       <c r="E203" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F203" s="9">
         <v>0</v>
@@ -9258,13 +9258,13 @@
       </c>
       <c r="B204" s="9"/>
       <c r="C204" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D204" s="9" t="s">
-        <v>429</v>
+        <v>408</v>
       </c>
       <c r="E204" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F204" s="9">
         <v>0</v>
@@ -9289,13 +9289,13 @@
       </c>
       <c r="B205" s="9"/>
       <c r="C205" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D205" s="9" t="s">
-        <v>430</v>
+        <v>409</v>
       </c>
       <c r="E205" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F205" s="9">
         <v>0</v>
@@ -9319,16 +9319,16 @@
         <v>4</v>
       </c>
       <c r="B206" s="9" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="C206" s="9" t="s">
-        <v>667</v>
+        <v>646</v>
       </c>
       <c r="D206" s="9" t="s">
-        <v>431</v>
+        <v>410</v>
       </c>
       <c r="E206" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F206" s="9">
         <v>0</v>
@@ -9353,13 +9353,13 @@
       </c>
       <c r="B207" s="9"/>
       <c r="C207" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D207" s="9" t="s">
-        <v>432</v>
+        <v>411</v>
       </c>
       <c r="E207" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F207" s="9">
         <v>0</v>
@@ -9383,16 +9383,16 @@
         <v>4</v>
       </c>
       <c r="B208" s="9" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="C208" s="9" t="s">
-        <v>668</v>
+        <v>647</v>
       </c>
       <c r="D208" s="9" t="s">
-        <v>433</v>
+        <v>412</v>
       </c>
       <c r="E208" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F208" s="9">
         <v>0</v>
@@ -9416,16 +9416,16 @@
         <v>4</v>
       </c>
       <c r="B209" s="9" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="C209" s="9" t="s">
-        <v>669</v>
+        <v>648</v>
       </c>
       <c r="D209" s="9" t="s">
-        <v>434</v>
+        <v>413</v>
       </c>
       <c r="E209" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F209" s="9">
         <v>0</v>
@@ -9450,13 +9450,13 @@
       </c>
       <c r="B210" s="9"/>
       <c r="C210" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D210" s="9" t="s">
-        <v>435</v>
+        <v>414</v>
       </c>
       <c r="E210" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F210" s="9">
         <v>0</v>
@@ -9481,13 +9481,13 @@
       </c>
       <c r="B211" s="9"/>
       <c r="C211" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D211" s="9" t="s">
-        <v>436</v>
+        <v>415</v>
       </c>
       <c r="E211" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F211" s="9">
         <v>0</v>
@@ -9512,13 +9512,13 @@
       </c>
       <c r="B212" s="9"/>
       <c r="C212" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D212" s="9" t="s">
-        <v>437</v>
+        <v>416</v>
       </c>
       <c r="E212" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F212" s="9">
         <v>0</v>
@@ -9542,16 +9542,16 @@
         <v>4</v>
       </c>
       <c r="B213" s="9" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="C213" s="9" t="s">
-        <v>670</v>
+        <v>649</v>
       </c>
       <c r="D213" s="9" t="s">
-        <v>438</v>
+        <v>417</v>
       </c>
       <c r="E213" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F213" s="9">
         <v>0</v>
@@ -9575,16 +9575,16 @@
         <v>4</v>
       </c>
       <c r="B214" s="9" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="C214" s="9" t="s">
-        <v>671</v>
+        <v>650</v>
       </c>
       <c r="D214" s="9" t="s">
-        <v>439</v>
+        <v>418</v>
       </c>
       <c r="E214" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F214" s="9">
         <v>0</v>
@@ -9608,16 +9608,16 @@
         <v>4</v>
       </c>
       <c r="B215" s="9" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C215" s="9" t="s">
-        <v>672</v>
+        <v>651</v>
       </c>
       <c r="D215" s="9" t="s">
-        <v>440</v>
+        <v>419</v>
       </c>
       <c r="E215" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F215" s="9">
         <v>0</v>
@@ -9641,16 +9641,16 @@
         <v>4</v>
       </c>
       <c r="B216" s="9" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="C216" s="9" t="s">
-        <v>673</v>
+        <v>652</v>
       </c>
       <c r="D216" s="9" t="s">
-        <v>441</v>
+        <v>420</v>
       </c>
       <c r="E216" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F216" s="9">
         <v>0</v>
@@ -9674,16 +9674,16 @@
         <v>4</v>
       </c>
       <c r="B217" s="9" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="C217" s="9" t="s">
-        <v>674</v>
+        <v>653</v>
       </c>
       <c r="D217" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="E217" s="9" t="s">
         <v>442</v>
-      </c>
-      <c r="E217" s="9" t="s">
-        <v>463</v>
       </c>
       <c r="F217" s="9">
         <v>0</v>
@@ -9708,13 +9708,13 @@
       </c>
       <c r="B218" s="9"/>
       <c r="C218" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D218" s="9" t="s">
-        <v>443</v>
+        <v>422</v>
       </c>
       <c r="E218" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F218" s="9">
         <v>0</v>
@@ -9739,13 +9739,13 @@
       </c>
       <c r="B219" s="9"/>
       <c r="C219" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D219" s="9" t="s">
-        <v>444</v>
+        <v>423</v>
       </c>
       <c r="E219" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F219" s="9">
         <v>0</v>
@@ -9770,13 +9770,13 @@
       </c>
       <c r="B220" s="9"/>
       <c r="C220" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D220" s="9" t="s">
-        <v>445</v>
+        <v>424</v>
       </c>
       <c r="E220" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F220" s="9">
         <v>0</v>
@@ -9801,13 +9801,13 @@
       </c>
       <c r="B221" s="9"/>
       <c r="C221" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D221" s="9" t="s">
-        <v>446</v>
+        <v>425</v>
       </c>
       <c r="E221" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F221" s="9">
         <v>0</v>
@@ -9832,13 +9832,13 @@
       </c>
       <c r="B222" s="9"/>
       <c r="C222" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D222" s="9" t="s">
-        <v>447</v>
+        <v>426</v>
       </c>
       <c r="E222" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F222" s="9">
         <v>0</v>
@@ -9863,13 +9863,13 @@
       </c>
       <c r="B223" s="9"/>
       <c r="C223" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D223" s="9" t="s">
-        <v>448</v>
+        <v>427</v>
       </c>
       <c r="E223" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F223" s="9">
         <v>0</v>
@@ -9894,13 +9894,13 @@
       </c>
       <c r="B224" s="9"/>
       <c r="C224" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D224" s="9" t="s">
-        <v>449</v>
+        <v>428</v>
       </c>
       <c r="E224" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F224" s="9">
         <v>0</v>
@@ -9925,13 +9925,13 @@
       </c>
       <c r="B225" s="9"/>
       <c r="C225" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D225" s="9" t="s">
-        <v>450</v>
+        <v>429</v>
       </c>
       <c r="E225" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F225" s="9">
         <v>0</v>
@@ -9956,13 +9956,13 @@
       </c>
       <c r="B226" s="9"/>
       <c r="C226" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D226" s="9" t="s">
-        <v>451</v>
+        <v>430</v>
       </c>
       <c r="E226" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F226" s="9">
         <v>0</v>
@@ -9987,13 +9987,13 @@
       </c>
       <c r="B227" s="9"/>
       <c r="C227" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D227" s="9" t="s">
-        <v>452</v>
+        <v>431</v>
       </c>
       <c r="E227" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F227" s="9">
         <v>0</v>
@@ -10018,13 +10018,13 @@
       </c>
       <c r="B228" s="9"/>
       <c r="C228" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D228" s="9" t="s">
-        <v>453</v>
+        <v>432</v>
       </c>
       <c r="E228" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F228" s="9">
         <v>0</v>
@@ -10049,13 +10049,13 @@
       </c>
       <c r="B229" s="9"/>
       <c r="C229" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D229" s="9" t="s">
-        <v>454</v>
+        <v>433</v>
       </c>
       <c r="E229" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F229" s="9">
         <v>0</v>
@@ -10080,13 +10080,13 @@
       </c>
       <c r="B230" s="9"/>
       <c r="C230" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D230" s="9" t="s">
-        <v>455</v>
+        <v>434</v>
       </c>
       <c r="E230" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="F230" s="9">
         <v>0</v>
@@ -10111,13 +10111,13 @@
       </c>
       <c r="B231" s="9"/>
       <c r="C231" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D231" s="9" t="s">
-        <v>456</v>
+        <v>435</v>
       </c>
       <c r="E231" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F231" s="9">
         <v>10</v>
@@ -10142,13 +10142,13 @@
       </c>
       <c r="B232" s="9"/>
       <c r="C232" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D232" s="9" t="s">
-        <v>457</v>
+        <v>436</v>
       </c>
       <c r="E232" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F232" s="9">
         <v>10</v>
@@ -10173,13 +10173,13 @@
       </c>
       <c r="B233" s="9"/>
       <c r="C233" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D233" s="9" t="s">
-        <v>458</v>
+        <v>437</v>
       </c>
       <c r="E233" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F233" s="9">
         <v>10</v>
@@ -10204,13 +10204,13 @@
       </c>
       <c r="B234" s="9"/>
       <c r="C234" s="9" t="s">
-        <v>666</v>
+        <v>645</v>
       </c>
       <c r="D234" s="9" t="s">
-        <v>459</v>
+        <v>438</v>
       </c>
       <c r="E234" s="9" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="F234" s="9">
         <v>10</v>
@@ -10230,6 +10230,7 @@
       <c r="S234" s="9"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:S234" xr:uid="{96666041-4A3A-42C1-A22D-86A52389C7E2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update replenishment files, CB master, fossil inventory ledger, and PO item export
</commit_message>
<xml_diff>
--- a/data/input/CB Replenishment_Master.xlsx
+++ b/data/input/CB Replenishment_Master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCCF692-4CE0-4D46-8E52-1D87210420AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA597A48-1660-41F8-BFF4-2F80776B551D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CFE25F1-D4D7-4072-B0D8-85CA58EF1A1A}"/>
   </bookViews>

</xml_diff>

<commit_message>
Update CB replenishment master and WM transit PO data
</commit_message>
<xml_diff>
--- a/data/input/CB Replenishment_Master.xlsx
+++ b/data/input/CB Replenishment_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA597A48-1660-41F8-BFF4-2F80776B551D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AADEB525-826B-4C31-9485-D2C6B7D57FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CFE25F1-D4D7-4072-B0D8-85CA58EF1A1A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$S$234</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$S$238</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1161" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1202" uniqueCount="731">
   <si>
     <t>ASIN</t>
   </si>
@@ -2062,6 +2062,174 @@
   </si>
   <si>
     <t>UB-03 (AM-S1 + AA-22)</t>
+  </si>
+  <si>
+    <t>B0CQX4K9P5</t>
+  </si>
+  <si>
+    <t>FBA79697</t>
+  </si>
+  <si>
+    <t>TD310</t>
+  </si>
+  <si>
+    <t>B0CQX3VB1R</t>
+  </si>
+  <si>
+    <t>FBA79696</t>
+  </si>
+  <si>
+    <t>TD310+</t>
+  </si>
+  <si>
+    <t>B08V1JS3NY</t>
+  </si>
+  <si>
+    <t>FBA77115</t>
+  </si>
+  <si>
+    <t>TC40</t>
+  </si>
+  <si>
+    <t>B0BBL47VR5</t>
+  </si>
+  <si>
+    <t>FBA77116</t>
+  </si>
+  <si>
+    <t>TC40 RGB</t>
+  </si>
+  <si>
+    <t>B0GXP97CZG</t>
+  </si>
+  <si>
+    <t>B0GXPBHDRF</t>
+  </si>
+  <si>
+    <t>FBA80085</t>
+  </si>
+  <si>
+    <t>B0GXP7LJ75</t>
+  </si>
+  <si>
+    <t>FBA79975</t>
+  </si>
+  <si>
+    <t>B0GV15BVQC</t>
+  </si>
+  <si>
+    <t>FBA79976</t>
+  </si>
+  <si>
+    <t>B0GV154XPQ</t>
+  </si>
+  <si>
+    <t>FBA79977</t>
+  </si>
+  <si>
+    <t>B0GW8Z556N</t>
+  </si>
+  <si>
+    <t>FBA79996</t>
+  </si>
+  <si>
+    <t>B0GW8VBCBL</t>
+  </si>
+  <si>
+    <t>FBA79995</t>
+  </si>
+  <si>
+    <t>B0GW9461N5</t>
+  </si>
+  <si>
+    <t>FBA79997</t>
+  </si>
+  <si>
+    <t>B0GW8YC59C</t>
+  </si>
+  <si>
+    <t>FBA79998</t>
+  </si>
+  <si>
+    <t>B0GW92TVVC</t>
+  </si>
+  <si>
+    <t>FBA79999</t>
+  </si>
+  <si>
+    <t>B0GW8XGPB2</t>
+  </si>
+  <si>
+    <t>FBA80000</t>
+  </si>
+  <si>
+    <t>B0GW92TQGV</t>
+  </si>
+  <si>
+    <t>FBA80001</t>
+  </si>
+  <si>
+    <t>B0GW96SHSK</t>
+  </si>
+  <si>
+    <t>FBA80002</t>
+  </si>
+  <si>
+    <t>B0GW92TTMS</t>
+  </si>
+  <si>
+    <t>FBA80003</t>
+  </si>
+  <si>
+    <t>B0GW92316G</t>
+  </si>
+  <si>
+    <t>FBA80004</t>
+  </si>
+  <si>
+    <t>B0GW96CQMG</t>
+  </si>
+  <si>
+    <t>FBA80005</t>
+  </si>
+  <si>
+    <t>B0GW8R2RYM</t>
+  </si>
+  <si>
+    <t>FBA80009</t>
+  </si>
+  <si>
+    <t>B0GW8ZQRFK</t>
+  </si>
+  <si>
+    <t>FBA80010</t>
+  </si>
+  <si>
+    <t>B0GTZND3ZN</t>
+  </si>
+  <si>
+    <t>FBA80011</t>
+  </si>
+  <si>
+    <t>B0GTZJF142</t>
+  </si>
+  <si>
+    <t>FBA80012</t>
+  </si>
+  <si>
+    <t>B0GTZLGPFR</t>
+  </si>
+  <si>
+    <t>FBA80013</t>
+  </si>
+  <si>
+    <t>B0GTZ9X8Q2</t>
+  </si>
+  <si>
+    <t>FBA80014</t>
+  </si>
+  <si>
+    <t>FBA79708</t>
   </si>
 </sst>
 </file>
@@ -2507,7 +2675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96666041-4A3A-42C1-A22D-86A52389C7E2}">
-  <dimension ref="A1:S234"/>
+  <dimension ref="A1:S238"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
@@ -7577,7 +7745,7 @@
         <v>232</v>
       </c>
       <c r="C153" s="9" t="s">
-        <v>595</v>
+        <v>730</v>
       </c>
       <c r="D153" s="9" t="s">
         <v>386</v>
@@ -9256,7 +9424,9 @@
       <c r="A204" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B204" s="9"/>
+      <c r="B204" s="9" t="s">
+        <v>687</v>
+      </c>
       <c r="C204" s="9" t="s">
         <v>645</v>
       </c>
@@ -9287,9 +9457,11 @@
       <c r="A205" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B205" s="9"/>
+      <c r="B205" s="9" t="s">
+        <v>688</v>
+      </c>
       <c r="C205" s="9" t="s">
-        <v>645</v>
+        <v>689</v>
       </c>
       <c r="D205" s="9" t="s">
         <v>409</v>
@@ -9352,9 +9524,7 @@
         <v>4</v>
       </c>
       <c r="B207" s="9"/>
-      <c r="C207" s="9" t="s">
-        <v>645</v>
-      </c>
+      <c r="C207" s="9"/>
       <c r="D207" s="9" t="s">
         <v>411</v>
       </c>
@@ -9448,9 +9618,11 @@
       <c r="A210" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B210" s="9"/>
+      <c r="B210" s="9" t="s">
+        <v>690</v>
+      </c>
       <c r="C210" s="9" t="s">
-        <v>645</v>
+        <v>691</v>
       </c>
       <c r="D210" s="9" t="s">
         <v>414</v>
@@ -9479,9 +9651,11 @@
       <c r="A211" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B211" s="9"/>
+      <c r="B211" s="9" t="s">
+        <v>692</v>
+      </c>
       <c r="C211" s="9" t="s">
-        <v>645</v>
+        <v>693</v>
       </c>
       <c r="D211" s="9" t="s">
         <v>415</v>
@@ -9510,9 +9684,11 @@
       <c r="A212" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B212" s="9"/>
+      <c r="B212" s="9" t="s">
+        <v>694</v>
+      </c>
       <c r="C212" s="9" t="s">
-        <v>645</v>
+        <v>695</v>
       </c>
       <c r="D212" s="9" t="s">
         <v>416</v>
@@ -9706,9 +9882,11 @@
       <c r="A218" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B218" s="9"/>
+      <c r="B218" s="9" t="s">
+        <v>696</v>
+      </c>
       <c r="C218" s="9" t="s">
-        <v>645</v>
+        <v>697</v>
       </c>
       <c r="D218" s="9" t="s">
         <v>422</v>
@@ -9737,9 +9915,11 @@
       <c r="A219" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B219" s="9"/>
+      <c r="B219" s="9" t="s">
+        <v>698</v>
+      </c>
       <c r="C219" s="9" t="s">
-        <v>645</v>
+        <v>699</v>
       </c>
       <c r="D219" s="9" t="s">
         <v>423</v>
@@ -9768,9 +9948,11 @@
       <c r="A220" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B220" s="9"/>
+      <c r="B220" s="9" t="s">
+        <v>700</v>
+      </c>
       <c r="C220" s="9" t="s">
-        <v>645</v>
+        <v>701</v>
       </c>
       <c r="D220" s="9" t="s">
         <v>424</v>
@@ -9799,9 +9981,11 @@
       <c r="A221" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B221" s="9"/>
+      <c r="B221" s="9" t="s">
+        <v>702</v>
+      </c>
       <c r="C221" s="9" t="s">
-        <v>645</v>
+        <v>703</v>
       </c>
       <c r="D221" s="9" t="s">
         <v>425</v>
@@ -9830,9 +10014,11 @@
       <c r="A222" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B222" s="9"/>
+      <c r="B222" s="9" t="s">
+        <v>704</v>
+      </c>
       <c r="C222" s="9" t="s">
-        <v>645</v>
+        <v>705</v>
       </c>
       <c r="D222" s="9" t="s">
         <v>426</v>
@@ -9861,9 +10047,11 @@
       <c r="A223" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B223" s="9"/>
+      <c r="B223" s="9" t="s">
+        <v>706</v>
+      </c>
       <c r="C223" s="9" t="s">
-        <v>645</v>
+        <v>707</v>
       </c>
       <c r="D223" s="9" t="s">
         <v>427</v>
@@ -9892,9 +10080,11 @@
       <c r="A224" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B224" s="9"/>
+      <c r="B224" s="9" t="s">
+        <v>708</v>
+      </c>
       <c r="C224" s="9" t="s">
-        <v>645</v>
+        <v>709</v>
       </c>
       <c r="D224" s="9" t="s">
         <v>428</v>
@@ -9923,9 +10113,11 @@
       <c r="A225" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B225" s="9"/>
+      <c r="B225" s="9" t="s">
+        <v>710</v>
+      </c>
       <c r="C225" s="9" t="s">
-        <v>645</v>
+        <v>711</v>
       </c>
       <c r="D225" s="9" t="s">
         <v>429</v>
@@ -9954,9 +10146,11 @@
       <c r="A226" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B226" s="9"/>
+      <c r="B226" s="9" t="s">
+        <v>712</v>
+      </c>
       <c r="C226" s="9" t="s">
-        <v>645</v>
+        <v>713</v>
       </c>
       <c r="D226" s="9" t="s">
         <v>430</v>
@@ -9985,9 +10179,11 @@
       <c r="A227" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B227" s="9"/>
+      <c r="B227" s="9" t="s">
+        <v>714</v>
+      </c>
       <c r="C227" s="9" t="s">
-        <v>645</v>
+        <v>715</v>
       </c>
       <c r="D227" s="9" t="s">
         <v>431</v>
@@ -10016,9 +10212,11 @@
       <c r="A228" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B228" s="9"/>
+      <c r="B228" s="9" t="s">
+        <v>716</v>
+      </c>
       <c r="C228" s="9" t="s">
-        <v>645</v>
+        <v>717</v>
       </c>
       <c r="D228" s="9" t="s">
         <v>432</v>
@@ -10047,9 +10245,11 @@
       <c r="A229" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B229" s="9"/>
+      <c r="B229" s="9" t="s">
+        <v>718</v>
+      </c>
       <c r="C229" s="9" t="s">
-        <v>645</v>
+        <v>719</v>
       </c>
       <c r="D229" s="9" t="s">
         <v>433</v>
@@ -10078,9 +10278,11 @@
       <c r="A230" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B230" s="9"/>
+      <c r="B230" s="9" t="s">
+        <v>720</v>
+      </c>
       <c r="C230" s="9" t="s">
-        <v>645</v>
+        <v>721</v>
       </c>
       <c r="D230" s="9" t="s">
         <v>434</v>
@@ -10109,9 +10311,11 @@
       <c r="A231" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B231" s="9"/>
+      <c r="B231" s="9" t="s">
+        <v>722</v>
+      </c>
       <c r="C231" s="9" t="s">
-        <v>645</v>
+        <v>723</v>
       </c>
       <c r="D231" s="9" t="s">
         <v>435</v>
@@ -10140,9 +10344,11 @@
       <c r="A232" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B232" s="9"/>
+      <c r="B232" s="9" t="s">
+        <v>724</v>
+      </c>
       <c r="C232" s="9" t="s">
-        <v>645</v>
+        <v>725</v>
       </c>
       <c r="D232" s="9" t="s">
         <v>436</v>
@@ -10171,9 +10377,11 @@
       <c r="A233" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B233" s="9"/>
+      <c r="B233" s="9" t="s">
+        <v>726</v>
+      </c>
       <c r="C233" s="9" t="s">
-        <v>645</v>
+        <v>727</v>
       </c>
       <c r="D233" s="9" t="s">
         <v>437</v>
@@ -10202,9 +10410,11 @@
       <c r="A234" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B234" s="9"/>
+      <c r="B234" s="9" t="s">
+        <v>728</v>
+      </c>
       <c r="C234" s="9" t="s">
-        <v>645</v>
+        <v>729</v>
       </c>
       <c r="D234" s="9" t="s">
         <v>438</v>
@@ -10229,8 +10439,76 @@
       <c r="R234" s="9"/>
       <c r="S234" s="9"/>
     </row>
+    <row r="235" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A235" t="s">
+        <v>80</v>
+      </c>
+      <c r="B235" t="s">
+        <v>675</v>
+      </c>
+      <c r="C235" t="s">
+        <v>676</v>
+      </c>
+      <c r="D235" t="s">
+        <v>677</v>
+      </c>
+      <c r="E235" s="9" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="236" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A236" t="s">
+        <v>80</v>
+      </c>
+      <c r="B236" t="s">
+        <v>678</v>
+      </c>
+      <c r="C236" t="s">
+        <v>679</v>
+      </c>
+      <c r="D236" t="s">
+        <v>680</v>
+      </c>
+      <c r="E236" s="9" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="237" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A237" t="s">
+        <v>80</v>
+      </c>
+      <c r="B237" t="s">
+        <v>681</v>
+      </c>
+      <c r="C237" t="s">
+        <v>682</v>
+      </c>
+      <c r="D237" t="s">
+        <v>683</v>
+      </c>
+      <c r="E237" s="9" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="238" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A238" t="s">
+        <v>80</v>
+      </c>
+      <c r="B238" t="s">
+        <v>684</v>
+      </c>
+      <c r="C238" t="s">
+        <v>685</v>
+      </c>
+      <c r="D238" t="s">
+        <v>686</v>
+      </c>
+      <c r="E238" s="9" t="s">
+        <v>442</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S234" xr:uid="{96666041-4A3A-42C1-A22D-86A52389C7E2}"/>
+  <autoFilter ref="A1:S238" xr:uid="{96666041-4A3A-42C1-A22D-86A52389C7E2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CB master: add TC40S (Tonor) and AM-Mix8 (Audio Array) so their sales flow through
</commit_message>
<xml_diff>
--- a/data/input/CB Replenishment_Master.xlsx
+++ b/data/input/CB Replenishment_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D56FA9-2749-42E5-BCE5-0291E20EEC1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3FA2CB-1D14-477B-A3B6-F76747E2EA9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CFE25F1-D4D7-4072-B0D8-85CA58EF1A1A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1202" uniqueCount="731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="733">
   <si>
     <t>ASIN</t>
   </si>
@@ -1068,9 +1068,6 @@
     <t xml:space="preserve">AM-C15 </t>
   </si>
   <si>
-    <t>AI-04	Black</t>
-  </si>
-  <si>
     <t xml:space="preserve">AM-C12 </t>
   </si>
   <si>
@@ -2230,6 +2227,15 @@
   </si>
   <si>
     <t>FBA79708</t>
+  </si>
+  <si>
+    <t>AI-04 Black</t>
+  </si>
+  <si>
+    <t>TC40S</t>
+  </si>
+  <si>
+    <t>AM-Mix8</t>
   </si>
 </sst>
 </file>
@@ -2302,7 +2308,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -2325,11 +2331,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2356,6 +2373,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2672,7 +2692,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96666041-4A3A-42C1-A22D-86A52389C7E2}">
-  <dimension ref="A1:S238"/>
+  <dimension ref="A1:S240"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
@@ -2700,16 +2720,16 @@
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>439</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>440</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>115</v>
@@ -2759,13 +2779,13 @@
         <v>125</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>277</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
@@ -2790,13 +2810,13 @@
         <v>5</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
@@ -2821,13 +2841,13 @@
         <v>7</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>8</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
@@ -2852,13 +2872,13 @@
         <v>9</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
@@ -2883,13 +2903,13 @@
         <v>11</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
@@ -2914,13 +2934,13 @@
         <v>13</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
@@ -2945,13 +2965,13 @@
         <v>126</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>278</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
@@ -2976,13 +2996,13 @@
         <v>15</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
@@ -3007,13 +3027,13 @@
         <v>17</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>18</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
@@ -3038,13 +3058,13 @@
         <v>19</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>20</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
@@ -3069,13 +3089,13 @@
         <v>127</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>279</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
@@ -3100,13 +3120,13 @@
         <v>128</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>280</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
@@ -3131,13 +3151,13 @@
         <v>21</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>22</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
@@ -3162,13 +3182,13 @@
         <v>23</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>24</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
@@ -3193,13 +3213,13 @@
         <v>25</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>26</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
@@ -3224,13 +3244,13 @@
         <v>27</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F17" s="8"/>
       <c r="G17" s="8"/>
@@ -3255,13 +3275,13 @@
         <v>29</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>30</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
@@ -3286,13 +3306,13 @@
         <v>31</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
@@ -3317,13 +3337,13 @@
         <v>33</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>34</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
@@ -3348,13 +3368,13 @@
         <v>129</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>281</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
@@ -3379,13 +3399,13 @@
         <v>35</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>36</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
@@ -3410,13 +3430,13 @@
         <v>37</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>38</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
@@ -3441,13 +3461,13 @@
         <v>130</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>282</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F24" s="8"/>
       <c r="G24" s="8"/>
@@ -3472,13 +3492,13 @@
         <v>39</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>40</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
@@ -3503,13 +3523,13 @@
         <v>41</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>42</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
@@ -3534,13 +3554,13 @@
         <v>131</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>283</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
@@ -3565,13 +3585,13 @@
         <v>43</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>44</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F28" s="8"/>
       <c r="G28" s="8"/>
@@ -3596,13 +3616,13 @@
         <v>45</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>46</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F29" s="8"/>
       <c r="G29" s="8"/>
@@ -3627,13 +3647,13 @@
         <v>132</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D30" s="8" t="s">
         <v>284</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F30" s="8"/>
       <c r="G30" s="8"/>
@@ -3658,13 +3678,13 @@
         <v>47</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="D31" s="8" t="s">
         <v>48</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F31" s="8"/>
       <c r="G31" s="8"/>
@@ -3689,13 +3709,13 @@
         <v>49</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D32" s="8" t="s">
         <v>50</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F32" s="8"/>
       <c r="G32" s="8"/>
@@ -3720,13 +3740,13 @@
         <v>51</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>52</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F33" s="8"/>
       <c r="G33" s="8"/>
@@ -3751,13 +3771,13 @@
         <v>133</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D34" s="8" t="s">
         <v>285</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F34" s="8"/>
       <c r="G34" s="8"/>
@@ -3782,13 +3802,13 @@
         <v>134</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="D35" s="8" t="s">
         <v>286</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F35" s="8"/>
       <c r="G35" s="8"/>
@@ -3813,13 +3833,13 @@
         <v>135</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D36" s="8" t="s">
         <v>287</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F36" s="8"/>
       <c r="G36" s="8"/>
@@ -3844,13 +3864,13 @@
         <v>55</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="D37" s="8" t="s">
         <v>56</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F37" s="8"/>
       <c r="G37" s="8"/>
@@ -3875,13 +3895,13 @@
         <v>136</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="D38" s="8" t="s">
         <v>288</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F38" s="8"/>
       <c r="G38" s="8"/>
@@ -3906,13 +3926,13 @@
         <v>137</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="D39" s="8" t="s">
         <v>289</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F39" s="8"/>
       <c r="G39" s="8"/>
@@ -3937,13 +3957,13 @@
         <v>138</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="D40" s="8" t="s">
         <v>290</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F40" s="8"/>
       <c r="G40" s="8"/>
@@ -3968,13 +3988,13 @@
         <v>139</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="D41" s="8" t="s">
         <v>291</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F41" s="8"/>
       <c r="G41" s="8"/>
@@ -3999,13 +4019,13 @@
         <v>57</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="D42" s="8" t="s">
         <v>58</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F42" s="8"/>
       <c r="G42" s="8"/>
@@ -4030,13 +4050,13 @@
         <v>140</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="D43" s="8" t="s">
         <v>292</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F43" s="8"/>
       <c r="G43" s="8"/>
@@ -4061,13 +4081,13 @@
         <v>141</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D44" s="8" t="s">
         <v>293</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>
@@ -4092,13 +4112,13 @@
         <v>142</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="D45" s="8" t="s">
         <v>294</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
@@ -4123,13 +4143,13 @@
         <v>143</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D46" s="8" t="s">
         <v>295</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F46" s="8"/>
       <c r="G46" s="8"/>
@@ -4154,13 +4174,13 @@
         <v>144</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D47" s="8" t="s">
         <v>296</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
@@ -4185,13 +4205,13 @@
         <v>145</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D48" s="8" t="s">
         <v>297</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F48" s="8"/>
       <c r="G48" s="8"/>
@@ -4216,13 +4236,13 @@
         <v>59</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D49" s="8" t="s">
         <v>60</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F49" s="8"/>
       <c r="G49" s="8"/>
@@ -4247,13 +4267,13 @@
         <v>61</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="D50" s="8" t="s">
         <v>62</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
@@ -4278,13 +4298,13 @@
         <v>75</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="D51" s="8" t="s">
         <v>298</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F51" s="8"/>
       <c r="G51" s="8"/>
@@ -4309,13 +4329,13 @@
         <v>146</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="D52" s="8" t="s">
         <v>299</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F52" s="8"/>
       <c r="G52" s="8"/>
@@ -4340,13 +4360,13 @@
         <v>147</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="D53" s="8" t="s">
         <v>300</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F53" s="8"/>
       <c r="G53" s="8"/>
@@ -4371,13 +4391,13 @@
         <v>148</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="D54" s="8" t="s">
         <v>301</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F54" s="8"/>
       <c r="G54" s="8"/>
@@ -4402,13 +4422,13 @@
         <v>63</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="D55" s="8" t="s">
         <v>64</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F55" s="8"/>
       <c r="G55" s="8"/>
@@ -4433,13 +4453,13 @@
         <v>149</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="D56" s="8" t="s">
         <v>302</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F56" s="8"/>
       <c r="G56" s="8"/>
@@ -4464,13 +4484,13 @@
         <v>150</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="D57" s="8" t="s">
         <v>303</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F57" s="8"/>
       <c r="G57" s="8"/>
@@ -4495,13 +4515,13 @@
         <v>151</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D58" s="8" t="s">
         <v>304</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F58" s="8"/>
       <c r="G58" s="8"/>
@@ -4526,13 +4546,13 @@
         <v>152</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D59" s="8" t="s">
         <v>305</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F59" s="8"/>
       <c r="G59" s="8"/>
@@ -4557,13 +4577,13 @@
         <v>153</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="D60" s="8" t="s">
         <v>306</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F60" s="8"/>
       <c r="G60" s="8"/>
@@ -4588,13 +4608,13 @@
         <v>65</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D61" s="8" t="s">
         <v>66</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F61" s="8"/>
       <c r="G61" s="8"/>
@@ -4619,13 +4639,13 @@
         <v>107</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D62" s="8" t="s">
         <v>307</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F62" s="8"/>
       <c r="G62" s="8"/>
@@ -4650,13 +4670,13 @@
         <v>154</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="D63" s="8" t="s">
         <v>308</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F63" s="8"/>
       <c r="G63" s="8"/>
@@ -4681,13 +4701,13 @@
         <v>67</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="D64" s="8" t="s">
         <v>68</v>
       </c>
       <c r="E64" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F64" s="8"/>
       <c r="G64" s="8"/>
@@ -4712,13 +4732,13 @@
         <v>155</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="D65" s="8" t="s">
         <v>309</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F65" s="8"/>
       <c r="G65" s="8"/>
@@ -4743,13 +4763,13 @@
         <v>156</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D66" s="8" t="s">
         <v>310</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F66" s="8"/>
       <c r="G66" s="8"/>
@@ -4774,13 +4794,13 @@
         <v>157</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="D67" s="8" t="s">
         <v>311</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F67" s="8"/>
       <c r="G67" s="8"/>
@@ -4805,13 +4825,13 @@
         <v>69</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="D68" s="8" t="s">
         <v>70</v>
       </c>
       <c r="E68" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F68" s="8"/>
       <c r="G68" s="8"/>
@@ -4836,13 +4856,13 @@
         <v>158</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="D69" s="8" t="s">
         <v>312</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F69" s="8"/>
       <c r="G69" s="8"/>
@@ -4867,13 +4887,13 @@
         <v>159</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="D70" s="8" t="s">
         <v>313</v>
       </c>
       <c r="E70" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F70" s="8"/>
       <c r="G70" s="8"/>
@@ -4898,13 +4918,13 @@
         <v>71</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="D71" s="8" t="s">
         <v>72</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F71" s="8"/>
       <c r="G71" s="8"/>
@@ -4929,13 +4949,13 @@
         <v>160</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="D72" s="8" t="s">
         <v>314</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F72" s="8"/>
       <c r="G72" s="8"/>
@@ -4960,13 +4980,13 @@
         <v>161</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="D73" s="8" t="s">
         <v>315</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F73" s="8"/>
       <c r="G73" s="8"/>
@@ -4991,13 +5011,13 @@
         <v>162</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="D74" s="8" t="s">
         <v>316</v>
       </c>
       <c r="E74" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F74" s="8"/>
       <c r="G74" s="8"/>
@@ -5022,13 +5042,13 @@
         <v>163</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D75" s="8" t="s">
         <v>317</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F75" s="8"/>
       <c r="G75" s="8"/>
@@ -5053,13 +5073,13 @@
         <v>164</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="D76" s="8" t="s">
         <v>318</v>
       </c>
       <c r="E76" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F76" s="8"/>
       <c r="G76" s="8"/>
@@ -5084,13 +5104,13 @@
         <v>165</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D77" s="8" t="s">
         <v>319</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F77" s="8"/>
       <c r="G77" s="8"/>
@@ -5115,13 +5135,13 @@
         <v>166</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="D78" s="8" t="s">
         <v>320</v>
       </c>
       <c r="E78" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F78" s="8"/>
       <c r="G78" s="8"/>
@@ -5146,13 +5166,13 @@
         <v>167</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="D79" s="8" t="s">
         <v>321</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F79" s="8"/>
       <c r="G79" s="8"/>
@@ -5177,13 +5197,13 @@
         <v>168</v>
       </c>
       <c r="C80" s="8" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D80" s="8" t="s">
         <v>322</v>
       </c>
       <c r="E80" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F80" s="8"/>
       <c r="G80" s="8"/>
@@ -5208,13 +5228,13 @@
         <v>169</v>
       </c>
       <c r="C81" s="8" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D81" s="8" t="s">
         <v>323</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F81" s="8"/>
       <c r="G81" s="8"/>
@@ -5239,13 +5259,13 @@
         <v>170</v>
       </c>
       <c r="C82" s="8" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="D82" s="8" t="s">
         <v>324</v>
       </c>
       <c r="E82" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F82" s="8"/>
       <c r="G82" s="8"/>
@@ -5270,13 +5290,13 @@
         <v>171</v>
       </c>
       <c r="C83" s="8" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="D83" s="8" t="s">
         <v>325</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F83" s="8"/>
       <c r="G83" s="8"/>
@@ -5301,13 +5321,13 @@
         <v>172</v>
       </c>
       <c r="C84" s="8" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="D84" s="8" t="s">
         <v>326</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F84" s="8"/>
       <c r="G84" s="8"/>
@@ -5332,13 +5352,13 @@
         <v>173</v>
       </c>
       <c r="C85" s="8" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="D85" s="8" t="s">
         <v>327</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F85" s="8"/>
       <c r="G85" s="8"/>
@@ -5363,13 +5383,13 @@
         <v>174</v>
       </c>
       <c r="C86" s="8" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="D86" s="8" t="s">
         <v>328</v>
       </c>
       <c r="E86" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F86" s="8"/>
       <c r="G86" s="8"/>
@@ -5394,13 +5414,13 @@
         <v>175</v>
       </c>
       <c r="C87" s="8" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="D87" s="8" t="s">
         <v>329</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F87" s="8"/>
       <c r="G87" s="8"/>
@@ -5425,13 +5445,13 @@
         <v>176</v>
       </c>
       <c r="C88" s="8" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D88" s="8" t="s">
         <v>330</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F88" s="8"/>
       <c r="G88" s="8"/>
@@ -5456,13 +5476,13 @@
         <v>177</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="D89" s="8" t="s">
         <v>331</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F89" s="8"/>
       <c r="G89" s="8"/>
@@ -5487,13 +5507,13 @@
         <v>178</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D90" s="8" t="s">
         <v>332</v>
       </c>
       <c r="E90" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F90" s="8"/>
       <c r="G90" s="8"/>
@@ -5518,13 +5538,13 @@
         <v>179</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="D91" s="8" t="s">
         <v>333</v>
       </c>
       <c r="E91" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F91" s="8"/>
       <c r="G91" s="8"/>
@@ -5549,13 +5569,13 @@
         <v>180</v>
       </c>
       <c r="C92" s="8" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D92" s="8" t="s">
         <v>334</v>
       </c>
       <c r="E92" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F92" s="8"/>
       <c r="G92" s="8"/>
@@ -5580,13 +5600,13 @@
         <v>181</v>
       </c>
       <c r="C93" s="8" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="D93" s="8" t="s">
         <v>335</v>
       </c>
       <c r="E93" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F93" s="8"/>
       <c r="G93" s="8"/>
@@ -5611,13 +5631,13 @@
         <v>182</v>
       </c>
       <c r="C94" s="8" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="D94" s="8" t="s">
         <v>336</v>
       </c>
       <c r="E94" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F94" s="8"/>
       <c r="G94" s="8"/>
@@ -5642,13 +5662,13 @@
         <v>183</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="D95" s="8" t="s">
         <v>337</v>
       </c>
       <c r="E95" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F95" s="8"/>
       <c r="G95" s="8"/>
@@ -5673,13 +5693,13 @@
         <v>184</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="D96" s="8" t="s">
         <v>338</v>
       </c>
       <c r="E96" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F96" s="8"/>
       <c r="G96" s="8"/>
@@ -5704,13 +5724,13 @@
         <v>185</v>
       </c>
       <c r="C97" s="8" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="D97" s="8" t="s">
         <v>339</v>
       </c>
       <c r="E97" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F97" s="8"/>
       <c r="G97" s="8"/>
@@ -5735,13 +5755,13 @@
         <v>186</v>
       </c>
       <c r="C98" s="8" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="D98" s="8" t="s">
         <v>340</v>
       </c>
       <c r="E98" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F98" s="8"/>
       <c r="G98" s="8"/>
@@ -5766,13 +5786,13 @@
         <v>187</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="D99" s="8" t="s">
         <v>341</v>
       </c>
       <c r="E99" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F99" s="8"/>
       <c r="G99" s="8"/>
@@ -5797,13 +5817,13 @@
         <v>188</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="D100" s="8" t="s">
         <v>342</v>
       </c>
       <c r="E100" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F100" s="8"/>
       <c r="G100" s="8"/>
@@ -5828,13 +5848,13 @@
         <v>189</v>
       </c>
       <c r="C101" s="8" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="D101" s="8" t="s">
-        <v>343</v>
+        <v>730</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F101" s="8"/>
       <c r="G101" s="8"/>
@@ -5859,13 +5879,13 @@
         <v>190</v>
       </c>
       <c r="C102" s="8" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="D102" s="8" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E102" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F102" s="8"/>
       <c r="G102" s="8"/>
@@ -5890,13 +5910,13 @@
         <v>191</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="D103" s="8" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F103" s="8"/>
       <c r="G103" s="8"/>
@@ -5921,13 +5941,13 @@
         <v>192</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="D104" s="8" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E104" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F104" s="8"/>
       <c r="G104" s="8"/>
@@ -5952,13 +5972,13 @@
         <v>193</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="D105" s="8" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E105" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F105" s="8"/>
       <c r="G105" s="8"/>
@@ -5983,13 +6003,13 @@
         <v>194</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="D106" s="8" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E106" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F106" s="8"/>
       <c r="G106" s="8"/>
@@ -6014,13 +6034,13 @@
         <v>195</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="D107" s="8" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E107" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F107" s="8"/>
       <c r="G107" s="8"/>
@@ -6045,13 +6065,13 @@
         <v>196</v>
       </c>
       <c r="C108" s="8" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="D108" s="8" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E108" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F108" s="8"/>
       <c r="G108" s="8"/>
@@ -6076,13 +6096,13 @@
         <v>197</v>
       </c>
       <c r="C109" s="8" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D109" s="8" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E109" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F109" s="8"/>
       <c r="G109" s="8"/>
@@ -6107,13 +6127,13 @@
         <v>198</v>
       </c>
       <c r="C110" s="8" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="D110" s="8" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E110" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F110" s="8"/>
       <c r="G110" s="8"/>
@@ -6138,13 +6158,13 @@
         <v>199</v>
       </c>
       <c r="C111" s="8" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="D111" s="8" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E111" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F111" s="8"/>
       <c r="G111" s="8"/>
@@ -6169,13 +6189,13 @@
         <v>200</v>
       </c>
       <c r="C112" s="8" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="D112" s="8" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E112" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F112" s="8"/>
       <c r="G112" s="8"/>
@@ -6200,13 +6220,13 @@
         <v>201</v>
       </c>
       <c r="C113" s="8" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="D113" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E113" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F113" s="8"/>
       <c r="G113" s="8"/>
@@ -6231,13 +6251,13 @@
         <v>202</v>
       </c>
       <c r="C114" s="8" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="D114" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E114" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F114" s="8"/>
       <c r="G114" s="8"/>
@@ -6262,13 +6282,13 @@
         <v>203</v>
       </c>
       <c r="C115" s="8" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D115" s="8" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E115" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F115" s="8"/>
       <c r="G115" s="8"/>
@@ -6293,13 +6313,13 @@
         <v>204</v>
       </c>
       <c r="C116" s="8" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="D116" s="8" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E116" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F116" s="8"/>
       <c r="G116" s="8"/>
@@ -6324,13 +6344,13 @@
         <v>205</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="D117" s="8" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E117" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F117" s="8"/>
       <c r="G117" s="8"/>
@@ -6355,13 +6375,13 @@
         <v>206</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D118" s="8" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E118" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F118" s="8"/>
       <c r="G118" s="8"/>
@@ -6386,13 +6406,13 @@
         <v>207</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="D119" s="8" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E119" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F119" s="8"/>
       <c r="G119" s="8"/>
@@ -6417,13 +6437,13 @@
         <v>208</v>
       </c>
       <c r="C120" s="8" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="D120" s="8" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E120" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F120" s="8"/>
       <c r="G120" s="8"/>
@@ -6448,13 +6468,13 @@
         <v>209</v>
       </c>
       <c r="C121" s="8" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="D121" s="8" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E121" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F121" s="8"/>
       <c r="G121" s="8"/>
@@ -6479,13 +6499,13 @@
         <v>210</v>
       </c>
       <c r="C122" s="8" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="D122" s="8" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E122" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F122" s="8"/>
       <c r="G122" s="8"/>
@@ -6510,13 +6530,13 @@
         <v>81</v>
       </c>
       <c r="C123" s="8" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D123" s="8" t="s">
         <v>82</v>
       </c>
       <c r="E123" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F123" s="8"/>
       <c r="G123" s="8"/>
@@ -6541,13 +6561,13 @@
         <v>211</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="D124" s="8" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E124" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F124" s="8"/>
       <c r="G124" s="8"/>
@@ -6572,13 +6592,13 @@
         <v>83</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="D125" s="8" t="s">
         <v>84</v>
       </c>
       <c r="E125" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F125" s="8"/>
       <c r="G125" s="8"/>
@@ -6603,13 +6623,13 @@
         <v>85</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="D126" s="8" t="s">
         <v>86</v>
       </c>
       <c r="E126" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F126" s="8"/>
       <c r="G126" s="8"/>
@@ -6634,13 +6654,13 @@
         <v>212</v>
       </c>
       <c r="C127" s="8" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="D127" s="8" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E127" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F127" s="8"/>
       <c r="G127" s="8"/>
@@ -6665,13 +6685,13 @@
         <v>87</v>
       </c>
       <c r="C128" s="8" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D128" s="8" t="s">
         <v>88</v>
       </c>
       <c r="E128" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F128" s="8"/>
       <c r="G128" s="8"/>
@@ -6696,13 +6716,13 @@
         <v>213</v>
       </c>
       <c r="C129" s="8" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D129" s="8" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E129" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F129" s="8"/>
       <c r="G129" s="8"/>
@@ -6727,13 +6747,13 @@
         <v>214</v>
       </c>
       <c r="C130" s="8" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D130" s="8" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E130" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F130" s="8"/>
       <c r="G130" s="8"/>
@@ -6758,13 +6778,13 @@
         <v>215</v>
       </c>
       <c r="C131" s="8" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D131" s="8" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E131" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F131" s="8"/>
       <c r="G131" s="8"/>
@@ -6789,13 +6809,13 @@
         <v>216</v>
       </c>
       <c r="C132" s="8" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="D132" s="8" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E132" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F132" s="8"/>
       <c r="G132" s="8"/>
@@ -6820,13 +6840,13 @@
         <v>217</v>
       </c>
       <c r="C133" s="8" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="D133" s="8" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E133" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F133" s="8"/>
       <c r="G133" s="8"/>
@@ -6851,13 +6871,13 @@
         <v>218</v>
       </c>
       <c r="C134" s="8" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="D134" s="8" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E134" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F134" s="8"/>
       <c r="G134" s="8"/>
@@ -6882,13 +6902,13 @@
         <v>219</v>
       </c>
       <c r="C135" s="8" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D135" s="8" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E135" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F135" s="8"/>
       <c r="G135" s="8"/>
@@ -6913,13 +6933,13 @@
         <v>220</v>
       </c>
       <c r="C136" s="8" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="D136" s="8" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E136" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F136" s="8"/>
       <c r="G136" s="8"/>
@@ -6944,13 +6964,13 @@
         <v>221</v>
       </c>
       <c r="C137" s="8" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D137" s="8" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E137" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F137" s="8"/>
       <c r="G137" s="8"/>
@@ -6975,13 +6995,13 @@
         <v>89</v>
       </c>
       <c r="C138" s="8" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="D138" s="8" t="s">
         <v>90</v>
       </c>
       <c r="E138" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F138" s="8"/>
       <c r="G138" s="8"/>
@@ -7006,13 +7026,13 @@
         <v>222</v>
       </c>
       <c r="C139" s="8" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="D139" s="8" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E139" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F139" s="8"/>
       <c r="G139" s="8"/>
@@ -7037,13 +7057,13 @@
         <v>223</v>
       </c>
       <c r="C140" s="8" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D140" s="8" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E140" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F140" s="8"/>
       <c r="G140" s="8"/>
@@ -7068,13 +7088,13 @@
         <v>91</v>
       </c>
       <c r="C141" s="8" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="D141" s="8" t="s">
         <v>92</v>
       </c>
       <c r="E141" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F141" s="8"/>
       <c r="G141" s="8"/>
@@ -7099,13 +7119,13 @@
         <v>224</v>
       </c>
       <c r="C142" s="8" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="D142" s="8" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E142" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F142" s="8"/>
       <c r="G142" s="8"/>
@@ -7130,13 +7150,13 @@
         <v>225</v>
       </c>
       <c r="C143" s="8" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="D143" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E143" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F143" s="8"/>
       <c r="G143" s="8"/>
@@ -7161,13 +7181,13 @@
         <v>226</v>
       </c>
       <c r="C144" s="8" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D144" s="8" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E144" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F144" s="8"/>
       <c r="G144" s="8"/>
@@ -7192,13 +7212,13 @@
         <v>227</v>
       </c>
       <c r="C145" s="8" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="D145" s="8" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E145" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F145" s="8"/>
       <c r="G145" s="8"/>
@@ -7223,13 +7243,13 @@
         <v>228</v>
       </c>
       <c r="C146" s="8" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="D146" s="8" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E146" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F146" s="8"/>
       <c r="G146" s="8"/>
@@ -7254,13 +7274,13 @@
         <v>229</v>
       </c>
       <c r="C147" s="8" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="D147" s="8" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E147" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F147" s="8"/>
       <c r="G147" s="8"/>
@@ -7285,13 +7305,13 @@
         <v>230</v>
       </c>
       <c r="C148" s="8" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D148" s="8" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E148" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F148" s="8"/>
       <c r="G148" s="8"/>
@@ -7316,13 +7336,13 @@
         <v>231</v>
       </c>
       <c r="C149" s="8" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="D149" s="8" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E149" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F149" s="8"/>
       <c r="G149" s="8"/>
@@ -7347,13 +7367,13 @@
         <v>76</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="D150" s="8" t="s">
         <v>77</v>
       </c>
       <c r="E150" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F150" s="8"/>
       <c r="G150" s="8"/>
@@ -7378,13 +7398,13 @@
         <v>78</v>
       </c>
       <c r="C151" s="8" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="D151" s="8" t="s">
         <v>79</v>
       </c>
       <c r="E151" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F151" s="8"/>
       <c r="G151" s="8"/>
@@ -7409,13 +7429,13 @@
         <v>73</v>
       </c>
       <c r="C152" s="8" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="D152" s="8" t="s">
         <v>74</v>
       </c>
       <c r="E152" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F152" s="8"/>
       <c r="G152" s="8"/>
@@ -7440,13 +7460,13 @@
         <v>232</v>
       </c>
       <c r="C153" s="8" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="D153" s="8" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E153" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F153" s="8"/>
       <c r="G153" s="8"/>
@@ -7471,13 +7491,13 @@
         <v>233</v>
       </c>
       <c r="C154" s="8" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="D154" s="8" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E154" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F154" s="8"/>
       <c r="G154" s="8"/>
@@ -7502,13 +7522,13 @@
         <v>234</v>
       </c>
       <c r="C155" s="8" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="D155" s="8" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E155" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F155" s="8"/>
       <c r="G155" s="8"/>
@@ -7533,13 +7553,13 @@
         <v>235</v>
       </c>
       <c r="C156" s="8" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="D156" s="8" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E156" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F156" s="8"/>
       <c r="G156" s="8"/>
@@ -7564,13 +7584,13 @@
         <v>236</v>
       </c>
       <c r="C157" s="8" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="D157" s="8" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E157" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F157" s="8"/>
       <c r="G157" s="8"/>
@@ -7595,13 +7615,13 @@
         <v>237</v>
       </c>
       <c r="C158" s="8" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="D158" s="8" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E158" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F158" s="8"/>
       <c r="G158" s="8"/>
@@ -7626,13 +7646,13 @@
         <v>108</v>
       </c>
       <c r="C159" s="8" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="D159" s="8" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E159" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F159" s="8"/>
       <c r="G159" s="8"/>
@@ -7657,13 +7677,13 @@
         <v>238</v>
       </c>
       <c r="C160" s="8" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D160" s="8" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E160" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F160" s="8"/>
       <c r="G160" s="8"/>
@@ -7688,13 +7708,13 @@
         <v>239</v>
       </c>
       <c r="C161" s="8" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="D161" s="8" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="E161" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F161" s="8"/>
       <c r="G161" s="8"/>
@@ -7719,13 +7739,13 @@
         <v>53</v>
       </c>
       <c r="C162" s="8" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D162" s="8" t="s">
         <v>54</v>
       </c>
       <c r="E162" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F162" s="8"/>
       <c r="G162" s="8"/>
@@ -7750,13 +7770,13 @@
         <v>98</v>
       </c>
       <c r="C163" s="8" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D163" s="8" t="s">
         <v>99</v>
       </c>
       <c r="E163" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F163" s="8"/>
       <c r="G163" s="8"/>
@@ -7781,13 +7801,13 @@
         <v>100</v>
       </c>
       <c r="C164" s="8" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D164" s="8" t="s">
         <v>101</v>
       </c>
       <c r="E164" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F164" s="8"/>
       <c r="G164" s="8"/>
@@ -7812,13 +7832,13 @@
         <v>240</v>
       </c>
       <c r="C165" s="8" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D165" s="8" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E165" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F165" s="8"/>
       <c r="G165" s="8"/>
@@ -7843,13 +7863,13 @@
         <v>102</v>
       </c>
       <c r="C166" s="8" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D166" s="8" t="s">
         <v>103</v>
       </c>
       <c r="E166" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F166" s="8"/>
       <c r="G166" s="8"/>
@@ -7874,13 +7894,13 @@
         <v>241</v>
       </c>
       <c r="C167" s="8" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D167" s="8" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E167" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F167" s="8"/>
       <c r="G167" s="8"/>
@@ -7905,13 +7925,13 @@
         <v>242</v>
       </c>
       <c r="C168" s="8" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D168" s="8" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E168" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F168" s="8"/>
       <c r="G168" s="8"/>
@@ -7936,13 +7956,13 @@
         <v>243</v>
       </c>
       <c r="C169" s="8" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D169" s="8" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="E169" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F169" s="8"/>
       <c r="G169" s="8"/>
@@ -7967,13 +7987,13 @@
         <v>244</v>
       </c>
       <c r="C170" s="8" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D170" s="8" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="E170" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F170" s="8"/>
       <c r="G170" s="8"/>
@@ -7998,13 +8018,13 @@
         <v>245</v>
       </c>
       <c r="C171" s="8" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D171" s="8" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E171" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F171" s="8"/>
       <c r="G171" s="8"/>
@@ -8029,13 +8049,13 @@
         <v>93</v>
       </c>
       <c r="C172" s="8" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D172" s="8" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E172" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F172" s="8"/>
       <c r="G172" s="8"/>
@@ -8060,13 +8080,13 @@
         <v>246</v>
       </c>
       <c r="C173" s="8" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D173" s="8" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E173" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F173" s="8"/>
       <c r="G173" s="8"/>
@@ -8091,13 +8111,13 @@
         <v>94</v>
       </c>
       <c r="C174" s="8" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D174" s="8" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="E174" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F174" s="8"/>
       <c r="G174" s="8"/>
@@ -8122,13 +8142,13 @@
         <v>247</v>
       </c>
       <c r="C175" s="8" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D175" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="E175" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F175" s="8"/>
       <c r="G175" s="8"/>
@@ -8153,13 +8173,13 @@
         <v>248</v>
       </c>
       <c r="C176" s="8" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D176" s="8" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="E176" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F176" s="8"/>
       <c r="G176" s="8"/>
@@ -8184,13 +8204,13 @@
         <v>249</v>
       </c>
       <c r="C177" s="8" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D177" s="8" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E177" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F177" s="8"/>
       <c r="G177" s="8"/>
@@ -8215,13 +8235,13 @@
         <v>95</v>
       </c>
       <c r="C178" s="8" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D178" s="8" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E178" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F178" s="8"/>
       <c r="G178" s="8"/>
@@ -8246,13 +8266,13 @@
         <v>96</v>
       </c>
       <c r="C179" s="8" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D179" s="8" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="E179" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F179" s="8"/>
       <c r="G179" s="8"/>
@@ -8277,13 +8297,13 @@
         <v>250</v>
       </c>
       <c r="C180" s="8" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D180" s="8" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="E180" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F180" s="8"/>
       <c r="G180" s="8"/>
@@ -8308,13 +8328,13 @@
         <v>251</v>
       </c>
       <c r="C181" s="8" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D181" s="8" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="E181" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F181" s="8"/>
       <c r="G181" s="8"/>
@@ -8339,13 +8359,13 @@
         <v>252</v>
       </c>
       <c r="C182" s="8" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D182" s="8" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="E182" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F182" s="8"/>
       <c r="G182" s="8"/>
@@ -8370,13 +8390,13 @@
         <v>97</v>
       </c>
       <c r="C183" s="8" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D183" s="8" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="E183" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F183" s="8"/>
       <c r="G183" s="8"/>
@@ -8401,13 +8421,13 @@
         <v>253</v>
       </c>
       <c r="C184" s="8" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D184" s="8" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E184" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F184" s="8"/>
       <c r="G184" s="8"/>
@@ -8432,13 +8452,13 @@
         <v>254</v>
       </c>
       <c r="C185" s="8" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D185" s="8" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="E185" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F185" s="8"/>
       <c r="G185" s="8"/>
@@ -8463,13 +8483,13 @@
         <v>255</v>
       </c>
       <c r="C186" s="8" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D186" s="8" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="E186" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F186" s="8"/>
       <c r="G186" s="8"/>
@@ -8494,13 +8514,13 @@
         <v>104</v>
       </c>
       <c r="C187" s="8" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D187" s="8" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="E187" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F187" s="8"/>
       <c r="G187" s="8"/>
@@ -8525,13 +8545,13 @@
         <v>256</v>
       </c>
       <c r="C188" s="8" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D188" s="8" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="E188" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F188" s="8"/>
       <c r="G188" s="8"/>
@@ -8556,13 +8576,13 @@
         <v>257</v>
       </c>
       <c r="C189" s="8" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D189" s="8" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="E189" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F189" s="8"/>
       <c r="G189" s="8"/>
@@ -8587,13 +8607,13 @@
         <v>105</v>
       </c>
       <c r="C190" s="8" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D190" s="8" t="s">
         <v>106</v>
       </c>
       <c r="E190" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F190" s="8"/>
       <c r="G190" s="8"/>
@@ -8618,13 +8638,13 @@
         <v>258</v>
       </c>
       <c r="C191" s="8" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D191" s="8" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="E191" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F191" s="8"/>
       <c r="G191" s="8"/>
@@ -8649,13 +8669,13 @@
         <v>259</v>
       </c>
       <c r="C192" s="8" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D192" s="8" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="E192" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F192" s="8"/>
       <c r="G192" s="8"/>
@@ -8680,13 +8700,13 @@
         <v>260</v>
       </c>
       <c r="C193" s="8" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D193" s="8" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="E193" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F193" s="8"/>
       <c r="G193" s="8"/>
@@ -8711,13 +8731,13 @@
         <v>261</v>
       </c>
       <c r="C194" s="8" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D194" s="8" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E194" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F194" s="8"/>
       <c r="G194" s="8"/>
@@ -8742,13 +8762,13 @@
         <v>109</v>
       </c>
       <c r="C195" s="8" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D195" s="8" t="s">
         <v>110</v>
       </c>
       <c r="E195" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F195" s="8"/>
       <c r="G195" s="8"/>
@@ -8773,13 +8793,13 @@
         <v>262</v>
       </c>
       <c r="C196" s="8" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D196" s="8" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E196" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F196" s="8"/>
       <c r="G196" s="8"/>
@@ -8804,13 +8824,13 @@
         <v>263</v>
       </c>
       <c r="C197" s="8" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D197" s="8" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E197" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F197" s="8"/>
       <c r="G197" s="8"/>
@@ -8835,13 +8855,13 @@
         <v>264</v>
       </c>
       <c r="C198" s="8" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D198" s="8" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E198" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F198" s="8"/>
       <c r="G198" s="8"/>
@@ -8866,13 +8886,13 @@
         <v>265</v>
       </c>
       <c r="C199" s="8" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D199" s="8" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E199" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F199" s="8"/>
       <c r="G199" s="8"/>
@@ -8897,13 +8917,13 @@
         <v>266</v>
       </c>
       <c r="C200" s="8" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D200" s="8" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E200" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F200" s="8"/>
       <c r="G200" s="8"/>
@@ -8928,13 +8948,13 @@
         <v>267</v>
       </c>
       <c r="C201" s="8" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D201" s="8" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E201" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F201" s="8"/>
       <c r="G201" s="8"/>
@@ -8959,13 +8979,13 @@
         <v>111</v>
       </c>
       <c r="C202" s="8" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D202" s="8" t="s">
         <v>112</v>
       </c>
       <c r="E202" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F202" s="8"/>
       <c r="G202" s="8"/>
@@ -8990,13 +9010,13 @@
         <v>268</v>
       </c>
       <c r="C203" s="8" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D203" s="8" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E203" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F203" s="8"/>
       <c r="G203" s="8"/>
@@ -9018,16 +9038,16 @@
         <v>4</v>
       </c>
       <c r="B204" s="8" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="C204" s="8" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="D204" s="8" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E204" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F204" s="8"/>
       <c r="G204" s="8"/>
@@ -9049,16 +9069,16 @@
         <v>4</v>
       </c>
       <c r="B205" s="8" t="s">
+        <v>687</v>
+      </c>
+      <c r="C205" s="8" t="s">
         <v>688</v>
       </c>
-      <c r="C205" s="8" t="s">
-        <v>689</v>
-      </c>
       <c r="D205" s="8" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E205" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F205" s="8"/>
       <c r="G205" s="8"/>
@@ -9083,13 +9103,13 @@
         <v>269</v>
       </c>
       <c r="C206" s="8" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D206" s="8" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E206" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F206" s="8"/>
       <c r="G206" s="8"/>
@@ -9113,10 +9133,10 @@
       <c r="B207" s="8"/>
       <c r="C207" s="8"/>
       <c r="D207" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E207" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F207" s="8"/>
       <c r="G207" s="8"/>
@@ -9141,13 +9161,13 @@
         <v>270</v>
       </c>
       <c r="C208" s="8" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D208" s="8" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E208" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F208" s="8"/>
       <c r="G208" s="8"/>
@@ -9172,13 +9192,13 @@
         <v>271</v>
       </c>
       <c r="C209" s="8" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D209" s="8" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E209" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F209" s="8"/>
       <c r="G209" s="8"/>
@@ -9200,16 +9220,16 @@
         <v>4</v>
       </c>
       <c r="B210" s="8" t="s">
+        <v>689</v>
+      </c>
+      <c r="C210" s="8" t="s">
         <v>690</v>
       </c>
-      <c r="C210" s="8" t="s">
-        <v>691</v>
-      </c>
       <c r="D210" s="8" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E210" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F210" s="8"/>
       <c r="G210" s="8"/>
@@ -9231,16 +9251,16 @@
         <v>4</v>
       </c>
       <c r="B211" s="8" t="s">
+        <v>691</v>
+      </c>
+      <c r="C211" s="8" t="s">
         <v>692</v>
       </c>
-      <c r="C211" s="8" t="s">
-        <v>693</v>
-      </c>
       <c r="D211" s="8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E211" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F211" s="8"/>
       <c r="G211" s="8"/>
@@ -9262,16 +9282,16 @@
         <v>4</v>
       </c>
       <c r="B212" s="8" t="s">
+        <v>693</v>
+      </c>
+      <c r="C212" s="8" t="s">
         <v>694</v>
       </c>
-      <c r="C212" s="8" t="s">
-        <v>695</v>
-      </c>
       <c r="D212" s="8" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E212" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F212" s="8"/>
       <c r="G212" s="8"/>
@@ -9296,13 +9316,13 @@
         <v>272</v>
       </c>
       <c r="C213" s="8" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D213" s="8" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E213" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F213" s="8"/>
       <c r="G213" s="8"/>
@@ -9327,13 +9347,13 @@
         <v>273</v>
       </c>
       <c r="C214" s="8" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D214" s="8" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E214" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F214" s="8"/>
       <c r="G214" s="8"/>
@@ -9358,13 +9378,13 @@
         <v>274</v>
       </c>
       <c r="C215" s="8" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D215" s="8" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E215" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F215" s="8"/>
       <c r="G215" s="8"/>
@@ -9389,13 +9409,13 @@
         <v>275</v>
       </c>
       <c r="C216" s="8" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D216" s="8" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E216" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F216" s="8"/>
       <c r="G216" s="8"/>
@@ -9420,13 +9440,13 @@
         <v>276</v>
       </c>
       <c r="C217" s="8" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D217" s="8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E217" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F217" s="8"/>
       <c r="G217" s="8"/>
@@ -9448,16 +9468,16 @@
         <v>4</v>
       </c>
       <c r="B218" s="8" t="s">
+        <v>695</v>
+      </c>
+      <c r="C218" s="8" t="s">
         <v>696</v>
       </c>
-      <c r="C218" s="8" t="s">
-        <v>697</v>
-      </c>
       <c r="D218" s="8" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E218" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F218" s="8"/>
       <c r="G218" s="8"/>
@@ -9479,16 +9499,16 @@
         <v>4</v>
       </c>
       <c r="B219" s="8" t="s">
+        <v>697</v>
+      </c>
+      <c r="C219" s="8" t="s">
         <v>698</v>
       </c>
-      <c r="C219" s="8" t="s">
-        <v>699</v>
-      </c>
       <c r="D219" s="8" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E219" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F219" s="8"/>
       <c r="G219" s="8"/>
@@ -9510,16 +9530,16 @@
         <v>4</v>
       </c>
       <c r="B220" s="8" t="s">
+        <v>699</v>
+      </c>
+      <c r="C220" s="8" t="s">
         <v>700</v>
       </c>
-      <c r="C220" s="8" t="s">
-        <v>701</v>
-      </c>
       <c r="D220" s="8" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E220" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F220" s="8"/>
       <c r="G220" s="8"/>
@@ -9541,16 +9561,16 @@
         <v>4</v>
       </c>
       <c r="B221" s="8" t="s">
+        <v>701</v>
+      </c>
+      <c r="C221" s="8" t="s">
         <v>702</v>
       </c>
-      <c r="C221" s="8" t="s">
-        <v>703</v>
-      </c>
       <c r="D221" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E221" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F221" s="8"/>
       <c r="G221" s="8"/>
@@ -9572,16 +9592,16 @@
         <v>4</v>
       </c>
       <c r="B222" s="8" t="s">
+        <v>703</v>
+      </c>
+      <c r="C222" s="8" t="s">
         <v>704</v>
       </c>
-      <c r="C222" s="8" t="s">
-        <v>705</v>
-      </c>
       <c r="D222" s="8" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E222" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F222" s="8"/>
       <c r="G222" s="8"/>
@@ -9603,16 +9623,16 @@
         <v>4</v>
       </c>
       <c r="B223" s="8" t="s">
+        <v>705</v>
+      </c>
+      <c r="C223" s="8" t="s">
         <v>706</v>
       </c>
-      <c r="C223" s="8" t="s">
-        <v>707</v>
-      </c>
       <c r="D223" s="8" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E223" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F223" s="8"/>
       <c r="G223" s="8"/>
@@ -9634,16 +9654,16 @@
         <v>4</v>
       </c>
       <c r="B224" s="8" t="s">
+        <v>707</v>
+      </c>
+      <c r="C224" s="8" t="s">
         <v>708</v>
       </c>
-      <c r="C224" s="8" t="s">
-        <v>709</v>
-      </c>
       <c r="D224" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E224" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F224" s="8"/>
       <c r="G224" s="8"/>
@@ -9665,16 +9685,16 @@
         <v>4</v>
       </c>
       <c r="B225" s="8" t="s">
+        <v>709</v>
+      </c>
+      <c r="C225" s="8" t="s">
         <v>710</v>
       </c>
-      <c r="C225" s="8" t="s">
-        <v>711</v>
-      </c>
       <c r="D225" s="8" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="E225" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F225" s="8"/>
       <c r="G225" s="8"/>
@@ -9696,16 +9716,16 @@
         <v>4</v>
       </c>
       <c r="B226" s="8" t="s">
+        <v>711</v>
+      </c>
+      <c r="C226" s="8" t="s">
         <v>712</v>
       </c>
-      <c r="C226" s="8" t="s">
-        <v>713</v>
-      </c>
       <c r="D226" s="8" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="E226" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F226" s="8"/>
       <c r="G226" s="8"/>
@@ -9727,16 +9747,16 @@
         <v>4</v>
       </c>
       <c r="B227" s="8" t="s">
+        <v>713</v>
+      </c>
+      <c r="C227" s="8" t="s">
         <v>714</v>
       </c>
-      <c r="C227" s="8" t="s">
-        <v>715</v>
-      </c>
       <c r="D227" s="8" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="E227" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F227" s="8"/>
       <c r="G227" s="8"/>
@@ -9758,16 +9778,16 @@
         <v>4</v>
       </c>
       <c r="B228" s="8" t="s">
+        <v>715</v>
+      </c>
+      <c r="C228" s="8" t="s">
         <v>716</v>
       </c>
-      <c r="C228" s="8" t="s">
-        <v>717</v>
-      </c>
       <c r="D228" s="8" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E228" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F228" s="8"/>
       <c r="G228" s="8"/>
@@ -9789,16 +9809,16 @@
         <v>4</v>
       </c>
       <c r="B229" s="8" t="s">
+        <v>717</v>
+      </c>
+      <c r="C229" s="8" t="s">
         <v>718</v>
       </c>
-      <c r="C229" s="8" t="s">
-        <v>719</v>
-      </c>
       <c r="D229" s="8" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="E229" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F229" s="8"/>
       <c r="G229" s="8"/>
@@ -9820,16 +9840,16 @@
         <v>4</v>
       </c>
       <c r="B230" s="8" t="s">
+        <v>719</v>
+      </c>
+      <c r="C230" s="8" t="s">
         <v>720</v>
       </c>
-      <c r="C230" s="8" t="s">
-        <v>721</v>
-      </c>
       <c r="D230" s="8" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E230" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F230" s="8"/>
       <c r="G230" s="8"/>
@@ -9851,16 +9871,16 @@
         <v>4</v>
       </c>
       <c r="B231" s="8" t="s">
+        <v>721</v>
+      </c>
+      <c r="C231" s="8" t="s">
         <v>722</v>
       </c>
-      <c r="C231" s="8" t="s">
-        <v>723</v>
-      </c>
       <c r="D231" s="8" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="E231" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F231" s="8"/>
       <c r="G231" s="8"/>
@@ -9882,16 +9902,16 @@
         <v>4</v>
       </c>
       <c r="B232" s="8" t="s">
+        <v>723</v>
+      </c>
+      <c r="C232" s="8" t="s">
         <v>724</v>
       </c>
-      <c r="C232" s="8" t="s">
-        <v>725</v>
-      </c>
       <c r="D232" s="8" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="E232" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F232" s="8"/>
       <c r="G232" s="8"/>
@@ -9913,16 +9933,16 @@
         <v>4</v>
       </c>
       <c r="B233" s="8" t="s">
+        <v>725</v>
+      </c>
+      <c r="C233" s="8" t="s">
         <v>726</v>
       </c>
-      <c r="C233" s="8" t="s">
-        <v>727</v>
-      </c>
       <c r="D233" s="8" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="E233" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F233" s="8"/>
       <c r="G233" s="8"/>
@@ -9944,16 +9964,16 @@
         <v>4</v>
       </c>
       <c r="B234" s="8" t="s">
+        <v>727</v>
+      </c>
+      <c r="C234" s="8" t="s">
         <v>728</v>
       </c>
-      <c r="C234" s="8" t="s">
-        <v>729</v>
-      </c>
       <c r="D234" s="8" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="E234" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F234" s="8"/>
       <c r="G234" s="8"/>
@@ -9975,16 +9995,16 @@
         <v>80</v>
       </c>
       <c r="B235" s="8" t="s">
+        <v>674</v>
+      </c>
+      <c r="C235" s="8" t="s">
         <v>675</v>
       </c>
-      <c r="C235" s="8" t="s">
+      <c r="D235" s="8" t="s">
         <v>676</v>
       </c>
-      <c r="D235" s="8" t="s">
-        <v>677</v>
-      </c>
       <c r="E235" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F235" s="8"/>
       <c r="G235" s="8"/>
@@ -10006,16 +10026,16 @@
         <v>80</v>
       </c>
       <c r="B236" s="8" t="s">
+        <v>677</v>
+      </c>
+      <c r="C236" s="8" t="s">
         <v>678</v>
       </c>
-      <c r="C236" s="8" t="s">
+      <c r="D236" s="8" t="s">
         <v>679</v>
       </c>
-      <c r="D236" s="8" t="s">
-        <v>680</v>
-      </c>
       <c r="E236" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F236" s="8"/>
       <c r="G236" s="8"/>
@@ -10037,16 +10057,16 @@
         <v>80</v>
       </c>
       <c r="B237" s="8" t="s">
+        <v>680</v>
+      </c>
+      <c r="C237" s="8" t="s">
         <v>681</v>
       </c>
-      <c r="C237" s="8" t="s">
+      <c r="D237" s="8" t="s">
         <v>682</v>
       </c>
-      <c r="D237" s="8" t="s">
-        <v>683</v>
-      </c>
       <c r="E237" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F237" s="8"/>
       <c r="G237" s="8"/>
@@ -10068,16 +10088,16 @@
         <v>80</v>
       </c>
       <c r="B238" s="8" t="s">
+        <v>683</v>
+      </c>
+      <c r="C238" s="8" t="s">
         <v>684</v>
       </c>
-      <c r="C238" s="8" t="s">
+      <c r="D238" s="8" t="s">
         <v>685</v>
       </c>
-      <c r="D238" s="8" t="s">
-        <v>686</v>
-      </c>
       <c r="E238" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F238" s="8"/>
       <c r="G238" s="8"/>
@@ -10094,8 +10114,35 @@
       <c r="R238" s="8"/>
       <c r="S238" s="8"/>
     </row>
+    <row r="239" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A239" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B239" t="s">
+        <v>683</v>
+      </c>
+      <c r="C239" t="s">
+        <v>684</v>
+      </c>
+      <c r="D239" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="240" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A240" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B240" t="s">
+        <v>263</v>
+      </c>
+      <c r="C240" t="s">
+        <v>637</v>
+      </c>
+      <c r="D240" t="s">
+        <v>732</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S238" xr:uid="{96666041-4A3A-42C1-A22D-86A52389C7E2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Data: refresh CB master, Fossil files, and Nexlev shipments
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/CB Replenishment_Master.xlsx
+++ b/data/input/CB Replenishment_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3FA2CB-1D14-477B-A3B6-F76747E2EA9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C9B64CD-E8FA-45CF-A57B-E10FF77EF82D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CFE25F1-D4D7-4072-B0D8-85CA58EF1A1A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="733">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="733">
   <si>
     <t>ASIN</t>
   </si>
@@ -2346,7 +2346,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2373,6 +2373,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -10127,6 +10130,9 @@
       <c r="D239" t="s">
         <v>731</v>
       </c>
+      <c r="E239" s="11" t="s">
+        <v>440</v>
+      </c>
     </row>
     <row r="240" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A240" s="10" t="s">
@@ -10140,6 +10146,9 @@
       </c>
       <c r="D240" t="s">
         <v>732</v>
+      </c>
+      <c r="E240" s="11" t="s">
+        <v>440</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data: weekly refresh — replenishment masters + inventory + FBA shipments + sales snapshots
Refreshed inputs across all brands:
- AA & WM replenishment master (now 222 / 44 rows, aligned with V2)
- CB replenishment master (now 246 rows, aligned with V2 — FBA79974 model still under reconciliation)
- Fossil replenishment + in-transit PO + FBA shipments
- Inventory snapshots: WM, Audio Array, Tonor, Nexlev
- FBA shipments: Audio Array, WM, Nexlev, Viomi
- Weekly sales snapshots: main, CB Replenishment, ChinaReorder

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/CB Replenishment_Master.xlsx
+++ b/data/input/CB Replenishment_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03DE13AF-4A91-4232-BD1D-8280089E164F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{754AEFBA-8895-42DA-9921-7A0CD00883AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CFE25F1-D4D7-4072-B0D8-85CA58EF1A1A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$S$237</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$S$247</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1199" uniqueCount="724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="750">
   <si>
     <t>ASIN</t>
   </si>
@@ -1164,9 +1164,6 @@
     <t>AA-25M</t>
   </si>
   <si>
-    <t>AM-S1 Bookshelf Speaker</t>
-  </si>
-  <si>
     <t>AM-C45 Pro</t>
   </si>
   <si>
@@ -1203,9 +1200,6 @@
     <t>AM-W24</t>
   </si>
   <si>
-    <t>AM-Mix4 OTG</t>
-  </si>
-  <si>
     <t>AM-Pro8</t>
   </si>
   <si>
@@ -2209,6 +2203,90 @@
   </si>
   <si>
     <t>FBK79708</t>
+  </si>
+  <si>
+    <t>BE-4T</t>
+  </si>
+  <si>
+    <t>B0GY827J9C</t>
+  </si>
+  <si>
+    <t>FBA80074</t>
+  </si>
+  <si>
+    <t>PB-15 (AH-50+AM-C2+AI-04)</t>
+  </si>
+  <si>
+    <t>B0GXPGBQB1</t>
+  </si>
+  <si>
+    <t>FBA80075</t>
+  </si>
+  <si>
+    <t>PB-16 (AH-50+AI-13+AM-C2)</t>
+  </si>
+  <si>
+    <t>B0GY857139</t>
+  </si>
+  <si>
+    <t>FBA80076</t>
+  </si>
+  <si>
+    <t>PB-17 (AH-40-SL+AM-C43+AI-13)</t>
+  </si>
+  <si>
+    <t>B0GY86ZT1X</t>
+  </si>
+  <si>
+    <t>FBA80077</t>
+  </si>
+  <si>
+    <t>PB-18 (AH-45-BK+AI-03+AM-C39)</t>
+  </si>
+  <si>
+    <t>B0GXY7YJWP</t>
+  </si>
+  <si>
+    <t>FBA80104</t>
+  </si>
+  <si>
+    <t>UB-04 (AM-S2+AA-21+AI-04+AM-C2)</t>
+  </si>
+  <si>
+    <t>B0H2FNV2RC</t>
+  </si>
+  <si>
+    <t>FBA80105</t>
+  </si>
+  <si>
+    <t>UB-05 (AM-S2+AA-21)</t>
+  </si>
+  <si>
+    <t>B0H2FCK54H</t>
+  </si>
+  <si>
+    <t>FBA80106</t>
+  </si>
+  <si>
+    <t>UB-06 (AM-S2+AA-22)</t>
+  </si>
+  <si>
+    <t>B0H1MTP2ZP</t>
+  </si>
+  <si>
+    <t>FBA80143</t>
+  </si>
+  <si>
+    <t>B0FJS57732</t>
+  </si>
+  <si>
+    <t>FBA80141</t>
+  </si>
+  <si>
+    <t>B0H1H3K6B2</t>
+  </si>
+  <si>
+    <t>FBA80128</t>
   </si>
 </sst>
 </file>
@@ -2681,7 +2759,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96666041-4A3A-42C1-A22D-86A52389C7E2}">
-  <dimension ref="A1:S237"/>
+  <dimension ref="A1:S247"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
@@ -2709,16 +2787,16 @@
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>113</v>
@@ -2768,13 +2846,13 @@
         <v>123</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>275</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
@@ -2799,13 +2877,13 @@
         <v>5</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
@@ -2830,13 +2908,13 @@
         <v>7</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>8</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
@@ -2861,13 +2939,13 @@
         <v>9</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
@@ -2892,13 +2970,13 @@
         <v>11</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
@@ -2923,13 +3001,13 @@
         <v>13</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
@@ -2954,13 +3032,13 @@
         <v>124</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>276</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
@@ -2985,13 +3063,13 @@
         <v>15</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
@@ -3016,13 +3094,13 @@
         <v>17</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>18</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
@@ -3047,13 +3125,13 @@
         <v>19</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>20</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
@@ -3078,13 +3156,13 @@
         <v>125</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>277</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
@@ -3109,13 +3187,13 @@
         <v>126</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>278</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
@@ -3140,13 +3218,13 @@
         <v>21</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>22</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
@@ -3171,13 +3249,13 @@
         <v>23</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>24</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
@@ -3202,13 +3280,13 @@
         <v>25</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>26</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
@@ -3233,13 +3311,13 @@
         <v>27</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F17" s="8"/>
       <c r="G17" s="8"/>
@@ -3264,13 +3342,13 @@
         <v>29</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>30</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
@@ -3295,13 +3373,13 @@
         <v>31</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>32</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
@@ -3326,13 +3404,13 @@
         <v>33</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>34</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
@@ -3357,13 +3435,13 @@
         <v>127</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>279</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
@@ -3388,13 +3466,13 @@
         <v>35</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>36</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
@@ -3419,13 +3497,13 @@
         <v>37</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>38</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
@@ -3450,13 +3528,13 @@
         <v>128</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>280</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F24" s="8"/>
       <c r="G24" s="8"/>
@@ -3481,13 +3559,13 @@
         <v>39</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>40</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
@@ -3512,13 +3590,13 @@
         <v>41</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>42</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
@@ -3543,13 +3621,13 @@
         <v>129</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>281</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
@@ -3574,13 +3652,13 @@
         <v>43</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>44</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F28" s="8"/>
       <c r="G28" s="8"/>
@@ -3605,13 +3683,13 @@
         <v>45</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>46</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F29" s="8"/>
       <c r="G29" s="8"/>
@@ -3636,13 +3714,13 @@
         <v>130</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="D30" s="8" t="s">
         <v>282</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F30" s="8"/>
       <c r="G30" s="8"/>
@@ -3667,13 +3745,13 @@
         <v>47</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="D31" s="8" t="s">
         <v>48</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F31" s="8"/>
       <c r="G31" s="8"/>
@@ -3698,13 +3776,13 @@
         <v>49</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="D32" s="8" t="s">
         <v>50</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F32" s="8"/>
       <c r="G32" s="8"/>
@@ -3729,13 +3807,13 @@
         <v>51</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>52</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F33" s="8"/>
       <c r="G33" s="8"/>
@@ -3760,13 +3838,13 @@
         <v>131</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="D34" s="8" t="s">
         <v>283</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F34" s="8"/>
       <c r="G34" s="8"/>
@@ -3791,13 +3869,13 @@
         <v>132</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="D35" s="8" t="s">
         <v>284</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F35" s="8"/>
       <c r="G35" s="8"/>
@@ -3822,13 +3900,13 @@
         <v>133</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D36" s="8" t="s">
         <v>285</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F36" s="8"/>
       <c r="G36" s="8"/>
@@ -3853,13 +3931,13 @@
         <v>55</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D37" s="8" t="s">
         <v>56</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F37" s="8"/>
       <c r="G37" s="8"/>
@@ -3884,13 +3962,13 @@
         <v>134</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D38" s="8" t="s">
         <v>286</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F38" s="8"/>
       <c r="G38" s="8"/>
@@ -3915,13 +3993,13 @@
         <v>135</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="D39" s="8" t="s">
         <v>287</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F39" s="8"/>
       <c r="G39" s="8"/>
@@ -3946,13 +4024,13 @@
         <v>136</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="D40" s="8" t="s">
         <v>288</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F40" s="8"/>
       <c r="G40" s="8"/>
@@ -3977,13 +4055,13 @@
         <v>137</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="D41" s="8" t="s">
         <v>289</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F41" s="8"/>
       <c r="G41" s="8"/>
@@ -4008,13 +4086,13 @@
         <v>57</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="D42" s="8" t="s">
         <v>58</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F42" s="8"/>
       <c r="G42" s="8"/>
@@ -4039,13 +4117,13 @@
         <v>138</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D43" s="8" t="s">
         <v>290</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F43" s="8"/>
       <c r="G43" s="8"/>
@@ -4070,13 +4148,13 @@
         <v>139</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="D44" s="8" t="s">
         <v>291</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>
@@ -4101,13 +4179,13 @@
         <v>140</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="D45" s="8" t="s">
         <v>292</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
@@ -4132,13 +4210,13 @@
         <v>141</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="D46" s="8" t="s">
         <v>292</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F46" s="8"/>
       <c r="G46" s="8"/>
@@ -4163,13 +4241,13 @@
         <v>142</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="D47" s="8" t="s">
         <v>293</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
@@ -4194,13 +4272,13 @@
         <v>143</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="D48" s="8" t="s">
         <v>294</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F48" s="8"/>
       <c r="G48" s="8"/>
@@ -4225,13 +4303,13 @@
         <v>59</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="D49" s="8" t="s">
         <v>60</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F49" s="8"/>
       <c r="G49" s="8"/>
@@ -4256,13 +4334,13 @@
         <v>61</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D50" s="8" t="s">
         <v>62</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
@@ -4287,13 +4365,13 @@
         <v>75</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D51" s="8" t="s">
         <v>62</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F51" s="8"/>
       <c r="G51" s="8"/>
@@ -4318,13 +4396,13 @@
         <v>144</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D52" s="8" t="s">
         <v>295</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F52" s="8"/>
       <c r="G52" s="8"/>
@@ -4349,13 +4427,13 @@
         <v>145</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D53" s="8" t="s">
         <v>296</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F53" s="8"/>
       <c r="G53" s="8"/>
@@ -4380,13 +4458,13 @@
         <v>146</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="D54" s="8" t="s">
         <v>297</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F54" s="8"/>
       <c r="G54" s="8"/>
@@ -4411,13 +4489,13 @@
         <v>63</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="D55" s="8" t="s">
         <v>64</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F55" s="8"/>
       <c r="G55" s="8"/>
@@ -4442,13 +4520,13 @@
         <v>147</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="D56" s="8" t="s">
         <v>298</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F56" s="8"/>
       <c r="G56" s="8"/>
@@ -4473,13 +4551,13 @@
         <v>148</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="D57" s="8" t="s">
         <v>299</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F57" s="8"/>
       <c r="G57" s="8"/>
@@ -4504,13 +4582,13 @@
         <v>149</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="D58" s="8" t="s">
         <v>300</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F58" s="8"/>
       <c r="G58" s="8"/>
@@ -4535,13 +4613,13 @@
         <v>150</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="D59" s="8" t="s">
         <v>301</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F59" s="8"/>
       <c r="G59" s="8"/>
@@ -4566,13 +4644,13 @@
         <v>151</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="D60" s="8" t="s">
         <v>302</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F60" s="8"/>
       <c r="G60" s="8"/>
@@ -4597,13 +4675,13 @@
         <v>65</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="D61" s="8" t="s">
         <v>66</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F61" s="8"/>
       <c r="G61" s="8"/>
@@ -4628,13 +4706,13 @@
         <v>105</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D62" s="8" t="s">
         <v>66</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F62" s="8"/>
       <c r="G62" s="8"/>
@@ -4659,13 +4737,13 @@
         <v>152</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="D63" s="8" t="s">
         <v>303</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F63" s="8"/>
       <c r="G63" s="8"/>
@@ -4690,13 +4768,13 @@
         <v>67</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D64" s="8" t="s">
         <v>68</v>
       </c>
       <c r="E64" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F64" s="8"/>
       <c r="G64" s="8"/>
@@ -4721,13 +4799,13 @@
         <v>153</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="D65" s="8" t="s">
         <v>304</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F65" s="8"/>
       <c r="G65" s="8"/>
@@ -4752,13 +4830,13 @@
         <v>154</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="D66" s="8" t="s">
         <v>305</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F66" s="8"/>
       <c r="G66" s="8"/>
@@ -4783,13 +4861,13 @@
         <v>155</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="D67" s="8" t="s">
         <v>306</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F67" s="8"/>
       <c r="G67" s="8"/>
@@ -4814,13 +4892,13 @@
         <v>69</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D68" s="8" t="s">
         <v>70</v>
       </c>
       <c r="E68" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F68" s="8"/>
       <c r="G68" s="8"/>
@@ -4845,13 +4923,13 @@
         <v>156</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="D69" s="8" t="s">
         <v>70</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F69" s="8"/>
       <c r="G69" s="8"/>
@@ -4876,13 +4954,13 @@
         <v>157</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="D70" s="8" t="s">
         <v>307</v>
       </c>
       <c r="E70" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F70" s="8"/>
       <c r="G70" s="8"/>
@@ -4907,13 +4985,13 @@
         <v>71</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="D71" s="8" t="s">
         <v>72</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F71" s="8"/>
       <c r="G71" s="8"/>
@@ -4938,13 +5016,13 @@
         <v>158</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="D72" s="8" t="s">
         <v>308</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F72" s="8"/>
       <c r="G72" s="8"/>
@@ -4969,13 +5047,13 @@
         <v>159</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="D73" s="8" t="s">
         <v>309</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F73" s="8"/>
       <c r="G73" s="8"/>
@@ -5000,13 +5078,13 @@
         <v>160</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D74" s="8" t="s">
         <v>310</v>
       </c>
       <c r="E74" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F74" s="8"/>
       <c r="G74" s="8"/>
@@ -5031,13 +5109,13 @@
         <v>161</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="D75" s="8" t="s">
         <v>311</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F75" s="8"/>
       <c r="G75" s="8"/>
@@ -5062,13 +5140,13 @@
         <v>162</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D76" s="8" t="s">
         <v>312</v>
       </c>
       <c r="E76" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F76" s="8"/>
       <c r="G76" s="8"/>
@@ -5093,13 +5171,13 @@
         <v>163</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="D77" s="8" t="s">
         <v>313</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F77" s="8"/>
       <c r="G77" s="8"/>
@@ -5124,13 +5202,13 @@
         <v>164</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D78" s="8" t="s">
         <v>314</v>
       </c>
       <c r="E78" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F78" s="8"/>
       <c r="G78" s="8"/>
@@ -5155,13 +5233,13 @@
         <v>165</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="D79" s="8" t="s">
         <v>315</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F79" s="8"/>
       <c r="G79" s="8"/>
@@ -5186,13 +5264,13 @@
         <v>166</v>
       </c>
       <c r="C80" s="8" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="D80" s="8" t="s">
         <v>316</v>
       </c>
       <c r="E80" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F80" s="8"/>
       <c r="G80" s="8"/>
@@ -5217,13 +5295,13 @@
         <v>167</v>
       </c>
       <c r="C81" s="8" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="D81" s="8" t="s">
         <v>317</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F81" s="8"/>
       <c r="G81" s="8"/>
@@ -5248,13 +5326,13 @@
         <v>168</v>
       </c>
       <c r="C82" s="8" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="D82" s="8" t="s">
         <v>318</v>
       </c>
       <c r="E82" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F82" s="8"/>
       <c r="G82" s="8"/>
@@ -5279,13 +5357,13 @@
         <v>169</v>
       </c>
       <c r="C83" s="8" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="D83" s="8" t="s">
         <v>319</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F83" s="8"/>
       <c r="G83" s="8"/>
@@ -5310,13 +5388,13 @@
         <v>170</v>
       </c>
       <c r="C84" s="8" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="D84" s="8" t="s">
         <v>320</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F84" s="8"/>
       <c r="G84" s="8"/>
@@ -5341,13 +5419,13 @@
         <v>171</v>
       </c>
       <c r="C85" s="8" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="D85" s="8" t="s">
         <v>321</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F85" s="8"/>
       <c r="G85" s="8"/>
@@ -5372,13 +5450,13 @@
         <v>172</v>
       </c>
       <c r="C86" s="8" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="D86" s="8" t="s">
         <v>322</v>
       </c>
       <c r="E86" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F86" s="8"/>
       <c r="G86" s="8"/>
@@ -5403,13 +5481,13 @@
         <v>173</v>
       </c>
       <c r="C87" s="8" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="D87" s="8" t="s">
         <v>323</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F87" s="8"/>
       <c r="G87" s="8"/>
@@ -5434,13 +5512,13 @@
         <v>174</v>
       </c>
       <c r="C88" s="8" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D88" s="8" t="s">
         <v>324</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F88" s="8"/>
       <c r="G88" s="8"/>
@@ -5465,13 +5543,13 @@
         <v>175</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D89" s="8" t="s">
         <v>325</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F89" s="8"/>
       <c r="G89" s="8"/>
@@ -5496,13 +5574,13 @@
         <v>176</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D90" s="8" t="s">
         <v>326</v>
       </c>
       <c r="E90" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F90" s="8"/>
       <c r="G90" s="8"/>
@@ -5527,13 +5605,13 @@
         <v>177</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="D91" s="8" t="s">
         <v>327</v>
       </c>
       <c r="E91" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F91" s="8"/>
       <c r="G91" s="8"/>
@@ -5558,13 +5636,13 @@
         <v>178</v>
       </c>
       <c r="C92" s="8" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="D92" s="8" t="s">
         <v>328</v>
       </c>
       <c r="E92" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F92" s="8"/>
       <c r="G92" s="8"/>
@@ -5589,13 +5667,13 @@
         <v>179</v>
       </c>
       <c r="C93" s="8" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="D93" s="8" t="s">
         <v>329</v>
       </c>
       <c r="E93" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F93" s="8"/>
       <c r="G93" s="8"/>
@@ -5620,13 +5698,13 @@
         <v>180</v>
       </c>
       <c r="C94" s="8" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="D94" s="8" t="s">
         <v>330</v>
       </c>
       <c r="E94" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F94" s="8"/>
       <c r="G94" s="8"/>
@@ -5651,13 +5729,13 @@
         <v>181</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="D95" s="8" t="s">
         <v>331</v>
       </c>
       <c r="E95" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F95" s="8"/>
       <c r="G95" s="8"/>
@@ -5682,13 +5760,13 @@
         <v>182</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="D96" s="8" t="s">
         <v>332</v>
       </c>
       <c r="E96" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F96" s="8"/>
       <c r="G96" s="8"/>
@@ -5713,13 +5791,13 @@
         <v>183</v>
       </c>
       <c r="C97" s="8" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="D97" s="8" t="s">
         <v>333</v>
       </c>
       <c r="E97" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F97" s="8"/>
       <c r="G97" s="8"/>
@@ -5744,13 +5822,13 @@
         <v>184</v>
       </c>
       <c r="C98" s="8" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="D98" s="8" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="E98" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F98" s="8"/>
       <c r="G98" s="8"/>
@@ -5775,13 +5853,13 @@
         <v>185</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="D99" s="8" t="s">
         <v>334</v>
       </c>
       <c r="E99" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F99" s="8"/>
       <c r="G99" s="8"/>
@@ -5806,13 +5884,13 @@
         <v>186</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="D100" s="8" t="s">
         <v>335</v>
       </c>
       <c r="E100" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F100" s="8"/>
       <c r="G100" s="8"/>
@@ -5837,13 +5915,13 @@
         <v>187</v>
       </c>
       <c r="C101" s="8" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="D101" s="8" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F101" s="8"/>
       <c r="G101" s="8"/>
@@ -5868,13 +5946,13 @@
         <v>188</v>
       </c>
       <c r="C102" s="8" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="D102" s="8" t="s">
         <v>336</v>
       </c>
       <c r="E102" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F102" s="8"/>
       <c r="G102" s="8"/>
@@ -5899,13 +5977,13 @@
         <v>189</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="D103" s="8" t="s">
         <v>337</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F103" s="8"/>
       <c r="G103" s="8"/>
@@ -5930,13 +6008,13 @@
         <v>190</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="D104" s="8" t="s">
         <v>338</v>
       </c>
       <c r="E104" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F104" s="8"/>
       <c r="G104" s="8"/>
@@ -5961,13 +6039,13 @@
         <v>191</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D105" s="8" t="s">
         <v>339</v>
       </c>
       <c r="E105" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F105" s="8"/>
       <c r="G105" s="8"/>
@@ -5992,13 +6070,13 @@
         <v>192</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="D106" s="8" t="s">
         <v>340</v>
       </c>
       <c r="E106" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F106" s="8"/>
       <c r="G106" s="8"/>
@@ -6023,13 +6101,13 @@
         <v>193</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="D107" s="8" t="s">
         <v>341</v>
       </c>
       <c r="E107" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F107" s="8"/>
       <c r="G107" s="8"/>
@@ -6054,13 +6132,13 @@
         <v>194</v>
       </c>
       <c r="C108" s="8" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="D108" s="8" t="s">
         <v>342</v>
       </c>
       <c r="E108" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F108" s="8"/>
       <c r="G108" s="8"/>
@@ -6085,13 +6163,13 @@
         <v>195</v>
       </c>
       <c r="C109" s="8" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="D109" s="8" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="E109" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F109" s="8"/>
       <c r="G109" s="8"/>
@@ -6116,13 +6194,13 @@
         <v>196</v>
       </c>
       <c r="C110" s="8" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="D110" s="8" t="s">
         <v>343</v>
       </c>
       <c r="E110" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F110" s="8"/>
       <c r="G110" s="8"/>
@@ -6147,13 +6225,13 @@
         <v>197</v>
       </c>
       <c r="C111" s="8" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="D111" s="8" t="s">
         <v>344</v>
       </c>
       <c r="E111" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F111" s="8"/>
       <c r="G111" s="8"/>
@@ -6178,13 +6256,13 @@
         <v>198</v>
       </c>
       <c r="C112" s="8" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="D112" s="8" t="s">
         <v>345</v>
       </c>
       <c r="E112" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F112" s="8"/>
       <c r="G112" s="8"/>
@@ -6209,13 +6287,13 @@
         <v>199</v>
       </c>
       <c r="C113" s="8" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="D113" s="8" t="s">
         <v>346</v>
       </c>
       <c r="E113" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F113" s="8"/>
       <c r="G113" s="8"/>
@@ -6240,13 +6318,13 @@
         <v>200</v>
       </c>
       <c r="C114" s="8" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="D114" s="8" t="s">
         <v>347</v>
       </c>
       <c r="E114" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F114" s="8"/>
       <c r="G114" s="8"/>
@@ -6271,13 +6349,13 @@
         <v>201</v>
       </c>
       <c r="C115" s="8" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="D115" s="8" t="s">
         <v>348</v>
       </c>
       <c r="E115" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F115" s="8"/>
       <c r="G115" s="8"/>
@@ -6302,13 +6380,13 @@
         <v>202</v>
       </c>
       <c r="C116" s="8" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="D116" s="8" t="s">
         <v>349</v>
       </c>
       <c r="E116" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F116" s="8"/>
       <c r="G116" s="8"/>
@@ -6333,13 +6411,13 @@
         <v>203</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="D117" s="8" t="s">
         <v>350</v>
       </c>
       <c r="E117" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F117" s="8"/>
       <c r="G117" s="8"/>
@@ -6364,13 +6442,13 @@
         <v>204</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="D118" s="8" t="s">
         <v>351</v>
       </c>
       <c r="E118" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F118" s="8"/>
       <c r="G118" s="8"/>
@@ -6395,13 +6473,13 @@
         <v>205</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="D119" s="8" t="s">
         <v>352</v>
       </c>
       <c r="E119" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F119" s="8"/>
       <c r="G119" s="8"/>
@@ -6426,13 +6504,13 @@
         <v>206</v>
       </c>
       <c r="C120" s="8" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="D120" s="8" t="s">
         <v>353</v>
       </c>
       <c r="E120" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F120" s="8"/>
       <c r="G120" s="8"/>
@@ -6457,13 +6535,13 @@
         <v>207</v>
       </c>
       <c r="C121" s="8" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="D121" s="8" t="s">
         <v>354</v>
       </c>
       <c r="E121" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F121" s="8"/>
       <c r="G121" s="8"/>
@@ -6488,13 +6566,13 @@
         <v>208</v>
       </c>
       <c r="C122" s="8" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="D122" s="8" t="s">
         <v>355</v>
       </c>
       <c r="E122" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F122" s="8"/>
       <c r="G122" s="8"/>
@@ -6519,13 +6597,13 @@
         <v>81</v>
       </c>
       <c r="C123" s="8" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="D123" s="8" t="s">
         <v>82</v>
       </c>
       <c r="E123" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F123" s="8"/>
       <c r="G123" s="8"/>
@@ -6550,13 +6628,13 @@
         <v>209</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="D124" s="8" t="s">
         <v>356</v>
       </c>
       <c r="E124" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F124" s="8"/>
       <c r="G124" s="8"/>
@@ -6581,13 +6659,13 @@
         <v>83</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="D125" s="8" t="s">
         <v>84</v>
       </c>
       <c r="E125" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F125" s="8"/>
       <c r="G125" s="8"/>
@@ -6612,13 +6690,13 @@
         <v>85</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="D126" s="8" t="s">
         <v>86</v>
       </c>
       <c r="E126" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F126" s="8"/>
       <c r="G126" s="8"/>
@@ -6643,13 +6721,13 @@
         <v>210</v>
       </c>
       <c r="C127" s="8" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="D127" s="8" t="s">
         <v>357</v>
       </c>
       <c r="E127" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F127" s="8"/>
       <c r="G127" s="8"/>
@@ -6674,13 +6752,13 @@
         <v>87</v>
       </c>
       <c r="C128" s="8" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="D128" s="8" t="s">
         <v>88</v>
       </c>
       <c r="E128" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F128" s="8"/>
       <c r="G128" s="8"/>
@@ -6705,13 +6783,13 @@
         <v>211</v>
       </c>
       <c r="C129" s="8" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="D129" s="8" t="s">
         <v>358</v>
       </c>
       <c r="E129" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F129" s="8"/>
       <c r="G129" s="8"/>
@@ -6736,13 +6814,13 @@
         <v>212</v>
       </c>
       <c r="C130" s="8" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="D130" s="8" t="s">
         <v>359</v>
       </c>
       <c r="E130" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F130" s="8"/>
       <c r="G130" s="8"/>
@@ -6767,13 +6845,13 @@
         <v>213</v>
       </c>
       <c r="C131" s="8" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="D131" s="8" t="s">
         <v>360</v>
       </c>
       <c r="E131" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F131" s="8"/>
       <c r="G131" s="8"/>
@@ -6798,13 +6876,13 @@
         <v>214</v>
       </c>
       <c r="C132" s="8" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="D132" s="8" t="s">
         <v>361</v>
       </c>
       <c r="E132" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F132" s="8"/>
       <c r="G132" s="8"/>
@@ -6829,13 +6907,13 @@
         <v>215</v>
       </c>
       <c r="C133" s="8" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="D133" s="8" t="s">
         <v>362</v>
       </c>
       <c r="E133" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F133" s="8"/>
       <c r="G133" s="8"/>
@@ -6860,13 +6938,13 @@
         <v>216</v>
       </c>
       <c r="C134" s="8" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="D134" s="8" t="s">
         <v>363</v>
       </c>
       <c r="E134" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F134" s="8"/>
       <c r="G134" s="8"/>
@@ -6891,13 +6969,13 @@
         <v>217</v>
       </c>
       <c r="C135" s="8" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="D135" s="8" t="s">
         <v>364</v>
       </c>
       <c r="E135" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F135" s="8"/>
       <c r="G135" s="8"/>
@@ -6922,13 +7000,13 @@
         <v>218</v>
       </c>
       <c r="C136" s="8" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="D136" s="8" t="s">
         <v>365</v>
       </c>
       <c r="E136" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F136" s="8"/>
       <c r="G136" s="8"/>
@@ -6953,13 +7031,13 @@
         <v>219</v>
       </c>
       <c r="C137" s="8" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="D137" s="8" t="s">
         <v>366</v>
       </c>
       <c r="E137" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F137" s="8"/>
       <c r="G137" s="8"/>
@@ -6984,13 +7062,13 @@
         <v>89</v>
       </c>
       <c r="C138" s="8" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="D138" s="8" t="s">
         <v>90</v>
       </c>
       <c r="E138" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F138" s="8"/>
       <c r="G138" s="8"/>
@@ -7015,13 +7093,13 @@
         <v>220</v>
       </c>
       <c r="C139" s="8" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="D139" s="8" t="s">
         <v>367</v>
       </c>
       <c r="E139" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F139" s="8"/>
       <c r="G139" s="8"/>
@@ -7046,13 +7124,13 @@
         <v>221</v>
       </c>
       <c r="C140" s="8" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="D140" s="8" t="s">
         <v>368</v>
       </c>
       <c r="E140" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F140" s="8"/>
       <c r="G140" s="8"/>
@@ -7077,13 +7155,13 @@
         <v>91</v>
       </c>
       <c r="C141" s="8" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="D141" s="8" t="s">
         <v>92</v>
       </c>
       <c r="E141" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F141" s="8"/>
       <c r="G141" s="8"/>
@@ -7108,13 +7186,13 @@
         <v>222</v>
       </c>
       <c r="C142" s="8" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="D142" s="8" t="s">
         <v>369</v>
       </c>
       <c r="E142" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F142" s="8"/>
       <c r="G142" s="8"/>
@@ -7139,13 +7217,13 @@
         <v>223</v>
       </c>
       <c r="C143" s="8" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="D143" s="8" t="s">
         <v>370</v>
       </c>
       <c r="E143" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F143" s="8"/>
       <c r="G143" s="8"/>
@@ -7170,13 +7248,13 @@
         <v>224</v>
       </c>
       <c r="C144" s="8" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="D144" s="8" t="s">
         <v>371</v>
       </c>
       <c r="E144" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F144" s="8"/>
       <c r="G144" s="8"/>
@@ -7201,13 +7279,13 @@
         <v>225</v>
       </c>
       <c r="C145" s="8" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="D145" s="8" t="s">
         <v>372</v>
       </c>
       <c r="E145" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F145" s="8"/>
       <c r="G145" s="8"/>
@@ -7232,13 +7310,13 @@
         <v>226</v>
       </c>
       <c r="C146" s="8" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="D146" s="8" t="s">
         <v>373</v>
       </c>
       <c r="E146" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F146" s="8"/>
       <c r="G146" s="8"/>
@@ -7263,13 +7341,13 @@
         <v>227</v>
       </c>
       <c r="C147" s="8" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="D147" s="8" t="s">
         <v>374</v>
       </c>
       <c r="E147" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F147" s="8"/>
       <c r="G147" s="8"/>
@@ -7294,13 +7372,13 @@
         <v>228</v>
       </c>
       <c r="C148" s="8" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="D148" s="8" t="s">
-        <v>375</v>
+        <v>347</v>
       </c>
       <c r="E148" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F148" s="8"/>
       <c r="G148" s="8"/>
@@ -7325,13 +7403,13 @@
         <v>229</v>
       </c>
       <c r="C149" s="8" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="D149" s="8" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E149" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F149" s="8"/>
       <c r="G149" s="8"/>
@@ -7356,13 +7434,13 @@
         <v>76</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="D150" s="8" t="s">
         <v>77</v>
       </c>
       <c r="E150" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F150" s="8"/>
       <c r="G150" s="8"/>
@@ -7387,13 +7465,13 @@
         <v>78</v>
       </c>
       <c r="C151" s="8" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="D151" s="8" t="s">
         <v>79</v>
       </c>
       <c r="E151" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F151" s="8"/>
       <c r="G151" s="8"/>
@@ -7418,13 +7496,13 @@
         <v>73</v>
       </c>
       <c r="C152" s="8" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="D152" s="8" t="s">
         <v>74</v>
       </c>
       <c r="E152" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F152" s="8"/>
       <c r="G152" s="8"/>
@@ -7449,13 +7527,13 @@
         <v>231</v>
       </c>
       <c r="C153" s="8" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="D153" s="8" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E153" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F153" s="8"/>
       <c r="G153" s="8"/>
@@ -7480,13 +7558,13 @@
         <v>230</v>
       </c>
       <c r="C154" s="8" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="D154" s="8" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E154" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F154" s="8"/>
       <c r="G154" s="8"/>
@@ -7511,13 +7589,13 @@
         <v>232</v>
       </c>
       <c r="C155" s="8" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="D155" s="8" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E155" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F155" s="8"/>
       <c r="G155" s="8"/>
@@ -7542,13 +7620,13 @@
         <v>233</v>
       </c>
       <c r="C156" s="8" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="D156" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E156" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F156" s="8"/>
       <c r="G156" s="8"/>
@@ -7573,13 +7651,13 @@
         <v>234</v>
       </c>
       <c r="C157" s="8" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="D157" s="8" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E157" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F157" s="8"/>
       <c r="G157" s="8"/>
@@ -7604,13 +7682,13 @@
         <v>235</v>
       </c>
       <c r="C158" s="8" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="D158" s="8" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E158" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F158" s="8"/>
       <c r="G158" s="8"/>
@@ -7635,13 +7713,13 @@
         <v>106</v>
       </c>
       <c r="C159" s="8" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="D159" s="8" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E159" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F159" s="8"/>
       <c r="G159" s="8"/>
@@ -7666,13 +7744,13 @@
         <v>236</v>
       </c>
       <c r="C160" s="8" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="D160" s="8" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E160" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F160" s="8"/>
       <c r="G160" s="8"/>
@@ -7697,13 +7775,13 @@
         <v>237</v>
       </c>
       <c r="C161" s="8" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="D161" s="8" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E161" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F161" s="8"/>
       <c r="G161" s="8"/>
@@ -7728,13 +7806,13 @@
         <v>53</v>
       </c>
       <c r="C162" s="8" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="D162" s="8" t="s">
         <v>54</v>
       </c>
       <c r="E162" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F162" s="8"/>
       <c r="G162" s="8"/>
@@ -7759,13 +7837,13 @@
         <v>98</v>
       </c>
       <c r="C163" s="8" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="D163" s="8" t="s">
         <v>99</v>
       </c>
       <c r="E163" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F163" s="8"/>
       <c r="G163" s="8"/>
@@ -7790,13 +7868,13 @@
         <v>100</v>
       </c>
       <c r="C164" s="8" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="D164" s="8" t="s">
         <v>101</v>
       </c>
       <c r="E164" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F164" s="8"/>
       <c r="G164" s="8"/>
@@ -7821,13 +7899,13 @@
         <v>238</v>
       </c>
       <c r="C165" s="8" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="D165" s="8" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="E165" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F165" s="8"/>
       <c r="G165" s="8"/>
@@ -7852,13 +7930,13 @@
         <v>102</v>
       </c>
       <c r="C166" s="8" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D166" s="8" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="E166" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F166" s="8"/>
       <c r="G166" s="8"/>
@@ -7883,13 +7961,13 @@
         <v>239</v>
       </c>
       <c r="C167" s="8" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="D167" s="8" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E167" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F167" s="8"/>
       <c r="G167" s="8"/>
@@ -7914,13 +7992,13 @@
         <v>240</v>
       </c>
       <c r="C168" s="8" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="D168" s="8" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="E168" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F168" s="8"/>
       <c r="G168" s="8"/>
@@ -7945,13 +8023,13 @@
         <v>241</v>
       </c>
       <c r="C169" s="8" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="D169" s="8" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="E169" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F169" s="8"/>
       <c r="G169" s="8"/>
@@ -7976,13 +8054,13 @@
         <v>242</v>
       </c>
       <c r="C170" s="8" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="D170" s="8" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="E170" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F170" s="8"/>
       <c r="G170" s="8"/>
@@ -8007,13 +8085,13 @@
         <v>243</v>
       </c>
       <c r="C171" s="8" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="D171" s="8" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="E171" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F171" s="8"/>
       <c r="G171" s="8"/>
@@ -8038,13 +8116,13 @@
         <v>93</v>
       </c>
       <c r="C172" s="8" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="D172" s="8" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="E172" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F172" s="8"/>
       <c r="G172" s="8"/>
@@ -8069,13 +8147,13 @@
         <v>244</v>
       </c>
       <c r="C173" s="8" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="D173" s="8" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="E173" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F173" s="8"/>
       <c r="G173" s="8"/>
@@ -8100,13 +8178,13 @@
         <v>94</v>
       </c>
       <c r="C174" s="8" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="D174" s="8" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="E174" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F174" s="8"/>
       <c r="G174" s="8"/>
@@ -8131,13 +8209,13 @@
         <v>245</v>
       </c>
       <c r="C175" s="8" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="D175" s="8" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="E175" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F175" s="8"/>
       <c r="G175" s="8"/>
@@ -8162,13 +8240,13 @@
         <v>246</v>
       </c>
       <c r="C176" s="8" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="D176" s="8" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="E176" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F176" s="8"/>
       <c r="G176" s="8"/>
@@ -8193,13 +8271,13 @@
         <v>247</v>
       </c>
       <c r="C177" s="8" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="D177" s="8" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="E177" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F177" s="8"/>
       <c r="G177" s="8"/>
@@ -8224,13 +8302,13 @@
         <v>95</v>
       </c>
       <c r="C178" s="8" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="D178" s="8" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="E178" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F178" s="8"/>
       <c r="G178" s="8"/>
@@ -8255,13 +8333,13 @@
         <v>96</v>
       </c>
       <c r="C179" s="8" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="D179" s="8" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="E179" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F179" s="8"/>
       <c r="G179" s="8"/>
@@ -8286,13 +8364,13 @@
         <v>248</v>
       </c>
       <c r="C180" s="8" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="D180" s="8" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="E180" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F180" s="8"/>
       <c r="G180" s="8"/>
@@ -8317,13 +8395,13 @@
         <v>249</v>
       </c>
       <c r="C181" s="8" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="D181" s="8" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="E181" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F181" s="8"/>
       <c r="G181" s="8"/>
@@ -8348,13 +8426,13 @@
         <v>250</v>
       </c>
       <c r="C182" s="8" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="D182" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="E182" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F182" s="8"/>
       <c r="G182" s="8"/>
@@ -8379,13 +8457,13 @@
         <v>97</v>
       </c>
       <c r="C183" s="8" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="D183" s="8" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="E183" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F183" s="8"/>
       <c r="G183" s="8"/>
@@ -8410,13 +8488,13 @@
         <v>251</v>
       </c>
       <c r="C184" s="8" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="D184" s="8" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E184" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F184" s="8"/>
       <c r="G184" s="8"/>
@@ -8441,13 +8519,13 @@
         <v>252</v>
       </c>
       <c r="C185" s="8" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="D185" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="E185" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F185" s="8"/>
       <c r="G185" s="8"/>
@@ -8472,13 +8550,13 @@
         <v>253</v>
       </c>
       <c r="C186" s="8" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="D186" s="8" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E186" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F186" s="8"/>
       <c r="G186" s="8"/>
@@ -8503,13 +8581,13 @@
         <v>103</v>
       </c>
       <c r="C187" s="8" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="D187" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="E187" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F187" s="8"/>
       <c r="G187" s="8"/>
@@ -8534,13 +8612,13 @@
         <v>254</v>
       </c>
       <c r="C188" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="D188" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="E188" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F188" s="8"/>
       <c r="G188" s="8"/>
@@ -8565,13 +8643,13 @@
         <v>255</v>
       </c>
       <c r="C189" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="D189" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="E189" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F189" s="8"/>
       <c r="G189" s="8"/>
@@ -8596,13 +8674,13 @@
         <v>104</v>
       </c>
       <c r="C190" s="8" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="D190" s="8" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="E190" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F190" s="8"/>
       <c r="G190" s="8"/>
@@ -8627,13 +8705,13 @@
         <v>256</v>
       </c>
       <c r="C191" s="8" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="D191" s="8" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="E191" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F191" s="8"/>
       <c r="G191" s="8"/>
@@ -8658,13 +8736,13 @@
         <v>257</v>
       </c>
       <c r="C192" s="8" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="D192" s="8" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="E192" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F192" s="8"/>
       <c r="G192" s="8"/>
@@ -8689,13 +8767,13 @@
         <v>258</v>
       </c>
       <c r="C193" s="8" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="D193" s="8" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E193" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F193" s="8"/>
       <c r="G193" s="8"/>
@@ -8720,13 +8798,13 @@
         <v>259</v>
       </c>
       <c r="C194" s="8" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="D194" s="8" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E194" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F194" s="8"/>
       <c r="G194" s="8"/>
@@ -8751,13 +8829,13 @@
         <v>107</v>
       </c>
       <c r="C195" s="8" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="D195" s="8" t="s">
         <v>108</v>
       </c>
       <c r="E195" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F195" s="8"/>
       <c r="G195" s="8"/>
@@ -8782,13 +8860,13 @@
         <v>260</v>
       </c>
       <c r="C196" s="8" t="s">
-        <v>622</v>
-      </c>
-      <c r="D196" s="8" t="s">
-        <v>388</v>
+        <v>620</v>
+      </c>
+      <c r="D196" s="11" t="s">
+        <v>722</v>
       </c>
       <c r="E196" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F196" s="8"/>
       <c r="G196" s="8"/>
@@ -8813,13 +8891,13 @@
         <v>261</v>
       </c>
       <c r="C197" s="8" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="D197" s="8" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="E197" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F197" s="8"/>
       <c r="G197" s="8"/>
@@ -8844,13 +8922,13 @@
         <v>262</v>
       </c>
       <c r="C198" s="8" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="D198" s="8" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E198" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F198" s="8"/>
       <c r="G198" s="8"/>
@@ -8875,13 +8953,13 @@
         <v>263</v>
       </c>
       <c r="C199" s="8" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="D199" s="8" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="E199" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F199" s="8"/>
       <c r="G199" s="8"/>
@@ -8906,13 +8984,13 @@
         <v>264</v>
       </c>
       <c r="C200" s="8" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="D200" s="8" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="E200" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F200" s="8"/>
       <c r="G200" s="8"/>
@@ -8937,13 +9015,13 @@
         <v>265</v>
       </c>
       <c r="C201" s="8" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="D201" s="8" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="E201" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F201" s="8"/>
       <c r="G201" s="8"/>
@@ -8968,13 +9046,13 @@
         <v>109</v>
       </c>
       <c r="C202" s="8" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D202" s="8" t="s">
         <v>110</v>
       </c>
       <c r="E202" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F202" s="8"/>
       <c r="G202" s="8"/>
@@ -8999,13 +9077,13 @@
         <v>266</v>
       </c>
       <c r="C203" s="8" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="D203" s="8" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E203" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F203" s="8"/>
       <c r="G203" s="8"/>
@@ -9027,16 +9105,16 @@
         <v>4</v>
       </c>
       <c r="B204" s="8" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="C204" s="8" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="D204" s="8" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="E204" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F204" s="8"/>
       <c r="G204" s="8"/>
@@ -9058,16 +9136,16 @@
         <v>4</v>
       </c>
       <c r="B205" s="8" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="C205" s="8" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="D205" s="8" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E205" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F205" s="8"/>
       <c r="G205" s="8"/>
@@ -9092,13 +9170,13 @@
         <v>267</v>
       </c>
       <c r="C206" s="8" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="D206" s="8" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="E206" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F206" s="8"/>
       <c r="G206" s="8"/>
@@ -9123,13 +9201,13 @@
         <v>268</v>
       </c>
       <c r="C207" s="8" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="D207" s="8" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="E207" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F207" s="8"/>
       <c r="G207" s="8"/>
@@ -9154,13 +9232,13 @@
         <v>269</v>
       </c>
       <c r="C208" s="8" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="D208" s="8" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E208" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F208" s="8"/>
       <c r="G208" s="8"/>
@@ -9182,16 +9260,16 @@
         <v>4</v>
       </c>
       <c r="B209" s="8" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="C209" s="8" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="D209" s="8" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="E209" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F209" s="8"/>
       <c r="G209" s="8"/>
@@ -9213,16 +9291,16 @@
         <v>4</v>
       </c>
       <c r="B210" s="8" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="C210" s="8" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="D210" s="8" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="E210" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F210" s="8"/>
       <c r="G210" s="8"/>
@@ -9244,16 +9322,16 @@
         <v>4</v>
       </c>
       <c r="B211" s="8" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="C211" s="8" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="D211" s="8" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="E211" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F211" s="8"/>
       <c r="G211" s="8"/>
@@ -9278,13 +9356,13 @@
         <v>270</v>
       </c>
       <c r="C212" s="8" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="D212" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E212" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F212" s="8"/>
       <c r="G212" s="8"/>
@@ -9309,13 +9387,13 @@
         <v>271</v>
       </c>
       <c r="C213" s="8" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="D213" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="E213" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F213" s="8"/>
       <c r="G213" s="8"/>
@@ -9340,13 +9418,13 @@
         <v>272</v>
       </c>
       <c r="C214" s="8" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="D214" s="8" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E214" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F214" s="8"/>
       <c r="G214" s="8"/>
@@ -9371,13 +9449,13 @@
         <v>273</v>
       </c>
       <c r="C215" s="8" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="D215" s="8" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="E215" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F215" s="8"/>
       <c r="G215" s="8"/>
@@ -9402,13 +9480,13 @@
         <v>274</v>
       </c>
       <c r="C216" s="8" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="D216" s="8" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="E216" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F216" s="8"/>
       <c r="G216" s="8"/>
@@ -9430,16 +9508,16 @@
         <v>4</v>
       </c>
       <c r="B217" s="8" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="C217" s="8" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="D217" s="8" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E217" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F217" s="8"/>
       <c r="G217" s="8"/>
@@ -9461,16 +9539,16 @@
         <v>4</v>
       </c>
       <c r="B218" s="8" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="C218" s="8" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="D218" s="8" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="E218" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F218" s="8"/>
       <c r="G218" s="8"/>
@@ -9492,16 +9570,16 @@
         <v>4</v>
       </c>
       <c r="B219" s="8" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="C219" s="8" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="D219" s="8" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="E219" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F219" s="8"/>
       <c r="G219" s="8"/>
@@ -9523,16 +9601,16 @@
         <v>4</v>
       </c>
       <c r="B220" s="8" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="C220" s="8" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="D220" s="8" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="E220" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F220" s="8"/>
       <c r="G220" s="8"/>
@@ -9554,16 +9632,16 @@
         <v>4</v>
       </c>
       <c r="B221" s="8" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="C221" s="8" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="D221" s="8" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="E221" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F221" s="8"/>
       <c r="G221" s="8"/>
@@ -9585,16 +9663,16 @@
         <v>4</v>
       </c>
       <c r="B222" s="8" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="C222" s="8" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="D222" s="8" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="E222" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F222" s="8"/>
       <c r="G222" s="8"/>
@@ -9616,16 +9694,16 @@
         <v>4</v>
       </c>
       <c r="B223" s="8" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C223" s="8" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="D223" s="8" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E223" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F223" s="8"/>
       <c r="G223" s="8"/>
@@ -9647,16 +9725,16 @@
         <v>4</v>
       </c>
       <c r="B224" s="8" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="C224" s="8" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="D224" s="8" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="E224" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F224" s="8"/>
       <c r="G224" s="8"/>
@@ -9678,16 +9756,16 @@
         <v>4</v>
       </c>
       <c r="B225" s="8" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="C225" s="8" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="D225" s="8" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E225" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F225" s="8"/>
       <c r="G225" s="8"/>
@@ -9709,16 +9787,16 @@
         <v>4</v>
       </c>
       <c r="B226" s="8" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="C226" s="8" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="D226" s="8" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E226" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F226" s="8"/>
       <c r="G226" s="8"/>
@@ -9740,16 +9818,16 @@
         <v>4</v>
       </c>
       <c r="B227" s="8" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="C227" s="8" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="D227" s="8" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="E227" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F227" s="8"/>
       <c r="G227" s="8"/>
@@ -9771,16 +9849,16 @@
         <v>4</v>
       </c>
       <c r="B228" s="8" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="C228" s="8" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="D228" s="8" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="E228" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F228" s="8"/>
       <c r="G228" s="8"/>
@@ -9802,16 +9880,16 @@
         <v>4</v>
       </c>
       <c r="B229" s="8" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="C229" s="8" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="D229" s="8" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="E229" s="8" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F229" s="8"/>
       <c r="G229" s="8"/>
@@ -9833,16 +9911,16 @@
         <v>4</v>
       </c>
       <c r="B230" s="8" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="C230" s="8" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="D230" s="8" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="E230" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F230" s="8"/>
       <c r="G230" s="8"/>
@@ -9864,16 +9942,16 @@
         <v>4</v>
       </c>
       <c r="B231" s="8" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="C231" s="8" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="D231" s="8" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="E231" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F231" s="8"/>
       <c r="G231" s="8"/>
@@ -9895,16 +9973,16 @@
         <v>4</v>
       </c>
       <c r="B232" s="8" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="C232" s="8" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="D232" s="8" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="E232" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F232" s="8"/>
       <c r="G232" s="8"/>
@@ -9926,16 +10004,16 @@
         <v>4</v>
       </c>
       <c r="B233" s="8" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="C233" s="8" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="D233" s="8" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="E233" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F233" s="8"/>
       <c r="G233" s="8"/>
@@ -9957,16 +10035,16 @@
         <v>80</v>
       </c>
       <c r="B234" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="C234" s="8" t="s">
+        <v>659</v>
+      </c>
+      <c r="D234" s="8" t="s">
         <v>660</v>
       </c>
-      <c r="C234" s="8" t="s">
-        <v>661</v>
-      </c>
-      <c r="D234" s="8" t="s">
-        <v>662</v>
-      </c>
       <c r="E234" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F234" s="8"/>
       <c r="G234" s="8"/>
@@ -9988,16 +10066,16 @@
         <v>80</v>
       </c>
       <c r="B235" s="8" t="s">
+        <v>661</v>
+      </c>
+      <c r="C235" s="8" t="s">
+        <v>662</v>
+      </c>
+      <c r="D235" s="8" t="s">
         <v>663</v>
       </c>
-      <c r="C235" s="8" t="s">
-        <v>664</v>
-      </c>
-      <c r="D235" s="8" t="s">
-        <v>665</v>
-      </c>
       <c r="E235" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F235" s="8"/>
       <c r="G235" s="8"/>
@@ -10019,16 +10097,16 @@
         <v>80</v>
       </c>
       <c r="B236" s="8" t="s">
+        <v>664</v>
+      </c>
+      <c r="C236" s="8" t="s">
+        <v>665</v>
+      </c>
+      <c r="D236" s="8" t="s">
         <v>666</v>
       </c>
-      <c r="C236" s="8" t="s">
-        <v>667</v>
-      </c>
-      <c r="D236" s="8" t="s">
-        <v>668</v>
-      </c>
       <c r="E236" s="8" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F236" s="8"/>
       <c r="G236" s="8"/>
@@ -10050,19 +10128,212 @@
         <v>80</v>
       </c>
       <c r="B237" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="C237" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="D237" s="8" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="E237" s="10" t="s">
-        <v>427</v>
-      </c>
+        <v>425</v>
+      </c>
+      <c r="F237" s="8"/>
+      <c r="G237" s="8"/>
+    </row>
+    <row r="238" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A238" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B238" s="8" t="s">
+        <v>723</v>
+      </c>
+      <c r="C238" s="8" t="s">
+        <v>724</v>
+      </c>
+      <c r="D238" s="8" t="s">
+        <v>725</v>
+      </c>
+      <c r="E238" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F238" s="8"/>
+      <c r="G238" s="8"/>
+    </row>
+    <row r="239" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A239" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B239" s="8" t="s">
+        <v>726</v>
+      </c>
+      <c r="C239" s="8" t="s">
+        <v>727</v>
+      </c>
+      <c r="D239" s="8" t="s">
+        <v>728</v>
+      </c>
+      <c r="E239" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F239" s="8"/>
+      <c r="G239" s="8"/>
+    </row>
+    <row r="240" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A240" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B240" s="8" t="s">
+        <v>729</v>
+      </c>
+      <c r="C240" s="8" t="s">
+        <v>730</v>
+      </c>
+      <c r="D240" s="8" t="s">
+        <v>731</v>
+      </c>
+      <c r="E240" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F240" s="8"/>
+      <c r="G240" s="8"/>
+    </row>
+    <row r="241" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A241" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B241" s="8" t="s">
+        <v>732</v>
+      </c>
+      <c r="C241" s="8" t="s">
+        <v>733</v>
+      </c>
+      <c r="D241" s="8" t="s">
+        <v>734</v>
+      </c>
+      <c r="E241" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F241" s="8"/>
+      <c r="G241" s="8"/>
+    </row>
+    <row r="242" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A242" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B242" s="8" t="s">
+        <v>735</v>
+      </c>
+      <c r="C242" s="8" t="s">
+        <v>736</v>
+      </c>
+      <c r="D242" s="8" t="s">
+        <v>737</v>
+      </c>
+      <c r="E242" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="F242" s="8"/>
+      <c r="G242" s="8"/>
+    </row>
+    <row r="243" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A243" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B243" s="8" t="s">
+        <v>738</v>
+      </c>
+      <c r="C243" s="8" t="s">
+        <v>739</v>
+      </c>
+      <c r="D243" s="8" t="s">
+        <v>740</v>
+      </c>
+      <c r="E243" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="F243" s="8"/>
+      <c r="G243" s="8"/>
+    </row>
+    <row r="244" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A244" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B244" s="8" t="s">
+        <v>741</v>
+      </c>
+      <c r="C244" s="8" t="s">
+        <v>742</v>
+      </c>
+      <c r="D244" s="8" t="s">
+        <v>743</v>
+      </c>
+      <c r="E244" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="F244" s="8"/>
+      <c r="G244" s="8"/>
+    </row>
+    <row r="245" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A245" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B245" s="8" t="s">
+        <v>744</v>
+      </c>
+      <c r="C245" s="8" t="s">
+        <v>745</v>
+      </c>
+      <c r="D245" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="E245" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="F245" s="8"/>
+      <c r="G245" s="8"/>
+    </row>
+    <row r="246" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A246" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B246" s="8" t="s">
+        <v>746</v>
+      </c>
+      <c r="C246" s="8" t="s">
+        <v>747</v>
+      </c>
+      <c r="D246" s="8" t="s">
+        <v>377</v>
+      </c>
+      <c r="E246" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F246" s="8"/>
+      <c r="G246" s="8"/>
+    </row>
+    <row r="247" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A247" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B247" s="8" t="s">
+        <v>748</v>
+      </c>
+      <c r="C247" s="8" t="s">
+        <v>749</v>
+      </c>
+      <c r="D247" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E247" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="F247" s="8"/>
+      <c r="G247" s="8"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:S247" xr:uid="{96666041-4A3A-42C1-A22D-86A52389C7E2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>